<commit_message>
[AUTO] Transformación Concrelab - 2026-09-17 18:15:36
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K171"/>
+  <dimension ref="A1:K181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3432,19 +3432,19 @@
         <v>46267</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="H67" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I67" t="n">
         <v>35</v>
       </c>
       <c r="J67" t="n">
-        <v>40.4</v>
+        <v>46.6</v>
       </c>
       <c r="K67" t="n">
-        <v>115.4</v>
+        <v>133.1</v>
       </c>
     </row>
     <row r="68">
@@ -3477,19 +3477,19 @@
         <v>46267</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="H68" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I68" t="n">
         <v>35</v>
       </c>
       <c r="J68" t="n">
-        <v>40.9</v>
+        <v>47.9</v>
       </c>
       <c r="K68" t="n">
-        <v>116.9</v>
+        <v>136.9</v>
       </c>
     </row>
     <row r="69">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>P-32</t>
+          <t>P-31</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
+          <t>Pilote 43 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F69" s="1" t="n">
@@ -3531,10 +3531,10 @@
         <v>35</v>
       </c>
       <c r="J69" t="n">
-        <v>45.9</v>
+        <v>40.4</v>
       </c>
       <c r="K69" t="n">
-        <v>131.1</v>
+        <v>115.4</v>
       </c>
     </row>
     <row r="70">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>P-32</t>
+          <t>P-31</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
+          <t>Pilote 43 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F70" s="1" t="n">
@@ -3576,10 +3576,10 @@
         <v>35</v>
       </c>
       <c r="J70" t="n">
-        <v>44.7</v>
+        <v>40.9</v>
       </c>
       <c r="K70" t="n">
-        <v>127.7</v>
+        <v>116.9</v>
       </c>
     </row>
     <row r="71">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>P-33</t>
+          <t>P-32</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3605,26 +3605,26 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pilote 47 torre 1 tipo 2</t>
+          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F71" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="H71" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I71" t="n">
         <v>35</v>
       </c>
       <c r="J71" t="n">
-        <v>32.5</v>
+        <v>54.9</v>
       </c>
       <c r="K71" t="n">
-        <v>92.90000000000001</v>
+        <v>156.9</v>
       </c>
     </row>
     <row r="72">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>P-33</t>
+          <t>P-32</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3650,26 +3650,26 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pilote 47 torre 1 tipo 2</t>
+          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F72" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="H72" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I72" t="n">
         <v>35</v>
       </c>
       <c r="J72" t="n">
-        <v>32.9</v>
+        <v>54.3</v>
       </c>
       <c r="K72" t="n">
-        <v>94</v>
+        <v>155.1</v>
       </c>
     </row>
     <row r="73">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>P-34</t>
+          <t>P-32</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3695,14 +3695,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
+          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F73" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="H73" t="n">
         <v>7</v>
@@ -3711,10 +3711,10 @@
         <v>35</v>
       </c>
       <c r="J73" t="n">
-        <v>28.3</v>
+        <v>45.9</v>
       </c>
       <c r="K73" t="n">
-        <v>80.90000000000001</v>
+        <v>131.1</v>
       </c>
     </row>
     <row r="74">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>P-34</t>
+          <t>P-32</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3740,14 +3740,14 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
+          <t>Pilote 11 torre 1 tipo 1, pilote 34 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F74" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="H74" t="n">
         <v>7</v>
@@ -3756,10 +3756,10 @@
         <v>35</v>
       </c>
       <c r="J74" t="n">
-        <v>27.5</v>
+        <v>44.7</v>
       </c>
       <c r="K74" t="n">
-        <v>78.59999999999999</v>
+        <v>127.7</v>
       </c>
     </row>
     <row r="75">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>P-33</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3785,14 +3785,14 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pilote 90 torre 2 tipo 2</t>
+          <t>Pilote 47 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F75" s="1" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="H75" t="n">
         <v>7</v>
@@ -3801,10 +3801,10 @@
         <v>35</v>
       </c>
       <c r="J75" t="n">
-        <v>27.2</v>
+        <v>32.5</v>
       </c>
       <c r="K75" t="n">
-        <v>77.7</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="76">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>P-33</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3830,14 +3830,14 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Pilote 90 torre 2 tipo 2</t>
+          <t>Pilote 47 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F76" s="1" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="H76" t="n">
         <v>7</v>
@@ -3846,10 +3846,10 @@
         <v>35</v>
       </c>
       <c r="J76" t="n">
-        <v>27.6</v>
+        <v>32.9</v>
       </c>
       <c r="K76" t="n">
-        <v>78.90000000000001</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3875,26 +3875,26 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F77" s="1" t="n">
-        <v>46249</v>
+        <v>46268</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H77" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I77" t="n">
         <v>35</v>
       </c>
       <c r="J77" t="n">
-        <v>37.2</v>
+        <v>28.3</v>
       </c>
       <c r="K77" t="n">
-        <v>106.3</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="78">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3920,26 +3920,26 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F78" s="1" t="n">
-        <v>46249</v>
+        <v>46268</v>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H78" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I78" t="n">
         <v>35</v>
       </c>
       <c r="J78" t="n">
-        <v>36.1</v>
+        <v>27.5</v>
       </c>
       <c r="K78" t="n">
-        <v>103.1</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="79">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3965,26 +3965,26 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F79" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="H79" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I79" t="n">
         <v>35</v>
       </c>
       <c r="J79" t="n">
-        <v>36.5</v>
+        <v>27.2</v>
       </c>
       <c r="K79" t="n">
-        <v>104.3</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="80">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4010,26 +4010,26 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F80" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46263</v>
+        <v>46276</v>
       </c>
       <c r="H80" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I80" t="n">
         <v>35</v>
       </c>
       <c r="J80" t="n">
-        <v>31.2</v>
+        <v>27.6</v>
       </c>
       <c r="K80" t="n">
-        <v>89.09999999999999</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="81">
@@ -4062,19 +4062,19 @@
         <v>46249</v>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="H81" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I81" t="n">
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>31.6</v>
+        <v>37.2</v>
       </c>
       <c r="K81" t="n">
-        <v>90.3</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="82">
@@ -4107,19 +4107,19 @@
         <v>46249</v>
       </c>
       <c r="G82" s="1" t="n">
-        <v>46256</v>
+        <v>46277</v>
       </c>
       <c r="H82" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I82" t="n">
         <v>35</v>
       </c>
       <c r="J82" t="n">
-        <v>23.3</v>
+        <v>36.1</v>
       </c>
       <c r="K82" t="n">
-        <v>66.59999999999999</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="83">
@@ -4152,19 +4152,19 @@
         <v>46249</v>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46256</v>
+        <v>46277</v>
       </c>
       <c r="H83" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I83" t="n">
         <v>35</v>
       </c>
       <c r="J83" t="n">
-        <v>23.5</v>
+        <v>36.5</v>
       </c>
       <c r="K83" t="n">
-        <v>67.09999999999999</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="84">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4190,26 +4190,26 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F84" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46280</v>
+        <v>46263</v>
       </c>
       <c r="H84" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I84" t="n">
         <v>35</v>
       </c>
       <c r="J84" t="n">
-        <v>49</v>
+        <v>31.2</v>
       </c>
       <c r="K84" t="n">
-        <v>140</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="85">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4235,26 +4235,26 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F85" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46280</v>
+        <v>46263</v>
       </c>
       <c r="H85" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I85" t="n">
         <v>35</v>
       </c>
       <c r="J85" t="n">
-        <v>48</v>
+        <v>31.6</v>
       </c>
       <c r="K85" t="n">
-        <v>137.1</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="86">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4280,26 +4280,26 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F86" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46280</v>
+        <v>46256</v>
       </c>
       <c r="H86" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I86" t="n">
         <v>35</v>
       </c>
       <c r="J86" t="n">
-        <v>47.5</v>
+        <v>23.3</v>
       </c>
       <c r="K86" t="n">
-        <v>135.7</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="87">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4325,26 +4325,26 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F87" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G87" s="1" t="n">
-        <v>46266</v>
+        <v>46256</v>
       </c>
       <c r="H87" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I87" t="n">
         <v>35</v>
       </c>
       <c r="J87" t="n">
-        <v>40.2</v>
+        <v>23.5</v>
       </c>
       <c r="K87" t="n">
-        <v>114.9</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -4377,19 +4377,19 @@
         <v>46252</v>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H88" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I88" t="n">
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>39.9</v>
+        <v>49</v>
       </c>
       <c r="K88" t="n">
-        <v>114</v>
+        <v>140</v>
       </c>
     </row>
     <row r="89">
@@ -4422,19 +4422,19 @@
         <v>46252</v>
       </c>
       <c r="G89" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H89" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I89" t="n">
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>34.7</v>
+        <v>48</v>
       </c>
       <c r="K89" t="n">
-        <v>99.09999999999999</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="90">
@@ -4467,19 +4467,19 @@
         <v>46252</v>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H90" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I90" t="n">
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>33.4</v>
+        <v>47.5</v>
       </c>
       <c r="K90" t="n">
-        <v>95.40000000000001</v>
+        <v>135.7</v>
       </c>
     </row>
     <row r="91">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4505,26 +4505,26 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F91" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G91" s="1" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="H91" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I91" t="n">
         <v>35</v>
       </c>
       <c r="J91" t="n">
-        <v>39.5</v>
+        <v>40.2</v>
       </c>
       <c r="K91" t="n">
-        <v>112.9</v>
+        <v>114.9</v>
       </c>
     </row>
     <row r="92">
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4550,26 +4550,26 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F92" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G92" s="1" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="H92" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I92" t="n">
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>40.1</v>
+        <v>39.9</v>
       </c>
       <c r="K92" t="n">
-        <v>114.6</v>
+        <v>114</v>
       </c>
     </row>
     <row r="93">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4595,26 +4595,26 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F93" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G93" s="1" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="H93" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I93" t="n">
         <v>35</v>
       </c>
       <c r="J93" t="n">
-        <v>39.7</v>
+        <v>34.7</v>
       </c>
       <c r="K93" t="n">
-        <v>113.4</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="94">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4640,26 +4640,26 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F94" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G94" s="1" t="n">
-        <v>46266</v>
+        <v>46259</v>
       </c>
       <c r="H94" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I94" t="n">
         <v>35</v>
       </c>
       <c r="J94" t="n">
-        <v>30.9</v>
+        <v>33.4</v>
       </c>
       <c r="K94" t="n">
-        <v>88.3</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="95">
@@ -4692,19 +4692,19 @@
         <v>46252</v>
       </c>
       <c r="G95" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H95" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I95" t="n">
         <v>35</v>
       </c>
       <c r="J95" t="n">
-        <v>31.3</v>
+        <v>39.5</v>
       </c>
       <c r="K95" t="n">
-        <v>89.40000000000001</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="96">
@@ -4737,19 +4737,19 @@
         <v>46252</v>
       </c>
       <c r="G96" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H96" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I96" t="n">
         <v>35</v>
       </c>
       <c r="J96" t="n">
-        <v>25</v>
+        <v>40.1</v>
       </c>
       <c r="K96" t="n">
-        <v>71.40000000000001</v>
+        <v>114.6</v>
       </c>
     </row>
     <row r="97">
@@ -4782,19 +4782,19 @@
         <v>46252</v>
       </c>
       <c r="G97" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H97" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I97" t="n">
         <v>35</v>
       </c>
       <c r="J97" t="n">
-        <v>24.5</v>
+        <v>39.7</v>
       </c>
       <c r="K97" t="n">
-        <v>70</v>
+        <v>113.4</v>
       </c>
     </row>
     <row r="98">
@@ -4805,12 +4805,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4820,14 +4820,14 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F98" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G98" s="1" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="H98" t="n">
         <v>14</v>
@@ -4836,10 +4836,10 @@
         <v>35</v>
       </c>
       <c r="J98" t="n">
-        <v>34.2</v>
+        <v>30.9</v>
       </c>
       <c r="K98" t="n">
-        <v>97.7</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="99">
@@ -4850,12 +4850,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4865,14 +4865,14 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F99" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G99" s="1" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="H99" t="n">
         <v>14</v>
@@ -4881,10 +4881,10 @@
         <v>35</v>
       </c>
       <c r="J99" t="n">
-        <v>34.6</v>
+        <v>31.3</v>
       </c>
       <c r="K99" t="n">
-        <v>98.90000000000001</v>
+        <v>89.40000000000001</v>
       </c>
     </row>
     <row r="100">
@@ -4895,12 +4895,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4910,14 +4910,14 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F100" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G100" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="H100" t="n">
         <v>7</v>
@@ -4926,10 +4926,10 @@
         <v>35</v>
       </c>
       <c r="J100" t="n">
-        <v>21.3</v>
+        <v>25</v>
       </c>
       <c r="K100" t="n">
-        <v>60.9</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="101">
@@ -4940,12 +4940,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4955,14 +4955,14 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F101" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G101" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="H101" t="n">
         <v>7</v>
@@ -4971,10 +4971,10 @@
         <v>35</v>
       </c>
       <c r="J101" t="n">
-        <v>21.5</v>
+        <v>24.5</v>
       </c>
       <c r="K101" t="n">
-        <v>61.4</v>
+        <v>70</v>
       </c>
     </row>
     <row r="102">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5000,26 +5000,26 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F102" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G102" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H102" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I102" t="n">
         <v>35</v>
       </c>
       <c r="J102" t="n">
-        <v>37.9</v>
+        <v>43.5</v>
       </c>
       <c r="K102" t="n">
-        <v>108.3</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="103">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5045,26 +5045,26 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F103" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G103" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H103" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I103" t="n">
         <v>35</v>
       </c>
       <c r="J103" t="n">
-        <v>38.4</v>
+        <v>41.6</v>
       </c>
       <c r="K103" t="n">
-        <v>109.7</v>
+        <v>118.9</v>
       </c>
     </row>
     <row r="104">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5090,26 +5090,26 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F104" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G104" s="1" t="n">
-        <v>46260</v>
+        <v>46281</v>
       </c>
       <c r="H104" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I104" t="n">
         <v>35</v>
       </c>
       <c r="J104" t="n">
-        <v>34.6</v>
+        <v>42.2</v>
       </c>
       <c r="K104" t="n">
-        <v>98.90000000000001</v>
+        <v>120.6</v>
       </c>
     </row>
     <row r="105">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5135,26 +5135,26 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F105" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G105" s="1" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="H105" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I105" t="n">
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>34.8</v>
+        <v>34.2</v>
       </c>
       <c r="K105" t="n">
-        <v>99.40000000000001</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="106">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5180,14 +5180,14 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F106" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G106" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="H106" t="n">
         <v>14</v>
@@ -5196,10 +5196,10 @@
         <v>35</v>
       </c>
       <c r="J106" t="n">
-        <v>30.9</v>
+        <v>34.6</v>
       </c>
       <c r="K106" t="n">
-        <v>88.3</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="107">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -5225,26 +5225,26 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F107" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G107" s="1" t="n">
-        <v>46268</v>
+        <v>46260</v>
       </c>
       <c r="H107" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I107" t="n">
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>32.3</v>
+        <v>21.3</v>
       </c>
       <c r="K107" t="n">
-        <v>92.3</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="108">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5270,14 +5270,14 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F108" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G108" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="H108" t="n">
         <v>7</v>
@@ -5286,10 +5286,10 @@
         <v>35</v>
       </c>
       <c r="J108" t="n">
-        <v>25.8</v>
+        <v>21.5</v>
       </c>
       <c r="K108" t="n">
-        <v>73.7</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="109">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5315,26 +5315,26 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F109" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G109" s="1" t="n">
-        <v>46261</v>
+        <v>46281</v>
       </c>
       <c r="H109" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I109" t="n">
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>23.9</v>
+        <v>45.7</v>
       </c>
       <c r="K109" t="n">
-        <v>68.3</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="110">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5360,26 +5360,26 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F110" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G110" s="1" t="n">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="H110" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I110" t="n">
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>33.8</v>
+        <v>46.1</v>
       </c>
       <c r="K110" t="n">
-        <v>96.59999999999999</v>
+        <v>131.7</v>
       </c>
     </row>
     <row r="111">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5405,26 +5405,26 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F111" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G111" s="1" t="n">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="H111" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I111" t="n">
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>32.1</v>
+        <v>44.4</v>
       </c>
       <c r="K111" t="n">
-        <v>91.7</v>
+        <v>126.9</v>
       </c>
     </row>
     <row r="112">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5450,26 +5450,26 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F112" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>46261</v>
+        <v>46267</v>
       </c>
       <c r="H112" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I112" t="n">
         <v>35</v>
       </c>
       <c r="J112" t="n">
-        <v>25.7</v>
+        <v>37.9</v>
       </c>
       <c r="K112" t="n">
-        <v>73.40000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="113">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5495,26 +5495,26 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F113" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G113" s="1" t="n">
-        <v>46261</v>
+        <v>46267</v>
       </c>
       <c r="H113" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I113" t="n">
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>25.5</v>
+        <v>38.4</v>
       </c>
       <c r="K113" t="n">
-        <v>72.90000000000001</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="114">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -5540,26 +5540,26 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F114" s="1" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="G114" s="1" t="n">
-        <v>46269</v>
+        <v>46260</v>
       </c>
       <c r="H114" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I114" t="n">
         <v>35</v>
       </c>
       <c r="J114" t="n">
-        <v>32.7</v>
+        <v>34.6</v>
       </c>
       <c r="K114" t="n">
-        <v>93.40000000000001</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="115">
@@ -5570,12 +5570,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -5585,26 +5585,26 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F115" s="1" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="G115" s="1" t="n">
-        <v>46269</v>
+        <v>46260</v>
       </c>
       <c r="H115" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I115" t="n">
         <v>35</v>
       </c>
       <c r="J115" t="n">
-        <v>32.5</v>
+        <v>34.8</v>
       </c>
       <c r="K115" t="n">
-        <v>92.90000000000001</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="116">
@@ -5615,12 +5615,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5630,26 +5630,26 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F116" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G116" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H116" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I116" t="n">
         <v>35</v>
       </c>
       <c r="J116" t="n">
-        <v>28.6</v>
+        <v>30.9</v>
       </c>
       <c r="K116" t="n">
-        <v>81.7</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="117">
@@ -5660,12 +5660,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -5675,26 +5675,26 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F117" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G117" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H117" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I117" t="n">
         <v>35</v>
       </c>
       <c r="J117" t="n">
-        <v>28.7</v>
+        <v>32.3</v>
       </c>
       <c r="K117" t="n">
-        <v>82</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="118">
@@ -5705,12 +5705,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -5720,26 +5720,26 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F118" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G118" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="H118" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I118" t="n">
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>38.8</v>
+        <v>25.8</v>
       </c>
       <c r="K118" t="n">
-        <v>110.9</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="119">
@@ -5750,12 +5750,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5765,26 +5765,26 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F119" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G119" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="H119" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I119" t="n">
         <v>35</v>
       </c>
       <c r="J119" t="n">
-        <v>38.6</v>
+        <v>23.9</v>
       </c>
       <c r="K119" t="n">
-        <v>110.3</v>
+        <v>68.3</v>
       </c>
     </row>
     <row r="120">
@@ -5795,12 +5795,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -5810,26 +5810,26 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F120" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G120" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H120" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I120" t="n">
         <v>35</v>
       </c>
       <c r="J120" t="n">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
       <c r="K120" t="n">
-        <v>96.3</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="121">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5855,26 +5855,26 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G121" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H121" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I121" t="n">
         <v>35</v>
       </c>
       <c r="J121" t="n">
-        <v>32.5</v>
+        <v>32.1</v>
       </c>
       <c r="K121" t="n">
-        <v>92.90000000000001</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="122">
@@ -5885,12 +5885,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -5900,26 +5900,26 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F122" s="1" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="G122" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="H122" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I122" t="n">
         <v>35</v>
       </c>
       <c r="J122" t="n">
-        <v>32.3</v>
+        <v>25.7</v>
       </c>
       <c r="K122" t="n">
-        <v>92.3</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="123">
@@ -5930,12 +5930,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -5945,26 +5945,26 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F123" s="1" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="G123" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="H123" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I123" t="n">
         <v>35</v>
       </c>
       <c r="J123" t="n">
-        <v>32.5</v>
+        <v>25.5</v>
       </c>
       <c r="K123" t="n">
-        <v>92.90000000000001</v>
+        <v>72.90000000000001</v>
       </c>
     </row>
     <row r="124">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -5990,26 +5990,26 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F124" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H124" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I124" t="n">
         <v>35</v>
       </c>
       <c r="J124" t="n">
-        <v>28.8</v>
+        <v>32.7</v>
       </c>
       <c r="K124" t="n">
-        <v>82.3</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="125">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -6035,26 +6035,26 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F125" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G125" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H125" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I125" t="n">
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>27.6</v>
+        <v>32.5</v>
       </c>
       <c r="K125" t="n">
-        <v>78.90000000000001</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="126">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -6080,26 +6080,26 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G126" s="1" t="n">
-        <v>46270</v>
+        <v>46262</v>
       </c>
       <c r="H126" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I126" t="n">
         <v>35</v>
       </c>
       <c r="J126" t="n">
-        <v>36.5</v>
+        <v>28.6</v>
       </c>
       <c r="K126" t="n">
-        <v>104.3</v>
+        <v>81.7</v>
       </c>
     </row>
     <row r="127">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -6125,26 +6125,26 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F127" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G127" s="1" t="n">
-        <v>46270</v>
+        <v>46262</v>
       </c>
       <c r="H127" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I127" t="n">
         <v>35</v>
       </c>
       <c r="J127" t="n">
-        <v>35.5</v>
+        <v>28.7</v>
       </c>
       <c r="K127" t="n">
-        <v>101.4</v>
+        <v>82</v>
       </c>
     </row>
     <row r="128">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -6170,26 +6170,26 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F128" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G128" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H128" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I128" t="n">
         <v>35</v>
       </c>
       <c r="J128" t="n">
-        <v>31.9</v>
+        <v>38.8</v>
       </c>
       <c r="K128" t="n">
-        <v>91.09999999999999</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="129">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -6215,26 +6215,26 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F129" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G129" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H129" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I129" t="n">
         <v>35</v>
       </c>
       <c r="J129" t="n">
-        <v>31</v>
+        <v>38.6</v>
       </c>
       <c r="K129" t="n">
-        <v>88.59999999999999</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="130">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -6260,26 +6260,26 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F130" s="1" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="G130" s="1" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="H130" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I130" t="n">
         <v>35</v>
       </c>
       <c r="J130" t="n">
-        <v>31.9</v>
+        <v>33.7</v>
       </c>
       <c r="K130" t="n">
-        <v>91.09999999999999</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="131">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6305,26 +6305,26 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F131" s="1" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="G131" s="1" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="H131" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I131" t="n">
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>30.5</v>
+        <v>32.5</v>
       </c>
       <c r="K131" t="n">
-        <v>87.09999999999999</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="132">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -6350,26 +6350,26 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F132" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G132" s="1" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="H132" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I132" t="n">
         <v>35</v>
       </c>
       <c r="J132" t="n">
-        <v>26.9</v>
+        <v>32.3</v>
       </c>
       <c r="K132" t="n">
-        <v>76.90000000000001</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="133">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -6395,26 +6395,26 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F133" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G133" s="1" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="H133" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I133" t="n">
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>26.5</v>
+        <v>32.5</v>
       </c>
       <c r="K133" t="n">
-        <v>75.7</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="134">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6440,26 +6440,26 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F134" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G134" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H134" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I134" t="n">
         <v>35</v>
       </c>
       <c r="J134" t="n">
-        <v>37.9</v>
+        <v>28.8</v>
       </c>
       <c r="K134" t="n">
-        <v>108.3</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="135">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -6485,26 +6485,26 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F135" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G135" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H135" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I135" t="n">
         <v>35</v>
       </c>
       <c r="J135" t="n">
-        <v>38</v>
+        <v>27.6</v>
       </c>
       <c r="K135" t="n">
-        <v>108.6</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="136">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -6530,26 +6530,26 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F136" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G136" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H136" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I136" t="n">
         <v>35</v>
       </c>
       <c r="J136" t="n">
-        <v>33.4</v>
+        <v>36.5</v>
       </c>
       <c r="K136" t="n">
-        <v>95.40000000000001</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="137">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6575,26 +6575,26 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F137" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G137" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H137" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I137" t="n">
         <v>35</v>
       </c>
       <c r="J137" t="n">
-        <v>31.6</v>
+        <v>35.5</v>
       </c>
       <c r="K137" t="n">
-        <v>90.3</v>
+        <v>101.4</v>
       </c>
     </row>
     <row r="138">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -6620,26 +6620,26 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F138" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G138" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H138" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I138" t="n">
         <v>35</v>
       </c>
       <c r="J138" t="n">
-        <v>33</v>
+        <v>31.9</v>
       </c>
       <c r="K138" t="n">
-        <v>94.3</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="139">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -6665,26 +6665,26 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F139" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G139" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H139" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I139" t="n">
         <v>35</v>
       </c>
       <c r="J139" t="n">
-        <v>32.6</v>
+        <v>31</v>
       </c>
       <c r="K139" t="n">
-        <v>93.09999999999999</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="140">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -6710,26 +6710,26 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F140" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G140" s="1" t="n">
-        <v>46266</v>
+        <v>46272</v>
       </c>
       <c r="H140" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I140" t="n">
         <v>35</v>
       </c>
       <c r="J140" t="n">
-        <v>28.7</v>
+        <v>31.9</v>
       </c>
       <c r="K140" t="n">
-        <v>82</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="141">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -6755,26 +6755,26 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F141" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G141" s="1" t="n">
-        <v>46266</v>
+        <v>46272</v>
       </c>
       <c r="H141" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I141" t="n">
         <v>35</v>
       </c>
       <c r="J141" t="n">
-        <v>26.9</v>
+        <v>30.5</v>
       </c>
       <c r="K141" t="n">
-        <v>76.90000000000001</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="142">
@@ -6785,12 +6785,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -6800,26 +6800,26 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F142" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G142" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H142" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I142" t="n">
         <v>35</v>
       </c>
       <c r="J142" t="n">
-        <v>38.9</v>
+        <v>26.9</v>
       </c>
       <c r="K142" t="n">
-        <v>111.1</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="143">
@@ -6830,12 +6830,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6845,26 +6845,26 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F143" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G143" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H143" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I143" t="n">
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>38</v>
+        <v>26.5</v>
       </c>
       <c r="K143" t="n">
-        <v>108.6</v>
+        <v>75.7</v>
       </c>
     </row>
     <row r="144">
@@ -6875,12 +6875,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -6890,26 +6890,26 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F144" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G144" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H144" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I144" t="n">
         <v>35</v>
       </c>
       <c r="J144" t="n">
-        <v>34.1</v>
+        <v>37.9</v>
       </c>
       <c r="K144" t="n">
-        <v>97.40000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="145">
@@ -6920,12 +6920,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -6935,26 +6935,26 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F145" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G145" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H145" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I145" t="n">
         <v>35</v>
       </c>
       <c r="J145" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K145" t="n">
-        <v>94.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="146">
@@ -6965,12 +6965,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6980,26 +6980,26 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F146" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G146" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H146" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I146" t="n">
         <v>35</v>
       </c>
       <c r="J146" t="n">
-        <v>43.4</v>
+        <v>33.4</v>
       </c>
       <c r="K146" t="n">
-        <v>124</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="147">
@@ -7010,12 +7010,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -7025,26 +7025,26 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F147" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G147" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H147" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I147" t="n">
         <v>35</v>
       </c>
       <c r="J147" t="n">
-        <v>43.9</v>
+        <v>31.6</v>
       </c>
       <c r="K147" t="n">
-        <v>125.4</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="148">
@@ -7055,12 +7055,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -7070,26 +7070,26 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F148" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G148" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H148" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I148" t="n">
         <v>35</v>
       </c>
       <c r="J148" t="n">
-        <v>37.8</v>
+        <v>33</v>
       </c>
       <c r="K148" t="n">
-        <v>108</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="149">
@@ -7100,12 +7100,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -7115,26 +7115,26 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F149" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G149" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H149" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I149" t="n">
         <v>35</v>
       </c>
       <c r="J149" t="n">
-        <v>36.5</v>
+        <v>32.6</v>
       </c>
       <c r="K149" t="n">
-        <v>104.3</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="150">
@@ -7145,12 +7145,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -7160,26 +7160,26 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F150" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G150" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H150" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I150" t="n">
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>36.3</v>
+        <v>28.7</v>
       </c>
       <c r="K150" t="n">
-        <v>103.7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="151">
@@ -7190,12 +7190,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -7205,26 +7205,26 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F151" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G151" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H151" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I151" t="n">
         <v>35</v>
       </c>
       <c r="J151" t="n">
-        <v>36.6</v>
+        <v>26.9</v>
       </c>
       <c r="K151" t="n">
-        <v>104.6</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="152">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7250,26 +7250,26 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F152" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G152" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H152" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I152" t="n">
         <v>35</v>
       </c>
       <c r="J152" t="n">
-        <v>31.6</v>
+        <v>38.9</v>
       </c>
       <c r="K152" t="n">
-        <v>90.3</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="153">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7295,26 +7295,26 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F153" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G153" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H153" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I153" t="n">
         <v>35</v>
       </c>
       <c r="J153" t="n">
-        <v>30.2</v>
+        <v>38</v>
       </c>
       <c r="K153" t="n">
-        <v>86.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="154">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7340,26 +7340,26 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F154" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G154" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H154" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I154" t="n">
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>38.1</v>
+        <v>34.1</v>
       </c>
       <c r="K154" t="n">
-        <v>108.9</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="155">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7385,26 +7385,26 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F155" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G155" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H155" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I155" t="n">
         <v>35</v>
       </c>
       <c r="J155" t="n">
-        <v>38.6</v>
+        <v>33</v>
       </c>
       <c r="K155" t="n">
-        <v>110.3</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="156">
@@ -7415,7 +7415,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7430,26 +7430,26 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F156" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G156" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H156" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I156" t="n">
         <v>35</v>
       </c>
       <c r="J156" t="n">
-        <v>32.1</v>
+        <v>43.4</v>
       </c>
       <c r="K156" t="n">
-        <v>91.7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="157">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7475,26 +7475,26 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F157" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G157" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H157" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I157" t="n">
         <v>35</v>
       </c>
       <c r="J157" t="n">
-        <v>32.7</v>
+        <v>43.9</v>
       </c>
       <c r="K157" t="n">
-        <v>93.40000000000001</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="158">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7520,26 +7520,26 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F158" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G158" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H158" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I158" t="n">
         <v>35</v>
       </c>
       <c r="J158" t="n">
-        <v>49</v>
+        <v>37.8</v>
       </c>
       <c r="K158" t="n">
-        <v>140</v>
+        <v>108</v>
       </c>
     </row>
     <row r="159">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -7565,26 +7565,26 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F159" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G159" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H159" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I159" t="n">
         <v>35</v>
       </c>
       <c r="J159" t="n">
-        <v>49.6</v>
+        <v>36.5</v>
       </c>
       <c r="K159" t="n">
-        <v>141.7</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="160">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7610,26 +7610,26 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F160" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G160" s="1" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="H160" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I160" t="n">
         <v>35</v>
       </c>
       <c r="J160" t="n">
-        <v>40.9</v>
+        <v>36.3</v>
       </c>
       <c r="K160" t="n">
-        <v>116.9</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="161">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7655,26 +7655,26 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F161" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G161" s="1" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="H161" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I161" t="n">
         <v>35</v>
       </c>
       <c r="J161" t="n">
-        <v>41.3</v>
+        <v>36.6</v>
       </c>
       <c r="K161" t="n">
-        <v>118</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="162">
@@ -7685,12 +7685,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -7700,14 +7700,14 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F162" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G162" s="1" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="H162" t="n">
         <v>7</v>
@@ -7716,10 +7716,10 @@
         <v>35</v>
       </c>
       <c r="J162" t="n">
-        <v>36.6</v>
+        <v>31.6</v>
       </c>
       <c r="K162" t="n">
-        <v>104.6</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="163">
@@ -7730,12 +7730,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -7745,14 +7745,14 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F163" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G163" s="1" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="H163" t="n">
         <v>7</v>
@@ -7761,10 +7761,10 @@
         <v>35</v>
       </c>
       <c r="J163" t="n">
-        <v>37.1</v>
+        <v>30.2</v>
       </c>
       <c r="K163" t="n">
-        <v>106</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="164">
@@ -7775,12 +7775,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -7790,26 +7790,26 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F164" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G164" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H164" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I164" t="n">
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>38.9</v>
+        <v>38.1</v>
       </c>
       <c r="K164" t="n">
-        <v>111.1</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="165">
@@ -7820,12 +7820,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -7835,26 +7835,26 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F165" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G165" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H165" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I165" t="n">
         <v>35</v>
       </c>
       <c r="J165" t="n">
-        <v>37.9</v>
+        <v>38.6</v>
       </c>
       <c r="K165" t="n">
-        <v>108.3</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="166">
@@ -7865,12 +7865,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -7880,14 +7880,14 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F166" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G166" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H166" t="n">
         <v>7</v>
@@ -7896,10 +7896,10 @@
         <v>35</v>
       </c>
       <c r="J166" t="n">
-        <v>40.3</v>
+        <v>32.1</v>
       </c>
       <c r="K166" t="n">
-        <v>115.1</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="167">
@@ -7910,12 +7910,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -7925,14 +7925,14 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F167" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G167" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H167" t="n">
         <v>7</v>
@@ -7941,10 +7941,10 @@
         <v>35</v>
       </c>
       <c r="J167" t="n">
-        <v>40.8</v>
+        <v>32.7</v>
       </c>
       <c r="K167" t="n">
-        <v>116.6</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="168">
@@ -7955,12 +7955,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -7970,26 +7970,26 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F168" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G168" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H168" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I168" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J168" t="n">
-        <v>27.1</v>
+        <v>49</v>
       </c>
       <c r="K168" t="n">
-        <v>110.6</v>
+        <v>140</v>
       </c>
     </row>
     <row r="169">
@@ -8000,12 +8000,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -8015,26 +8015,26 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F169" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G169" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H169" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I169" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>25.8</v>
+        <v>49.6</v>
       </c>
       <c r="K169" t="n">
-        <v>105.3</v>
+        <v>141.7</v>
       </c>
     </row>
     <row r="170">
@@ -8045,12 +8045,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -8060,26 +8060,26 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F170" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G170" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H170" t="n">
         <v>7</v>
       </c>
       <c r="I170" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J170" t="n">
-        <v>24.8</v>
+        <v>40.9</v>
       </c>
       <c r="K170" t="n">
-        <v>101.2</v>
+        <v>116.9</v>
       </c>
     </row>
     <row r="171">
@@ -8090,12 +8090,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -8105,25 +8105,475 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F171" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G171" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H171" t="n">
         <v>7</v>
       </c>
       <c r="I171" t="n">
+        <v>35</v>
+      </c>
+      <c r="J171" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="K171" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F172" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G172" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H172" t="n">
+        <v>7</v>
+      </c>
+      <c r="I172" t="n">
+        <v>35</v>
+      </c>
+      <c r="J172" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="K172" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F173" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G173" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H173" t="n">
+        <v>7</v>
+      </c>
+      <c r="I173" t="n">
+        <v>35</v>
+      </c>
+      <c r="J173" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="K173" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F174" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G174" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H174" t="n">
+        <v>7</v>
+      </c>
+      <c r="I174" t="n">
+        <v>35</v>
+      </c>
+      <c r="J174" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K174" t="n">
+        <v>111.1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F175" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G175" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H175" t="n">
+        <v>7</v>
+      </c>
+      <c r="I175" t="n">
+        <v>35</v>
+      </c>
+      <c r="J175" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="K175" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F176" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G176" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H176" t="n">
+        <v>7</v>
+      </c>
+      <c r="I176" t="n">
+        <v>35</v>
+      </c>
+      <c r="J176" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="K176" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F177" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G177" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H177" t="n">
+        <v>7</v>
+      </c>
+      <c r="I177" t="n">
+        <v>35</v>
+      </c>
+      <c r="J177" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K177" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F178" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G178" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H178" t="n">
+        <v>7</v>
+      </c>
+      <c r="I178" t="n">
         <v>24.5</v>
       </c>
-      <c r="J171" t="n">
+      <c r="J178" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K178" t="n">
+        <v>110.6</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F179" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G179" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H179" t="n">
+        <v>7</v>
+      </c>
+      <c r="I179" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J179" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K179" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F180" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G180" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H180" t="n">
+        <v>7</v>
+      </c>
+      <c r="I180" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J180" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K180" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F181" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G181" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H181" t="n">
+        <v>7</v>
+      </c>
+      <c r="I181" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J181" t="n">
         <v>24.6</v>
       </c>
-      <c r="K171" t="n">
+      <c r="K181" t="n">
         <v>100.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-09-18 20:18:47
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K181"/>
+  <dimension ref="A1:K193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3792,19 +3792,19 @@
         <v>46268</v>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="H75" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I75" t="n">
         <v>35</v>
       </c>
       <c r="J75" t="n">
-        <v>32.5</v>
+        <v>37.5</v>
       </c>
       <c r="K75" t="n">
-        <v>92.90000000000001</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="76">
@@ -3837,19 +3837,19 @@
         <v>46268</v>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="H76" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I76" t="n">
         <v>35</v>
       </c>
       <c r="J76" t="n">
-        <v>32.9</v>
+        <v>38</v>
       </c>
       <c r="K76" t="n">
-        <v>94</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="77">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>P-34</t>
+          <t>P-33</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
+          <t>Pilote 47 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F77" s="1" t="n">
@@ -3891,10 +3891,10 @@
         <v>35</v>
       </c>
       <c r="J77" t="n">
-        <v>28.3</v>
+        <v>32.5</v>
       </c>
       <c r="K77" t="n">
-        <v>80.90000000000001</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="78">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>P-34</t>
+          <t>P-33</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
+          <t>Pilote 47 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F78" s="1" t="n">
@@ -3936,10 +3936,10 @@
         <v>35</v>
       </c>
       <c r="J78" t="n">
-        <v>27.5</v>
+        <v>32.9</v>
       </c>
       <c r="K78" t="n">
-        <v>78.59999999999999</v>
+        <v>94</v>
       </c>
     </row>
     <row r="79">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3965,26 +3965,26 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Pilote 90 torre 2 tipo 2</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F79" s="1" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="H79" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I79" t="n">
         <v>35</v>
       </c>
       <c r="J79" t="n">
-        <v>27.2</v>
+        <v>37.2</v>
       </c>
       <c r="K79" t="n">
-        <v>77.7</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="80">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4010,26 +4010,26 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Pilote 90 torre 2 tipo 2</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F80" s="1" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="H80" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I80" t="n">
         <v>35</v>
       </c>
       <c r="J80" t="n">
-        <v>27.6</v>
+        <v>36.3</v>
       </c>
       <c r="K80" t="n">
-        <v>78.90000000000001</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="81">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4055,26 +4055,26 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F81" s="1" t="n">
-        <v>46249</v>
+        <v>46268</v>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H81" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I81" t="n">
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>37.2</v>
+        <v>28.3</v>
       </c>
       <c r="K81" t="n">
-        <v>106.3</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="82">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-34</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4100,26 +4100,26 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 38 torre 1 tipo 2, pilote 29 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F82" s="1" t="n">
-        <v>46249</v>
+        <v>46268</v>
       </c>
       <c r="G82" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H82" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I82" t="n">
         <v>35</v>
       </c>
       <c r="J82" t="n">
-        <v>36.1</v>
+        <v>27.5</v>
       </c>
       <c r="K82" t="n">
-        <v>103.1</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="83">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4145,26 +4145,26 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F83" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="H83" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I83" t="n">
         <v>35</v>
       </c>
       <c r="J83" t="n">
-        <v>36.5</v>
+        <v>27.2</v>
       </c>
       <c r="K83" t="n">
-        <v>104.3</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="84">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4190,26 +4190,26 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F84" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46263</v>
+        <v>46276</v>
       </c>
       <c r="H84" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I84" t="n">
         <v>35</v>
       </c>
       <c r="J84" t="n">
-        <v>31.2</v>
+        <v>27.6</v>
       </c>
       <c r="K84" t="n">
-        <v>89.09999999999999</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="85">
@@ -4242,19 +4242,19 @@
         <v>46249</v>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="H85" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I85" t="n">
         <v>35</v>
       </c>
       <c r="J85" t="n">
-        <v>31.6</v>
+        <v>37.2</v>
       </c>
       <c r="K85" t="n">
-        <v>90.3</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="86">
@@ -4287,19 +4287,19 @@
         <v>46249</v>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46256</v>
+        <v>46277</v>
       </c>
       <c r="H86" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I86" t="n">
         <v>35</v>
       </c>
       <c r="J86" t="n">
-        <v>23.3</v>
+        <v>36.1</v>
       </c>
       <c r="K86" t="n">
-        <v>66.59999999999999</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="87">
@@ -4332,19 +4332,19 @@
         <v>46249</v>
       </c>
       <c r="G87" s="1" t="n">
-        <v>46256</v>
+        <v>46277</v>
       </c>
       <c r="H87" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I87" t="n">
         <v>35</v>
       </c>
       <c r="J87" t="n">
-        <v>23.5</v>
+        <v>36.5</v>
       </c>
       <c r="K87" t="n">
-        <v>67.09999999999999</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="88">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4370,26 +4370,26 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F88" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46280</v>
+        <v>46263</v>
       </c>
       <c r="H88" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I88" t="n">
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>49</v>
+        <v>31.2</v>
       </c>
       <c r="K88" t="n">
-        <v>140</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="89">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4415,26 +4415,26 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F89" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G89" s="1" t="n">
-        <v>46280</v>
+        <v>46263</v>
       </c>
       <c r="H89" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I89" t="n">
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>48</v>
+        <v>31.6</v>
       </c>
       <c r="K89" t="n">
-        <v>137.1</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="90">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4460,26 +4460,26 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F90" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46280</v>
+        <v>46256</v>
       </c>
       <c r="H90" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I90" t="n">
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>47.5</v>
+        <v>23.3</v>
       </c>
       <c r="K90" t="n">
-        <v>135.7</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="91">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4505,26 +4505,26 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F91" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G91" s="1" t="n">
-        <v>46266</v>
+        <v>46256</v>
       </c>
       <c r="H91" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I91" t="n">
         <v>35</v>
       </c>
       <c r="J91" t="n">
-        <v>40.2</v>
+        <v>23.5</v>
       </c>
       <c r="K91" t="n">
-        <v>114.9</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="92">
@@ -4557,19 +4557,19 @@
         <v>46252</v>
       </c>
       <c r="G92" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H92" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I92" t="n">
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>39.9</v>
+        <v>49</v>
       </c>
       <c r="K92" t="n">
-        <v>114</v>
+        <v>140</v>
       </c>
     </row>
     <row r="93">
@@ -4602,19 +4602,19 @@
         <v>46252</v>
       </c>
       <c r="G93" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H93" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I93" t="n">
         <v>35</v>
       </c>
       <c r="J93" t="n">
-        <v>34.7</v>
+        <v>48</v>
       </c>
       <c r="K93" t="n">
-        <v>99.09999999999999</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="94">
@@ -4647,19 +4647,19 @@
         <v>46252</v>
       </c>
       <c r="G94" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H94" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I94" t="n">
         <v>35</v>
       </c>
       <c r="J94" t="n">
-        <v>33.4</v>
+        <v>47.5</v>
       </c>
       <c r="K94" t="n">
-        <v>95.40000000000001</v>
+        <v>135.7</v>
       </c>
     </row>
     <row r="95">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4685,26 +4685,26 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F95" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G95" s="1" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="H95" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I95" t="n">
         <v>35</v>
       </c>
       <c r="J95" t="n">
-        <v>39.5</v>
+        <v>40.2</v>
       </c>
       <c r="K95" t="n">
-        <v>112.9</v>
+        <v>114.9</v>
       </c>
     </row>
     <row r="96">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4730,26 +4730,26 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F96" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G96" s="1" t="n">
-        <v>46280</v>
+        <v>46266</v>
       </c>
       <c r="H96" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I96" t="n">
         <v>35</v>
       </c>
       <c r="J96" t="n">
-        <v>40.1</v>
+        <v>39.9</v>
       </c>
       <c r="K96" t="n">
-        <v>114.6</v>
+        <v>114</v>
       </c>
     </row>
     <row r="97">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4775,26 +4775,26 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F97" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G97" s="1" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="H97" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I97" t="n">
         <v>35</v>
       </c>
       <c r="J97" t="n">
-        <v>39.7</v>
+        <v>34.7</v>
       </c>
       <c r="K97" t="n">
-        <v>113.4</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="98">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4820,26 +4820,26 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F98" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G98" s="1" t="n">
-        <v>46266</v>
+        <v>46259</v>
       </c>
       <c r="H98" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I98" t="n">
         <v>35</v>
       </c>
       <c r="J98" t="n">
-        <v>30.9</v>
+        <v>33.4</v>
       </c>
       <c r="K98" t="n">
-        <v>88.3</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="99">
@@ -4872,19 +4872,19 @@
         <v>46252</v>
       </c>
       <c r="G99" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H99" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I99" t="n">
         <v>35</v>
       </c>
       <c r="J99" t="n">
-        <v>31.3</v>
+        <v>39.5</v>
       </c>
       <c r="K99" t="n">
-        <v>89.40000000000001</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="100">
@@ -4917,19 +4917,19 @@
         <v>46252</v>
       </c>
       <c r="G100" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H100" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I100" t="n">
         <v>35</v>
       </c>
       <c r="J100" t="n">
-        <v>25</v>
+        <v>40.1</v>
       </c>
       <c r="K100" t="n">
-        <v>71.40000000000001</v>
+        <v>114.6</v>
       </c>
     </row>
     <row r="101">
@@ -4962,19 +4962,19 @@
         <v>46252</v>
       </c>
       <c r="G101" s="1" t="n">
-        <v>46259</v>
+        <v>46280</v>
       </c>
       <c r="H101" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I101" t="n">
         <v>35</v>
       </c>
       <c r="J101" t="n">
-        <v>24.5</v>
+        <v>39.7</v>
       </c>
       <c r="K101" t="n">
-        <v>70</v>
+        <v>113.4</v>
       </c>
     </row>
     <row r="102">
@@ -4985,12 +4985,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5000,26 +5000,26 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F102" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G102" s="1" t="n">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="H102" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I102" t="n">
         <v>35</v>
       </c>
       <c r="J102" t="n">
-        <v>43.5</v>
+        <v>30.9</v>
       </c>
       <c r="K102" t="n">
-        <v>124.3</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="103">
@@ -5030,12 +5030,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5045,26 +5045,26 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F103" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G103" s="1" t="n">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="H103" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I103" t="n">
         <v>35</v>
       </c>
       <c r="J103" t="n">
-        <v>41.6</v>
+        <v>31.3</v>
       </c>
       <c r="K103" t="n">
-        <v>118.9</v>
+        <v>89.40000000000001</v>
       </c>
     </row>
     <row r="104">
@@ -5075,12 +5075,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5090,26 +5090,26 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F104" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G104" s="1" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="H104" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I104" t="n">
         <v>35</v>
       </c>
       <c r="J104" t="n">
-        <v>42.2</v>
+        <v>25</v>
       </c>
       <c r="K104" t="n">
-        <v>120.6</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="105">
@@ -5120,12 +5120,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5135,26 +5135,26 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F105" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G105" s="1" t="n">
-        <v>46267</v>
+        <v>46259</v>
       </c>
       <c r="H105" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I105" t="n">
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>34.2</v>
+        <v>24.5</v>
       </c>
       <c r="K105" t="n">
-        <v>97.7</v>
+        <v>70</v>
       </c>
     </row>
     <row r="106">
@@ -5187,19 +5187,19 @@
         <v>46253</v>
       </c>
       <c r="G106" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H106" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I106" t="n">
         <v>35</v>
       </c>
       <c r="J106" t="n">
-        <v>34.6</v>
+        <v>43.5</v>
       </c>
       <c r="K106" t="n">
-        <v>98.90000000000001</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="107">
@@ -5232,19 +5232,19 @@
         <v>46253</v>
       </c>
       <c r="G107" s="1" t="n">
-        <v>46260</v>
+        <v>46281</v>
       </c>
       <c r="H107" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I107" t="n">
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>21.3</v>
+        <v>41.6</v>
       </c>
       <c r="K107" t="n">
-        <v>60.9</v>
+        <v>118.9</v>
       </c>
     </row>
     <row r="108">
@@ -5277,19 +5277,19 @@
         <v>46253</v>
       </c>
       <c r="G108" s="1" t="n">
-        <v>46260</v>
+        <v>46281</v>
       </c>
       <c r="H108" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I108" t="n">
         <v>35</v>
       </c>
       <c r="J108" t="n">
-        <v>21.5</v>
+        <v>42.2</v>
       </c>
       <c r="K108" t="n">
-        <v>61.4</v>
+        <v>120.6</v>
       </c>
     </row>
     <row r="109">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5315,26 +5315,26 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F109" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G109" s="1" t="n">
-        <v>46281</v>
+        <v>46267</v>
       </c>
       <c r="H109" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I109" t="n">
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>45.7</v>
+        <v>34.2</v>
       </c>
       <c r="K109" t="n">
-        <v>130.6</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="110">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5360,26 +5360,26 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F110" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G110" s="1" t="n">
-        <v>46281</v>
+        <v>46267</v>
       </c>
       <c r="H110" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="I110" t="n">
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>46.1</v>
+        <v>34.6</v>
       </c>
       <c r="K110" t="n">
-        <v>131.7</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="111">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5405,26 +5405,26 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F111" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G111" s="1" t="n">
-        <v>46281</v>
+        <v>46260</v>
       </c>
       <c r="H111" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I111" t="n">
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>44.4</v>
+        <v>21.3</v>
       </c>
       <c r="K111" t="n">
-        <v>126.9</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="112">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5450,26 +5450,26 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F112" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>46267</v>
+        <v>46260</v>
       </c>
       <c r="H112" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I112" t="n">
         <v>35</v>
       </c>
       <c r="J112" t="n">
-        <v>37.9</v>
+        <v>21.5</v>
       </c>
       <c r="K112" t="n">
-        <v>108.3</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="113">
@@ -5502,19 +5502,19 @@
         <v>46253</v>
       </c>
       <c r="G113" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H113" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I113" t="n">
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>38.4</v>
+        <v>45.7</v>
       </c>
       <c r="K113" t="n">
-        <v>109.7</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="114">
@@ -5547,19 +5547,19 @@
         <v>46253</v>
       </c>
       <c r="G114" s="1" t="n">
-        <v>46260</v>
+        <v>46281</v>
       </c>
       <c r="H114" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I114" t="n">
         <v>35</v>
       </c>
       <c r="J114" t="n">
-        <v>34.6</v>
+        <v>46.1</v>
       </c>
       <c r="K114" t="n">
-        <v>98.90000000000001</v>
+        <v>131.7</v>
       </c>
     </row>
     <row r="115">
@@ -5592,19 +5592,19 @@
         <v>46253</v>
       </c>
       <c r="G115" s="1" t="n">
-        <v>46260</v>
+        <v>46281</v>
       </c>
       <c r="H115" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I115" t="n">
         <v>35</v>
       </c>
       <c r="J115" t="n">
-        <v>34.8</v>
+        <v>44.4</v>
       </c>
       <c r="K115" t="n">
-        <v>99.40000000000001</v>
+        <v>126.9</v>
       </c>
     </row>
     <row r="116">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5630,14 +5630,14 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F116" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G116" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="H116" t="n">
         <v>14</v>
@@ -5646,10 +5646,10 @@
         <v>35</v>
       </c>
       <c r="J116" t="n">
-        <v>30.9</v>
+        <v>37.9</v>
       </c>
       <c r="K116" t="n">
-        <v>88.3</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="117">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5675,14 +5675,14 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F117" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G117" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="H117" t="n">
         <v>14</v>
@@ -5691,10 +5691,10 @@
         <v>35</v>
       </c>
       <c r="J117" t="n">
-        <v>32.3</v>
+        <v>38.4</v>
       </c>
       <c r="K117" t="n">
-        <v>92.3</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="118">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5720,14 +5720,14 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F118" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G118" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="H118" t="n">
         <v>7</v>
@@ -5736,10 +5736,10 @@
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>25.8</v>
+        <v>34.6</v>
       </c>
       <c r="K118" t="n">
-        <v>73.7</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="119">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5765,14 +5765,14 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F119" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G119" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="H119" t="n">
         <v>7</v>
@@ -5781,10 +5781,10 @@
         <v>35</v>
       </c>
       <c r="J119" t="n">
-        <v>23.9</v>
+        <v>34.8</v>
       </c>
       <c r="K119" t="n">
-        <v>68.3</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="120">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5810,26 +5810,26 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F120" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G120" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H120" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I120" t="n">
         <v>35</v>
       </c>
       <c r="J120" t="n">
-        <v>33.8</v>
+        <v>39.1</v>
       </c>
       <c r="K120" t="n">
-        <v>96.59999999999999</v>
+        <v>111.7</v>
       </c>
     </row>
     <row r="121">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5855,26 +5855,26 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F121" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G121" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H121" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I121" t="n">
         <v>35</v>
       </c>
       <c r="J121" t="n">
-        <v>32.1</v>
+        <v>39.6</v>
       </c>
       <c r="K121" t="n">
-        <v>91.7</v>
+        <v>113.1</v>
       </c>
     </row>
     <row r="122">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5900,26 +5900,26 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F122" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G122" s="1" t="n">
-        <v>46261</v>
+        <v>46282</v>
       </c>
       <c r="H122" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I122" t="n">
         <v>35</v>
       </c>
       <c r="J122" t="n">
-        <v>25.7</v>
+        <v>40.2</v>
       </c>
       <c r="K122" t="n">
-        <v>73.40000000000001</v>
+        <v>114.9</v>
       </c>
     </row>
     <row r="123">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5945,26 +5945,26 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F123" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G123" s="1" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="H123" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I123" t="n">
         <v>35</v>
       </c>
       <c r="J123" t="n">
-        <v>25.5</v>
+        <v>30.9</v>
       </c>
       <c r="K123" t="n">
-        <v>72.90000000000001</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="124">
@@ -5975,12 +5975,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5990,14 +5990,14 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F124" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="H124" t="n">
         <v>14</v>
@@ -6006,10 +6006,10 @@
         <v>35</v>
       </c>
       <c r="J124" t="n">
-        <v>32.7</v>
+        <v>32.3</v>
       </c>
       <c r="K124" t="n">
-        <v>93.40000000000001</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="125">
@@ -6020,12 +6020,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -6035,26 +6035,26 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F125" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G125" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="H125" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I125" t="n">
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>32.5</v>
+        <v>25.8</v>
       </c>
       <c r="K125" t="n">
-        <v>92.90000000000001</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="126">
@@ -6065,12 +6065,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -6080,14 +6080,14 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F126" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G126" s="1" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="H126" t="n">
         <v>7</v>
@@ -6096,10 +6096,10 @@
         <v>35</v>
       </c>
       <c r="J126" t="n">
-        <v>28.6</v>
+        <v>23.9</v>
       </c>
       <c r="K126" t="n">
-        <v>81.7</v>
+        <v>68.3</v>
       </c>
     </row>
     <row r="127">
@@ -6110,12 +6110,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -6125,26 +6125,26 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F127" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G127" s="1" t="n">
-        <v>46262</v>
+        <v>46282</v>
       </c>
       <c r="H127" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I127" t="n">
         <v>35</v>
       </c>
       <c r="J127" t="n">
-        <v>28.7</v>
+        <v>42.8</v>
       </c>
       <c r="K127" t="n">
-        <v>82</v>
+        <v>122.3</v>
       </c>
     </row>
     <row r="128">
@@ -6155,12 +6155,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -6170,26 +6170,26 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F128" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G128" s="1" t="n">
-        <v>46269</v>
+        <v>46282</v>
       </c>
       <c r="H128" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I128" t="n">
         <v>35</v>
       </c>
       <c r="J128" t="n">
-        <v>38.8</v>
+        <v>41.1</v>
       </c>
       <c r="K128" t="n">
-        <v>110.9</v>
+        <v>117.4</v>
       </c>
     </row>
     <row r="129">
@@ -6200,12 +6200,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -6215,26 +6215,26 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F129" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G129" s="1" t="n">
-        <v>46269</v>
+        <v>46282</v>
       </c>
       <c r="H129" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I129" t="n">
         <v>35</v>
       </c>
       <c r="J129" t="n">
-        <v>38.6</v>
+        <v>41.4</v>
       </c>
       <c r="K129" t="n">
-        <v>110.3</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="130">
@@ -6245,12 +6245,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -6260,26 +6260,26 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F130" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G130" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H130" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I130" t="n">
         <v>35</v>
       </c>
       <c r="J130" t="n">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
       <c r="K130" t="n">
-        <v>96.3</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="131">
@@ -6290,12 +6290,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -6305,26 +6305,26 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F131" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G131" s="1" t="n">
-        <v>46262</v>
+        <v>46268</v>
       </c>
       <c r="H131" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I131" t="n">
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>32.5</v>
+        <v>32.1</v>
       </c>
       <c r="K131" t="n">
-        <v>92.90000000000001</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="132">
@@ -6335,12 +6335,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -6350,26 +6350,26 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F132" s="1" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="G132" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="H132" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I132" t="n">
         <v>35</v>
       </c>
       <c r="J132" t="n">
-        <v>32.3</v>
+        <v>25.7</v>
       </c>
       <c r="K132" t="n">
-        <v>92.3</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="133">
@@ -6380,12 +6380,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -6395,26 +6395,26 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F133" s="1" t="n">
-        <v>46256</v>
+        <v>46254</v>
       </c>
       <c r="G133" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="H133" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I133" t="n">
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>32.5</v>
+        <v>25.5</v>
       </c>
       <c r="K133" t="n">
-        <v>92.90000000000001</v>
+        <v>72.90000000000001</v>
       </c>
     </row>
     <row r="134">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6440,26 +6440,26 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F134" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G134" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H134" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I134" t="n">
         <v>35</v>
       </c>
       <c r="J134" t="n">
-        <v>28.8</v>
+        <v>32.7</v>
       </c>
       <c r="K134" t="n">
-        <v>82.3</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="135">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -6485,26 +6485,26 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F135" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G135" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H135" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I135" t="n">
         <v>35</v>
       </c>
       <c r="J135" t="n">
-        <v>27.6</v>
+        <v>32.5</v>
       </c>
       <c r="K135" t="n">
-        <v>78.90000000000001</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="136">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -6530,26 +6530,26 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F136" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G136" s="1" t="n">
-        <v>46270</v>
+        <v>46262</v>
       </c>
       <c r="H136" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I136" t="n">
         <v>35</v>
       </c>
       <c r="J136" t="n">
-        <v>36.5</v>
+        <v>28.6</v>
       </c>
       <c r="K136" t="n">
-        <v>104.3</v>
+        <v>81.7</v>
       </c>
     </row>
     <row r="137">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6575,26 +6575,26 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F137" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G137" s="1" t="n">
-        <v>46270</v>
+        <v>46262</v>
       </c>
       <c r="H137" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I137" t="n">
         <v>35</v>
       </c>
       <c r="J137" t="n">
-        <v>35.5</v>
+        <v>28.7</v>
       </c>
       <c r="K137" t="n">
-        <v>101.4</v>
+        <v>82</v>
       </c>
     </row>
     <row r="138">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -6620,26 +6620,26 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F138" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G138" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H138" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I138" t="n">
         <v>35</v>
       </c>
       <c r="J138" t="n">
-        <v>31.9</v>
+        <v>38.8</v>
       </c>
       <c r="K138" t="n">
-        <v>91.09999999999999</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="139">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -6665,26 +6665,26 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F139" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G139" s="1" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="H139" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I139" t="n">
         <v>35</v>
       </c>
       <c r="J139" t="n">
-        <v>31</v>
+        <v>38.6</v>
       </c>
       <c r="K139" t="n">
-        <v>88.59999999999999</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="140">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -6710,26 +6710,26 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F140" s="1" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="G140" s="1" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="H140" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I140" t="n">
         <v>35</v>
       </c>
       <c r="J140" t="n">
-        <v>31.9</v>
+        <v>33.7</v>
       </c>
       <c r="K140" t="n">
-        <v>91.09999999999999</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="141">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -6755,26 +6755,26 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F141" s="1" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="G141" s="1" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="H141" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I141" t="n">
         <v>35</v>
       </c>
       <c r="J141" t="n">
-        <v>30.5</v>
+        <v>32.5</v>
       </c>
       <c r="K141" t="n">
-        <v>87.09999999999999</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="142">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6800,26 +6800,26 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F142" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G142" s="1" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="H142" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I142" t="n">
         <v>35</v>
       </c>
       <c r="J142" t="n">
-        <v>26.9</v>
+        <v>32.3</v>
       </c>
       <c r="K142" t="n">
-        <v>76.90000000000001</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="143">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6845,26 +6845,26 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F143" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G143" s="1" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="H143" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I143" t="n">
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>26.5</v>
+        <v>32.5</v>
       </c>
       <c r="K143" t="n">
-        <v>75.7</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="144">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6890,26 +6890,26 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F144" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G144" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H144" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I144" t="n">
         <v>35</v>
       </c>
       <c r="J144" t="n">
-        <v>37.9</v>
+        <v>28.8</v>
       </c>
       <c r="K144" t="n">
-        <v>108.3</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="145">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6935,26 +6935,26 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F145" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G145" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H145" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I145" t="n">
         <v>35</v>
       </c>
       <c r="J145" t="n">
-        <v>38</v>
+        <v>27.6</v>
       </c>
       <c r="K145" t="n">
-        <v>108.6</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="146">
@@ -6965,7 +6965,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6980,26 +6980,26 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F146" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G146" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H146" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I146" t="n">
         <v>35</v>
       </c>
       <c r="J146" t="n">
-        <v>33.4</v>
+        <v>36.5</v>
       </c>
       <c r="K146" t="n">
-        <v>95.40000000000001</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="147">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -7025,26 +7025,26 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F147" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G147" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H147" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I147" t="n">
         <v>35</v>
       </c>
       <c r="J147" t="n">
-        <v>31.6</v>
+        <v>35.5</v>
       </c>
       <c r="K147" t="n">
-        <v>90.3</v>
+        <v>101.4</v>
       </c>
     </row>
     <row r="148">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -7070,26 +7070,26 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F148" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G148" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H148" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I148" t="n">
         <v>35</v>
       </c>
       <c r="J148" t="n">
-        <v>33</v>
+        <v>31.9</v>
       </c>
       <c r="K148" t="n">
-        <v>94.3</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="149">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7115,26 +7115,26 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F149" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G149" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H149" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I149" t="n">
         <v>35</v>
       </c>
       <c r="J149" t="n">
-        <v>32.6</v>
+        <v>31</v>
       </c>
       <c r="K149" t="n">
-        <v>93.09999999999999</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="150">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7160,26 +7160,26 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F150" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G150" s="1" t="n">
-        <v>46266</v>
+        <v>46272</v>
       </c>
       <c r="H150" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I150" t="n">
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>28.7</v>
+        <v>31.9</v>
       </c>
       <c r="K150" t="n">
-        <v>82</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="151">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7205,26 +7205,26 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F151" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G151" s="1" t="n">
-        <v>46266</v>
+        <v>46272</v>
       </c>
       <c r="H151" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I151" t="n">
         <v>35</v>
       </c>
       <c r="J151" t="n">
-        <v>26.9</v>
+        <v>30.5</v>
       </c>
       <c r="K151" t="n">
-        <v>76.90000000000001</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="152">
@@ -7235,12 +7235,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -7250,26 +7250,26 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F152" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G152" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H152" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I152" t="n">
         <v>35</v>
       </c>
       <c r="J152" t="n">
-        <v>38.9</v>
+        <v>26.9</v>
       </c>
       <c r="K152" t="n">
-        <v>111.1</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="153">
@@ -7280,12 +7280,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -7295,26 +7295,26 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F153" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G153" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H153" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I153" t="n">
         <v>35</v>
       </c>
       <c r="J153" t="n">
-        <v>38</v>
+        <v>26.5</v>
       </c>
       <c r="K153" t="n">
-        <v>108.6</v>
+        <v>75.7</v>
       </c>
     </row>
     <row r="154">
@@ -7325,12 +7325,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -7340,26 +7340,26 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F154" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G154" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H154" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I154" t="n">
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>34.1</v>
+        <v>37.9</v>
       </c>
       <c r="K154" t="n">
-        <v>97.40000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="155">
@@ -7370,12 +7370,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -7385,26 +7385,26 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F155" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G155" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H155" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I155" t="n">
         <v>35</v>
       </c>
       <c r="J155" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K155" t="n">
-        <v>94.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="156">
@@ -7415,12 +7415,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -7430,26 +7430,26 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F156" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G156" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H156" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I156" t="n">
         <v>35</v>
       </c>
       <c r="J156" t="n">
-        <v>43.4</v>
+        <v>33.4</v>
       </c>
       <c r="K156" t="n">
-        <v>124</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="157">
@@ -7460,12 +7460,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -7475,26 +7475,26 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F157" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G157" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H157" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I157" t="n">
         <v>35</v>
       </c>
       <c r="J157" t="n">
-        <v>43.9</v>
+        <v>31.6</v>
       </c>
       <c r="K157" t="n">
-        <v>125.4</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="158">
@@ -7505,12 +7505,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -7520,26 +7520,26 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F158" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G158" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H158" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I158" t="n">
         <v>35</v>
       </c>
       <c r="J158" t="n">
-        <v>37.8</v>
+        <v>33</v>
       </c>
       <c r="K158" t="n">
-        <v>108</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="159">
@@ -7550,12 +7550,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -7565,26 +7565,26 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F159" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G159" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H159" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I159" t="n">
         <v>35</v>
       </c>
       <c r="J159" t="n">
-        <v>36.5</v>
+        <v>32.6</v>
       </c>
       <c r="K159" t="n">
-        <v>104.3</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="160">
@@ -7595,12 +7595,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -7610,26 +7610,26 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F160" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G160" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H160" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I160" t="n">
         <v>35</v>
       </c>
       <c r="J160" t="n">
-        <v>36.3</v>
+        <v>28.7</v>
       </c>
       <c r="K160" t="n">
-        <v>103.7</v>
+        <v>82</v>
       </c>
     </row>
     <row r="161">
@@ -7640,12 +7640,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -7655,26 +7655,26 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F161" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G161" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H161" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I161" t="n">
         <v>35</v>
       </c>
       <c r="J161" t="n">
-        <v>36.6</v>
+        <v>26.9</v>
       </c>
       <c r="K161" t="n">
-        <v>104.6</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="162">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -7700,26 +7700,26 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F162" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G162" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H162" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I162" t="n">
         <v>35</v>
       </c>
       <c r="J162" t="n">
-        <v>31.6</v>
+        <v>38.9</v>
       </c>
       <c r="K162" t="n">
-        <v>90.3</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="163">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -7745,26 +7745,26 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F163" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G163" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H163" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I163" t="n">
         <v>35</v>
       </c>
       <c r="J163" t="n">
-        <v>30.2</v>
+        <v>38</v>
       </c>
       <c r="K163" t="n">
-        <v>86.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="164">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -7790,26 +7790,26 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F164" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G164" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H164" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I164" t="n">
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>38.1</v>
+        <v>34.1</v>
       </c>
       <c r="K164" t="n">
-        <v>108.9</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="165">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -7835,26 +7835,26 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F165" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G165" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H165" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I165" t="n">
         <v>35</v>
       </c>
       <c r="J165" t="n">
-        <v>38.6</v>
+        <v>33</v>
       </c>
       <c r="K165" t="n">
-        <v>110.3</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="166">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -7880,26 +7880,26 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F166" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G166" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H166" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I166" t="n">
         <v>35</v>
       </c>
       <c r="J166" t="n">
-        <v>32.1</v>
+        <v>43.4</v>
       </c>
       <c r="K166" t="n">
-        <v>91.7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="167">
@@ -7910,7 +7910,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -7925,26 +7925,26 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F167" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G167" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H167" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I167" t="n">
         <v>35</v>
       </c>
       <c r="J167" t="n">
-        <v>32.7</v>
+        <v>43.9</v>
       </c>
       <c r="K167" t="n">
-        <v>93.40000000000001</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="168">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -7970,26 +7970,26 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F168" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G168" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H168" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I168" t="n">
         <v>35</v>
       </c>
       <c r="J168" t="n">
-        <v>49</v>
+        <v>37.8</v>
       </c>
       <c r="K168" t="n">
-        <v>140</v>
+        <v>108</v>
       </c>
     </row>
     <row r="169">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8015,26 +8015,26 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F169" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G169" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H169" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I169" t="n">
         <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>49.6</v>
+        <v>36.5</v>
       </c>
       <c r="K169" t="n">
-        <v>141.7</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="170">
@@ -8045,7 +8045,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8060,26 +8060,26 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F170" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G170" s="1" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="H170" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I170" t="n">
         <v>35</v>
       </c>
       <c r="J170" t="n">
-        <v>40.9</v>
+        <v>36.3</v>
       </c>
       <c r="K170" t="n">
-        <v>116.9</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="171">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -8105,26 +8105,26 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F171" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G171" s="1" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="H171" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I171" t="n">
         <v>35</v>
       </c>
       <c r="J171" t="n">
-        <v>41.3</v>
+        <v>36.6</v>
       </c>
       <c r="K171" t="n">
-        <v>118</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="172">
@@ -8135,12 +8135,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -8150,14 +8150,14 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F172" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G172" s="1" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="H172" t="n">
         <v>7</v>
@@ -8166,10 +8166,10 @@
         <v>35</v>
       </c>
       <c r="J172" t="n">
-        <v>36.6</v>
+        <v>31.6</v>
       </c>
       <c r="K172" t="n">
-        <v>104.6</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="173">
@@ -8180,12 +8180,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -8195,14 +8195,14 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F173" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G173" s="1" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="H173" t="n">
         <v>7</v>
@@ -8211,10 +8211,10 @@
         <v>35</v>
       </c>
       <c r="J173" t="n">
-        <v>37.1</v>
+        <v>30.2</v>
       </c>
       <c r="K173" t="n">
-        <v>106</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="174">
@@ -8225,12 +8225,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -8240,26 +8240,26 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F174" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G174" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H174" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I174" t="n">
         <v>35</v>
       </c>
       <c r="J174" t="n">
-        <v>38.9</v>
+        <v>38.1</v>
       </c>
       <c r="K174" t="n">
-        <v>111.1</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="175">
@@ -8270,12 +8270,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -8285,26 +8285,26 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F175" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G175" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H175" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I175" t="n">
         <v>35</v>
       </c>
       <c r="J175" t="n">
-        <v>37.9</v>
+        <v>38.6</v>
       </c>
       <c r="K175" t="n">
-        <v>108.3</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="176">
@@ -8315,12 +8315,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -8330,14 +8330,14 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F176" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G176" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H176" t="n">
         <v>7</v>
@@ -8346,10 +8346,10 @@
         <v>35</v>
       </c>
       <c r="J176" t="n">
-        <v>40.3</v>
+        <v>32.1</v>
       </c>
       <c r="K176" t="n">
-        <v>115.1</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="177">
@@ -8360,12 +8360,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -8375,14 +8375,14 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F177" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G177" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H177" t="n">
         <v>7</v>
@@ -8391,10 +8391,10 @@
         <v>35</v>
       </c>
       <c r="J177" t="n">
-        <v>40.8</v>
+        <v>32.7</v>
       </c>
       <c r="K177" t="n">
-        <v>116.6</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="178">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -8420,26 +8420,26 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F178" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G178" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H178" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I178" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J178" t="n">
-        <v>27.1</v>
+        <v>49</v>
       </c>
       <c r="K178" t="n">
-        <v>110.6</v>
+        <v>140</v>
       </c>
     </row>
     <row r="179">
@@ -8450,12 +8450,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -8465,26 +8465,26 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F179" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G179" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H179" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I179" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>25.8</v>
+        <v>49.6</v>
       </c>
       <c r="K179" t="n">
-        <v>105.3</v>
+        <v>141.7</v>
       </c>
     </row>
     <row r="180">
@@ -8495,12 +8495,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -8510,26 +8510,26 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F180" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G180" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H180" t="n">
         <v>7</v>
       </c>
       <c r="I180" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J180" t="n">
-        <v>24.8</v>
+        <v>40.9</v>
       </c>
       <c r="K180" t="n">
-        <v>101.2</v>
+        <v>116.9</v>
       </c>
     </row>
     <row r="181">
@@ -8540,12 +8540,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -8555,26 +8555,566 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F181" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G181" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H181" t="n">
         <v>7</v>
       </c>
       <c r="I181" t="n">
+        <v>35</v>
+      </c>
+      <c r="J181" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="K181" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F182" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G182" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H182" t="n">
+        <v>7</v>
+      </c>
+      <c r="I182" t="n">
+        <v>35</v>
+      </c>
+      <c r="J182" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="K182" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F183" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G183" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H183" t="n">
+        <v>7</v>
+      </c>
+      <c r="I183" t="n">
+        <v>35</v>
+      </c>
+      <c r="J183" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="K183" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F184" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G184" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H184" t="n">
+        <v>7</v>
+      </c>
+      <c r="I184" t="n">
+        <v>35</v>
+      </c>
+      <c r="J184" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K184" t="n">
+        <v>111.1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F185" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G185" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H185" t="n">
+        <v>7</v>
+      </c>
+      <c r="I185" t="n">
+        <v>35</v>
+      </c>
+      <c r="J185" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="K185" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F186" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G186" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H186" t="n">
+        <v>7</v>
+      </c>
+      <c r="I186" t="n">
+        <v>35</v>
+      </c>
+      <c r="J186" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="K186" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F187" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G187" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H187" t="n">
+        <v>7</v>
+      </c>
+      <c r="I187" t="n">
+        <v>35</v>
+      </c>
+      <c r="J187" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K187" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F188" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G188" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H188" t="n">
+        <v>7</v>
+      </c>
+      <c r="I188" t="n">
         <v>24.5</v>
       </c>
-      <c r="J181" t="n">
+      <c r="J188" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K188" t="n">
+        <v>110.6</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F189" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G189" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H189" t="n">
+        <v>7</v>
+      </c>
+      <c r="I189" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J189" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K189" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F190" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G190" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H190" t="n">
+        <v>7</v>
+      </c>
+      <c r="I190" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J190" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K190" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F191" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G191" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H191" t="n">
+        <v>7</v>
+      </c>
+      <c r="I191" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J191" t="n">
         <v>24.6</v>
       </c>
-      <c r="K181" t="n">
+      <c r="K191" t="n">
         <v>100.4</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F192" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G192" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H192" t="n">
+        <v>7</v>
+      </c>
+      <c r="I192" t="n">
+        <v>35</v>
+      </c>
+      <c r="J192" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="K192" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F193" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G193" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H193" t="n">
+        <v>7</v>
+      </c>
+      <c r="I193" t="n">
+        <v>35</v>
+      </c>
+      <c r="J193" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K193" t="n">
+        <v>104.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-09-21 21:37:51
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K193"/>
+  <dimension ref="A1:K211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4152,19 +4152,19 @@
         <v>46269</v>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="H83" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I83" t="n">
         <v>35</v>
       </c>
       <c r="J83" t="n">
-        <v>27.2</v>
+        <v>38.1</v>
       </c>
       <c r="K83" t="n">
-        <v>77.7</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="84">
@@ -4197,19 +4197,19 @@
         <v>46269</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="H84" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I84" t="n">
         <v>35</v>
       </c>
       <c r="J84" t="n">
-        <v>27.6</v>
+        <v>38.6</v>
       </c>
       <c r="K84" t="n">
-        <v>78.90000000000001</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="85">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4235,26 +4235,26 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F85" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="H85" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I85" t="n">
         <v>35</v>
       </c>
       <c r="J85" t="n">
-        <v>37.2</v>
+        <v>27.2</v>
       </c>
       <c r="K85" t="n">
-        <v>106.3</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="86">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P-35</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4280,26 +4280,26 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Pilotes 23-15</t>
+          <t>Pilote 90 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F86" s="1" t="n">
-        <v>46249</v>
+        <v>46269</v>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="H86" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I86" t="n">
         <v>35</v>
       </c>
       <c r="J86" t="n">
-        <v>36.1</v>
+        <v>27.6</v>
       </c>
       <c r="K86" t="n">
-        <v>103.1</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="87">
@@ -4341,10 +4341,10 @@
         <v>35</v>
       </c>
       <c r="J87" t="n">
-        <v>36.5</v>
+        <v>37.2</v>
       </c>
       <c r="K87" t="n">
-        <v>104.3</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="88">
@@ -4377,19 +4377,19 @@
         <v>46249</v>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="H88" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I88" t="n">
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>31.2</v>
+        <v>36.1</v>
       </c>
       <c r="K88" t="n">
-        <v>89.09999999999999</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="89">
@@ -4422,19 +4422,19 @@
         <v>46249</v>
       </c>
       <c r="G89" s="1" t="n">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="H89" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I89" t="n">
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>31.6</v>
+        <v>36.5</v>
       </c>
       <c r="K89" t="n">
-        <v>90.3</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="90">
@@ -4467,19 +4467,19 @@
         <v>46249</v>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="H90" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I90" t="n">
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>23.3</v>
+        <v>31.2</v>
       </c>
       <c r="K90" t="n">
-        <v>66.59999999999999</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="91">
@@ -4512,19 +4512,19 @@
         <v>46249</v>
       </c>
       <c r="G91" s="1" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="H91" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I91" t="n">
         <v>35</v>
       </c>
       <c r="J91" t="n">
-        <v>23.5</v>
+        <v>31.6</v>
       </c>
       <c r="K91" t="n">
-        <v>67.09999999999999</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="92">
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4550,26 +4550,26 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F92" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G92" s="1" t="n">
-        <v>46280</v>
+        <v>46256</v>
       </c>
       <c r="H92" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I92" t="n">
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>49</v>
+        <v>23.3</v>
       </c>
       <c r="K92" t="n">
-        <v>140</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="93">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4595,26 +4595,26 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pilote 55</t>
+          <t>Pilotes 23-15</t>
         </is>
       </c>
       <c r="F93" s="1" t="n">
-        <v>46252</v>
+        <v>46249</v>
       </c>
       <c r="G93" s="1" t="n">
-        <v>46280</v>
+        <v>46256</v>
       </c>
       <c r="H93" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I93" t="n">
         <v>35</v>
       </c>
       <c r="J93" t="n">
-        <v>48</v>
+        <v>23.5</v>
       </c>
       <c r="K93" t="n">
-        <v>137.1</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="94">
@@ -4656,10 +4656,10 @@
         <v>35</v>
       </c>
       <c r="J94" t="n">
-        <v>47.5</v>
+        <v>49</v>
       </c>
       <c r="K94" t="n">
-        <v>135.7</v>
+        <v>140</v>
       </c>
     </row>
     <row r="95">
@@ -4692,19 +4692,19 @@
         <v>46252</v>
       </c>
       <c r="G95" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H95" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I95" t="n">
         <v>35</v>
       </c>
       <c r="J95" t="n">
-        <v>40.2</v>
+        <v>48</v>
       </c>
       <c r="K95" t="n">
-        <v>114.9</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="96">
@@ -4737,19 +4737,19 @@
         <v>46252</v>
       </c>
       <c r="G96" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H96" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I96" t="n">
         <v>35</v>
       </c>
       <c r="J96" t="n">
-        <v>39.9</v>
+        <v>47.5</v>
       </c>
       <c r="K96" t="n">
-        <v>114</v>
+        <v>135.7</v>
       </c>
     </row>
     <row r="97">
@@ -4782,19 +4782,19 @@
         <v>46252</v>
       </c>
       <c r="G97" s="1" t="n">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="H97" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I97" t="n">
         <v>35</v>
       </c>
       <c r="J97" t="n">
-        <v>34.7</v>
+        <v>40.2</v>
       </c>
       <c r="K97" t="n">
-        <v>99.09999999999999</v>
+        <v>114.9</v>
       </c>
     </row>
     <row r="98">
@@ -4827,19 +4827,19 @@
         <v>46252</v>
       </c>
       <c r="G98" s="1" t="n">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="H98" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I98" t="n">
         <v>35</v>
       </c>
       <c r="J98" t="n">
-        <v>33.4</v>
+        <v>39.9</v>
       </c>
       <c r="K98" t="n">
-        <v>95.40000000000001</v>
+        <v>114</v>
       </c>
     </row>
     <row r="99">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4865,26 +4865,26 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F99" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G99" s="1" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="H99" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I99" t="n">
         <v>35</v>
       </c>
       <c r="J99" t="n">
-        <v>39.5</v>
+        <v>34.7</v>
       </c>
       <c r="K99" t="n">
-        <v>112.9</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="100">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4910,26 +4910,26 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pilote 50</t>
+          <t>Pilote 55</t>
         </is>
       </c>
       <c r="F100" s="1" t="n">
         <v>46252</v>
       </c>
       <c r="G100" s="1" t="n">
-        <v>46280</v>
+        <v>46259</v>
       </c>
       <c r="H100" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I100" t="n">
         <v>35</v>
       </c>
       <c r="J100" t="n">
-        <v>40.1</v>
+        <v>33.4</v>
       </c>
       <c r="K100" t="n">
-        <v>114.6</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="101">
@@ -4971,10 +4971,10 @@
         <v>35</v>
       </c>
       <c r="J101" t="n">
-        <v>39.7</v>
+        <v>39.5</v>
       </c>
       <c r="K101" t="n">
-        <v>113.4</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="102">
@@ -5007,19 +5007,19 @@
         <v>46252</v>
       </c>
       <c r="G102" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H102" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I102" t="n">
         <v>35</v>
       </c>
       <c r="J102" t="n">
-        <v>30.9</v>
+        <v>40.1</v>
       </c>
       <c r="K102" t="n">
-        <v>88.3</v>
+        <v>114.6</v>
       </c>
     </row>
     <row r="103">
@@ -5052,19 +5052,19 @@
         <v>46252</v>
       </c>
       <c r="G103" s="1" t="n">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="H103" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I103" t="n">
         <v>35</v>
       </c>
       <c r="J103" t="n">
-        <v>31.3</v>
+        <v>39.7</v>
       </c>
       <c r="K103" t="n">
-        <v>89.40000000000001</v>
+        <v>113.4</v>
       </c>
     </row>
     <row r="104">
@@ -5097,19 +5097,19 @@
         <v>46252</v>
       </c>
       <c r="G104" s="1" t="n">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="H104" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I104" t="n">
         <v>35</v>
       </c>
       <c r="J104" t="n">
-        <v>25</v>
+        <v>30.9</v>
       </c>
       <c r="K104" t="n">
-        <v>71.40000000000001</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="105">
@@ -5142,19 +5142,19 @@
         <v>46252</v>
       </c>
       <c r="G105" s="1" t="n">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="H105" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I105" t="n">
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>24.5</v>
+        <v>31.3</v>
       </c>
       <c r="K105" t="n">
-        <v>70</v>
+        <v>89.40000000000001</v>
       </c>
     </row>
     <row r="106">
@@ -5165,12 +5165,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5180,26 +5180,26 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F106" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G106" s="1" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="H106" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I106" t="n">
         <v>35</v>
       </c>
       <c r="J106" t="n">
-        <v>43.5</v>
+        <v>25</v>
       </c>
       <c r="K106" t="n">
-        <v>124.3</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="107">
@@ -5210,12 +5210,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5225,26 +5225,26 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 46 Torre 1 </t>
+          <t>Pilote 50</t>
         </is>
       </c>
       <c r="F107" s="1" t="n">
-        <v>46253</v>
+        <v>46252</v>
       </c>
       <c r="G107" s="1" t="n">
-        <v>46281</v>
+        <v>46259</v>
       </c>
       <c r="H107" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I107" t="n">
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>41.6</v>
+        <v>24.5</v>
       </c>
       <c r="K107" t="n">
-        <v>118.9</v>
+        <v>70</v>
       </c>
     </row>
     <row r="108">
@@ -5286,10 +5286,10 @@
         <v>35</v>
       </c>
       <c r="J108" t="n">
-        <v>42.2</v>
+        <v>43.5</v>
       </c>
       <c r="K108" t="n">
-        <v>120.6</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="109">
@@ -5322,19 +5322,19 @@
         <v>46253</v>
       </c>
       <c r="G109" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H109" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I109" t="n">
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>34.2</v>
+        <v>41.6</v>
       </c>
       <c r="K109" t="n">
-        <v>97.7</v>
+        <v>118.9</v>
       </c>
     </row>
     <row r="110">
@@ -5367,19 +5367,19 @@
         <v>46253</v>
       </c>
       <c r="G110" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H110" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I110" t="n">
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>34.6</v>
+        <v>42.2</v>
       </c>
       <c r="K110" t="n">
-        <v>98.90000000000001</v>
+        <v>120.6</v>
       </c>
     </row>
     <row r="111">
@@ -5412,19 +5412,19 @@
         <v>46253</v>
       </c>
       <c r="G111" s="1" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="H111" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I111" t="n">
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>21.3</v>
+        <v>34.2</v>
       </c>
       <c r="K111" t="n">
-        <v>60.9</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="112">
@@ -5457,19 +5457,19 @@
         <v>46253</v>
       </c>
       <c r="G112" s="1" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="H112" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I112" t="n">
         <v>35</v>
       </c>
       <c r="J112" t="n">
-        <v>21.5</v>
+        <v>34.6</v>
       </c>
       <c r="K112" t="n">
-        <v>61.4</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="113">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5495,26 +5495,26 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F113" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G113" s="1" t="n">
-        <v>46281</v>
+        <v>46260</v>
       </c>
       <c r="H113" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I113" t="n">
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>45.7</v>
+        <v>21.3</v>
       </c>
       <c r="K113" t="n">
-        <v>130.6</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="114">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5540,26 +5540,26 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 46 Torre 1 </t>
         </is>
       </c>
       <c r="F114" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="G114" s="1" t="n">
-        <v>46281</v>
+        <v>46260</v>
       </c>
       <c r="H114" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I114" t="n">
         <v>35</v>
       </c>
       <c r="J114" t="n">
-        <v>46.1</v>
+        <v>21.5</v>
       </c>
       <c r="K114" t="n">
-        <v>131.7</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="115">
@@ -5601,10 +5601,10 @@
         <v>35</v>
       </c>
       <c r="J115" t="n">
-        <v>44.4</v>
+        <v>45.7</v>
       </c>
       <c r="K115" t="n">
-        <v>126.9</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="116">
@@ -5637,19 +5637,19 @@
         <v>46253</v>
       </c>
       <c r="G116" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H116" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I116" t="n">
         <v>35</v>
       </c>
       <c r="J116" t="n">
-        <v>37.9</v>
+        <v>46.1</v>
       </c>
       <c r="K116" t="n">
-        <v>108.3</v>
+        <v>131.7</v>
       </c>
     </row>
     <row r="117">
@@ -5682,19 +5682,19 @@
         <v>46253</v>
       </c>
       <c r="G117" s="1" t="n">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="H117" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I117" t="n">
         <v>35</v>
       </c>
       <c r="J117" t="n">
-        <v>38.4</v>
+        <v>44.4</v>
       </c>
       <c r="K117" t="n">
-        <v>109.7</v>
+        <v>126.9</v>
       </c>
     </row>
     <row r="118">
@@ -5727,19 +5727,19 @@
         <v>46253</v>
       </c>
       <c r="G118" s="1" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="H118" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I118" t="n">
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>34.6</v>
+        <v>37.9</v>
       </c>
       <c r="K118" t="n">
-        <v>98.90000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="119">
@@ -5772,19 +5772,19 @@
         <v>46253</v>
       </c>
       <c r="G119" s="1" t="n">
-        <v>46260</v>
+        <v>46267</v>
       </c>
       <c r="H119" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I119" t="n">
         <v>35</v>
       </c>
       <c r="J119" t="n">
-        <v>34.8</v>
+        <v>38.4</v>
       </c>
       <c r="K119" t="n">
-        <v>99.40000000000001</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="120">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5810,26 +5810,26 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F120" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G120" s="1" t="n">
-        <v>46282</v>
+        <v>46260</v>
       </c>
       <c r="H120" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I120" t="n">
         <v>35</v>
       </c>
       <c r="J120" t="n">
-        <v>39.1</v>
+        <v>34.6</v>
       </c>
       <c r="K120" t="n">
-        <v>111.7</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="121">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5855,26 +5855,26 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 25 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F121" s="1" t="n">
-        <v>46254</v>
+        <v>46253</v>
       </c>
       <c r="G121" s="1" t="n">
-        <v>46282</v>
+        <v>46260</v>
       </c>
       <c r="H121" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I121" t="n">
         <v>35</v>
       </c>
       <c r="J121" t="n">
-        <v>39.6</v>
+        <v>34.8</v>
       </c>
       <c r="K121" t="n">
-        <v>113.1</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="122">
@@ -5916,10 +5916,10 @@
         <v>35</v>
       </c>
       <c r="J122" t="n">
-        <v>40.2</v>
+        <v>39.1</v>
       </c>
       <c r="K122" t="n">
-        <v>114.9</v>
+        <v>111.7</v>
       </c>
     </row>
     <row r="123">
@@ -5952,19 +5952,19 @@
         <v>46254</v>
       </c>
       <c r="G123" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H123" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I123" t="n">
         <v>35</v>
       </c>
       <c r="J123" t="n">
-        <v>30.9</v>
+        <v>39.6</v>
       </c>
       <c r="K123" t="n">
-        <v>88.3</v>
+        <v>113.1</v>
       </c>
     </row>
     <row r="124">
@@ -5997,19 +5997,19 @@
         <v>46254</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H124" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I124" t="n">
         <v>35</v>
       </c>
       <c r="J124" t="n">
-        <v>32.3</v>
+        <v>40.2</v>
       </c>
       <c r="K124" t="n">
-        <v>92.3</v>
+        <v>114.9</v>
       </c>
     </row>
     <row r="125">
@@ -6042,19 +6042,19 @@
         <v>46254</v>
       </c>
       <c r="G125" s="1" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="H125" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I125" t="n">
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>25.8</v>
+        <v>30.9</v>
       </c>
       <c r="K125" t="n">
-        <v>73.7</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="126">
@@ -6087,19 +6087,19 @@
         <v>46254</v>
       </c>
       <c r="G126" s="1" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="H126" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I126" t="n">
         <v>35</v>
       </c>
       <c r="J126" t="n">
-        <v>23.9</v>
+        <v>32.3</v>
       </c>
       <c r="K126" t="n">
-        <v>68.3</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="127">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -6125,26 +6125,26 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F127" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G127" s="1" t="n">
-        <v>46282</v>
+        <v>46261</v>
       </c>
       <c r="H127" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I127" t="n">
         <v>35</v>
       </c>
       <c r="J127" t="n">
-        <v>42.8</v>
+        <v>25.8</v>
       </c>
       <c r="K127" t="n">
-        <v>122.3</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="128">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -6170,26 +6170,26 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
+          <t xml:space="preserve">Pilote 49 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F128" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="G128" s="1" t="n">
-        <v>46282</v>
+        <v>46261</v>
       </c>
       <c r="H128" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="I128" t="n">
         <v>35</v>
       </c>
       <c r="J128" t="n">
-        <v>41.1</v>
+        <v>23.9</v>
       </c>
       <c r="K128" t="n">
-        <v>117.4</v>
+        <v>68.3</v>
       </c>
     </row>
     <row r="129">
@@ -6231,10 +6231,10 @@
         <v>35</v>
       </c>
       <c r="J129" t="n">
-        <v>41.4</v>
+        <v>42.8</v>
       </c>
       <c r="K129" t="n">
-        <v>118.3</v>
+        <v>122.3</v>
       </c>
     </row>
     <row r="130">
@@ -6267,19 +6267,19 @@
         <v>46254</v>
       </c>
       <c r="G130" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H130" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I130" t="n">
         <v>35</v>
       </c>
       <c r="J130" t="n">
-        <v>33.8</v>
+        <v>41.1</v>
       </c>
       <c r="K130" t="n">
-        <v>96.59999999999999</v>
+        <v>117.4</v>
       </c>
     </row>
     <row r="131">
@@ -6312,19 +6312,19 @@
         <v>46254</v>
       </c>
       <c r="G131" s="1" t="n">
-        <v>46268</v>
+        <v>46282</v>
       </c>
       <c r="H131" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I131" t="n">
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>32.1</v>
+        <v>41.4</v>
       </c>
       <c r="K131" t="n">
-        <v>91.7</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="132">
@@ -6357,19 +6357,19 @@
         <v>46254</v>
       </c>
       <c r="G132" s="1" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="H132" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I132" t="n">
         <v>35</v>
       </c>
       <c r="J132" t="n">
-        <v>25.7</v>
+        <v>33.8</v>
       </c>
       <c r="K132" t="n">
-        <v>73.40000000000001</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="133">
@@ -6402,19 +6402,19 @@
         <v>46254</v>
       </c>
       <c r="G133" s="1" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="H133" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I133" t="n">
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>25.5</v>
+        <v>32.1</v>
       </c>
       <c r="K133" t="n">
-        <v>72.90000000000001</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="134">
@@ -6425,12 +6425,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -6440,26 +6440,26 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F134" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G134" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="H134" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I134" t="n">
         <v>35</v>
       </c>
       <c r="J134" t="n">
-        <v>32.7</v>
+        <v>25.7</v>
       </c>
       <c r="K134" t="n">
-        <v>93.40000000000001</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="135">
@@ -6470,12 +6470,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -6485,26 +6485,26 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Pilote 9 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 44 Torre 1 Tipo 2 </t>
         </is>
       </c>
       <c r="F135" s="1" t="n">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="G135" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="H135" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I135" t="n">
         <v>35</v>
       </c>
       <c r="J135" t="n">
-        <v>32.5</v>
+        <v>25.5</v>
       </c>
       <c r="K135" t="n">
-        <v>92.90000000000001</v>
+        <v>72.90000000000001</v>
       </c>
     </row>
     <row r="136">
@@ -6537,19 +6537,19 @@
         <v>46255</v>
       </c>
       <c r="G136" s="1" t="n">
-        <v>46262</v>
+        <v>46283</v>
       </c>
       <c r="H136" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I136" t="n">
         <v>35</v>
       </c>
       <c r="J136" t="n">
-        <v>28.6</v>
+        <v>37.9</v>
       </c>
       <c r="K136" t="n">
-        <v>81.7</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="137">
@@ -6582,19 +6582,19 @@
         <v>46255</v>
       </c>
       <c r="G137" s="1" t="n">
-        <v>46262</v>
+        <v>46283</v>
       </c>
       <c r="H137" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I137" t="n">
         <v>35</v>
       </c>
       <c r="J137" t="n">
-        <v>28.7</v>
+        <v>36.9</v>
       </c>
       <c r="K137" t="n">
-        <v>82</v>
+        <v>105.4</v>
       </c>
     </row>
     <row r="138">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -6620,26 +6620,26 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F138" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="G138" s="1" t="n">
-        <v>46269</v>
+        <v>46283</v>
       </c>
       <c r="H138" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I138" t="n">
         <v>35</v>
       </c>
       <c r="J138" t="n">
-        <v>38.8</v>
+        <v>37.8</v>
       </c>
       <c r="K138" t="n">
-        <v>110.9</v>
+        <v>108</v>
       </c>
     </row>
     <row r="139">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F139" s="1" t="n">
@@ -6681,10 +6681,10 @@
         <v>35</v>
       </c>
       <c r="J139" t="n">
-        <v>38.6</v>
+        <v>32.7</v>
       </c>
       <c r="K139" t="n">
-        <v>110.3</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="140">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -6710,26 +6710,26 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F140" s="1" t="n">
         <v>46255</v>
       </c>
       <c r="G140" s="1" t="n">
-        <v>46262</v>
+        <v>46269</v>
       </c>
       <c r="H140" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I140" t="n">
         <v>35</v>
       </c>
       <c r="J140" t="n">
-        <v>33.7</v>
+        <v>32.5</v>
       </c>
       <c r="K140" t="n">
-        <v>96.3</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="141">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -6755,7 +6755,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F141" s="1" t="n">
@@ -6771,10 +6771,10 @@
         <v>35</v>
       </c>
       <c r="J141" t="n">
-        <v>32.5</v>
+        <v>28.6</v>
       </c>
       <c r="K141" t="n">
-        <v>92.90000000000001</v>
+        <v>81.7</v>
       </c>
     </row>
     <row r="142">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6800,26 +6800,26 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 9 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F142" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G142" s="1" t="n">
-        <v>46270</v>
+        <v>46262</v>
       </c>
       <c r="H142" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I142" t="n">
         <v>35</v>
       </c>
       <c r="J142" t="n">
-        <v>32.3</v>
+        <v>28.7</v>
       </c>
       <c r="K142" t="n">
-        <v>92.3</v>
+        <v>82</v>
       </c>
     </row>
     <row r="143">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6845,26 +6845,26 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F143" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G143" s="1" t="n">
-        <v>46270</v>
+        <v>46283</v>
       </c>
       <c r="H143" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I143" t="n">
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>32.5</v>
+        <v>46.3</v>
       </c>
       <c r="K143" t="n">
-        <v>92.90000000000001</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="144">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6890,26 +6890,26 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F144" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G144" s="1" t="n">
-        <v>46263</v>
+        <v>46283</v>
       </c>
       <c r="H144" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I144" t="n">
         <v>35</v>
       </c>
       <c r="J144" t="n">
-        <v>28.8</v>
+        <v>46.9</v>
       </c>
       <c r="K144" t="n">
-        <v>82.3</v>
+        <v>134</v>
       </c>
     </row>
     <row r="145">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>P17</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6935,26 +6935,26 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Pilote 22 torre 1 tipo 1</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F145" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G145" s="1" t="n">
-        <v>46263</v>
+        <v>46283</v>
       </c>
       <c r="H145" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I145" t="n">
         <v>35</v>
       </c>
       <c r="J145" t="n">
-        <v>27.6</v>
+        <v>46.8</v>
       </c>
       <c r="K145" t="n">
-        <v>78.90000000000001</v>
+        <v>133.7</v>
       </c>
     </row>
     <row r="146">
@@ -6965,7 +6965,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6980,14 +6980,14 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F146" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G146" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="H146" t="n">
         <v>14</v>
@@ -6996,10 +6996,10 @@
         <v>35</v>
       </c>
       <c r="J146" t="n">
-        <v>36.5</v>
+        <v>38.8</v>
       </c>
       <c r="K146" t="n">
-        <v>104.3</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="147">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -7025,14 +7025,14 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F147" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G147" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="H147" t="n">
         <v>14</v>
@@ -7041,10 +7041,10 @@
         <v>35</v>
       </c>
       <c r="J147" t="n">
-        <v>35.5</v>
+        <v>38.6</v>
       </c>
       <c r="K147" t="n">
-        <v>101.4</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="148">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -7070,14 +7070,14 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F148" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G148" s="1" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="H148" t="n">
         <v>7</v>
@@ -7086,10 +7086,10 @@
         <v>35</v>
       </c>
       <c r="J148" t="n">
-        <v>31.9</v>
+        <v>33.7</v>
       </c>
       <c r="K148" t="n">
-        <v>91.09999999999999</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="149">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>P18</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7115,14 +7115,14 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Pilote 45 torre 1 tipo 2</t>
+          <t>Pilote 54 torre 2 tipo 2 pilote 26 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F149" s="1" t="n">
-        <v>46256</v>
+        <v>46255</v>
       </c>
       <c r="G149" s="1" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="H149" t="n">
         <v>7</v>
@@ -7131,10 +7131,10 @@
         <v>35</v>
       </c>
       <c r="J149" t="n">
-        <v>31</v>
+        <v>32.5</v>
       </c>
       <c r="K149" t="n">
-        <v>88.59999999999999</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="150">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7160,26 +7160,26 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F150" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G150" s="1" t="n">
-        <v>46272</v>
+        <v>46284</v>
       </c>
       <c r="H150" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I150" t="n">
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>31.9</v>
+        <v>40.5</v>
       </c>
       <c r="K150" t="n">
-        <v>91.09999999999999</v>
+        <v>115.7</v>
       </c>
     </row>
     <row r="151">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7205,26 +7205,26 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F151" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G151" s="1" t="n">
-        <v>46272</v>
+        <v>46284</v>
       </c>
       <c r="H151" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I151" t="n">
         <v>35</v>
       </c>
       <c r="J151" t="n">
-        <v>30.5</v>
+        <v>39</v>
       </c>
       <c r="K151" t="n">
-        <v>87.09999999999999</v>
+        <v>111.4</v>
       </c>
     </row>
     <row r="152">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7250,26 +7250,26 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F152" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G152" s="1" t="n">
-        <v>46265</v>
+        <v>46284</v>
       </c>
       <c r="H152" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I152" t="n">
         <v>35</v>
       </c>
       <c r="J152" t="n">
-        <v>26.9</v>
+        <v>39.5</v>
       </c>
       <c r="K152" t="n">
-        <v>76.90000000000001</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="153">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>P19</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7295,26 +7295,26 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F153" s="1" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="G153" s="1" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="H153" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I153" t="n">
         <v>35</v>
       </c>
       <c r="J153" t="n">
-        <v>26.5</v>
+        <v>32.3</v>
       </c>
       <c r="K153" t="n">
-        <v>75.7</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="154">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7340,14 +7340,14 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F154" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G154" s="1" t="n">
-        <v>46273</v>
+        <v>46270</v>
       </c>
       <c r="H154" t="n">
         <v>14</v>
@@ -7356,10 +7356,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>37.9</v>
+        <v>32.5</v>
       </c>
       <c r="K154" t="n">
-        <v>108.3</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="155">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7385,26 +7385,26 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F155" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G155" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="H155" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I155" t="n">
         <v>35</v>
       </c>
       <c r="J155" t="n">
-        <v>38</v>
+        <v>28.8</v>
       </c>
       <c r="K155" t="n">
-        <v>108.6</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="156">
@@ -7415,7 +7415,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P17</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7430,14 +7430,14 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 22 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F156" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G156" s="1" t="n">
-        <v>46266</v>
+        <v>46263</v>
       </c>
       <c r="H156" t="n">
         <v>7</v>
@@ -7446,10 +7446,10 @@
         <v>35</v>
       </c>
       <c r="J156" t="n">
-        <v>33.4</v>
+        <v>27.6</v>
       </c>
       <c r="K156" t="n">
-        <v>95.40000000000001</v>
+        <v>78.90000000000001</v>
       </c>
     </row>
     <row r="157">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7475,26 +7475,26 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F157" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G157" s="1" t="n">
-        <v>46266</v>
+        <v>46284</v>
       </c>
       <c r="H157" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I157" t="n">
         <v>35</v>
       </c>
       <c r="J157" t="n">
-        <v>31.6</v>
+        <v>43.3</v>
       </c>
       <c r="K157" t="n">
-        <v>90.3</v>
+        <v>123.7</v>
       </c>
     </row>
     <row r="158">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7520,26 +7520,26 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F158" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G158" s="1" t="n">
-        <v>46273</v>
+        <v>46284</v>
       </c>
       <c r="H158" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I158" t="n">
         <v>35</v>
       </c>
       <c r="J158" t="n">
-        <v>33</v>
+        <v>42.9</v>
       </c>
       <c r="K158" t="n">
-        <v>94.3</v>
+        <v>122.6</v>
       </c>
     </row>
     <row r="159">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -7565,26 +7565,26 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F159" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G159" s="1" t="n">
-        <v>46273</v>
+        <v>46284</v>
       </c>
       <c r="H159" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I159" t="n">
         <v>35</v>
       </c>
       <c r="J159" t="n">
-        <v>32.6</v>
+        <v>43.6</v>
       </c>
       <c r="K159" t="n">
-        <v>93.09999999999999</v>
+        <v>124.6</v>
       </c>
     </row>
     <row r="160">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7610,26 +7610,26 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F160" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G160" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H160" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I160" t="n">
         <v>35</v>
       </c>
       <c r="J160" t="n">
-        <v>28.7</v>
+        <v>36.5</v>
       </c>
       <c r="K160" t="n">
-        <v>82</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="161">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7655,26 +7655,26 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F161" s="1" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="G161" s="1" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="H161" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I161" t="n">
         <v>35</v>
       </c>
       <c r="J161" t="n">
-        <v>26.9</v>
+        <v>35.5</v>
       </c>
       <c r="K161" t="n">
-        <v>76.90000000000001</v>
+        <v>101.4</v>
       </c>
     </row>
     <row r="162">
@@ -7685,12 +7685,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -7700,26 +7700,26 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F162" s="1" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="G162" s="1" t="n">
-        <v>46274</v>
+        <v>46263</v>
       </c>
       <c r="H162" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I162" t="n">
         <v>35</v>
       </c>
       <c r="J162" t="n">
-        <v>38.9</v>
+        <v>31.9</v>
       </c>
       <c r="K162" t="n">
-        <v>111.1</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="163">
@@ -7730,12 +7730,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P18</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -7745,26 +7745,26 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t>Pilote 45 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F163" s="1" t="n">
-        <v>46260</v>
+        <v>46256</v>
       </c>
       <c r="G163" s="1" t="n">
-        <v>46274</v>
+        <v>46263</v>
       </c>
       <c r="H163" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I163" t="n">
         <v>35</v>
       </c>
       <c r="J163" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="K163" t="n">
-        <v>108.6</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="164">
@@ -7775,12 +7775,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -7790,26 +7790,26 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F164" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G164" s="1" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="H164" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I164" t="n">
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>34.1</v>
+        <v>31.9</v>
       </c>
       <c r="K164" t="n">
-        <v>97.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="165">
@@ -7820,12 +7820,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -7835,26 +7835,26 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F165" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G165" s="1" t="n">
-        <v>46267</v>
+        <v>46272</v>
       </c>
       <c r="H165" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I165" t="n">
         <v>35</v>
       </c>
       <c r="J165" t="n">
-        <v>33</v>
+        <v>30.5</v>
       </c>
       <c r="K165" t="n">
-        <v>94.3</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="166">
@@ -7865,12 +7865,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -7880,26 +7880,26 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F166" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G166" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H166" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I166" t="n">
         <v>35</v>
       </c>
       <c r="J166" t="n">
-        <v>43.4</v>
+        <v>26.9</v>
       </c>
       <c r="K166" t="n">
-        <v>124</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="167">
@@ -7910,12 +7910,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -7925,26 +7925,26 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F167" s="1" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="G167" s="1" t="n">
-        <v>46274</v>
+        <v>46265</v>
       </c>
       <c r="H167" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I167" t="n">
         <v>35</v>
       </c>
       <c r="J167" t="n">
-        <v>43.9</v>
+        <v>26.5</v>
       </c>
       <c r="K167" t="n">
-        <v>125.4</v>
+        <v>75.7</v>
       </c>
     </row>
     <row r="168">
@@ -7955,12 +7955,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -7970,26 +7970,26 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F168" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G168" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H168" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I168" t="n">
         <v>35</v>
       </c>
       <c r="J168" t="n">
-        <v>37.8</v>
+        <v>37.9</v>
       </c>
       <c r="K168" t="n">
-        <v>108</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="169">
@@ -8000,12 +8000,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -8015,26 +8015,26 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F169" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G169" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H169" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I169" t="n">
         <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>36.5</v>
+        <v>38</v>
       </c>
       <c r="K169" t="n">
-        <v>104.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="170">
@@ -8045,12 +8045,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -8060,26 +8060,26 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F170" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G170" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H170" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I170" t="n">
         <v>35</v>
       </c>
       <c r="J170" t="n">
-        <v>36.3</v>
+        <v>33.4</v>
       </c>
       <c r="K170" t="n">
-        <v>103.7</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="171">
@@ -8090,12 +8090,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -8105,26 +8105,26 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F171" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G171" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H171" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I171" t="n">
         <v>35</v>
       </c>
       <c r="J171" t="n">
-        <v>36.6</v>
+        <v>31.6</v>
       </c>
       <c r="K171" t="n">
-        <v>104.6</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="172">
@@ -8135,12 +8135,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -8150,26 +8150,26 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F172" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G172" s="1" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="H172" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I172" t="n">
         <v>35</v>
       </c>
       <c r="J172" t="n">
-        <v>31.6</v>
+        <v>33</v>
       </c>
       <c r="K172" t="n">
-        <v>90.3</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="173">
@@ -8180,12 +8180,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -8195,26 +8195,26 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F173" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G173" s="1" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="H173" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I173" t="n">
         <v>35</v>
       </c>
       <c r="J173" t="n">
-        <v>30.2</v>
+        <v>32.6</v>
       </c>
       <c r="K173" t="n">
-        <v>86.3</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="174">
@@ -8225,12 +8225,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -8240,26 +8240,26 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F174" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G174" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H174" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I174" t="n">
         <v>35</v>
       </c>
       <c r="J174" t="n">
-        <v>38.1</v>
+        <v>28.7</v>
       </c>
       <c r="K174" t="n">
-        <v>108.9</v>
+        <v>82</v>
       </c>
     </row>
     <row r="175">
@@ -8270,12 +8270,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -8285,26 +8285,26 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F175" s="1" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="G175" s="1" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="H175" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I175" t="n">
         <v>35</v>
       </c>
       <c r="J175" t="n">
-        <v>38.6</v>
+        <v>26.9</v>
       </c>
       <c r="K175" t="n">
-        <v>110.3</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="176">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8330,26 +8330,26 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F176" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G176" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H176" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I176" t="n">
         <v>35</v>
       </c>
       <c r="J176" t="n">
-        <v>32.1</v>
+        <v>38.9</v>
       </c>
       <c r="K176" t="n">
-        <v>91.7</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="177">
@@ -8360,7 +8360,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8375,26 +8375,26 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F177" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G177" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H177" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I177" t="n">
         <v>35</v>
       </c>
       <c r="J177" t="n">
-        <v>32.7</v>
+        <v>38</v>
       </c>
       <c r="K177" t="n">
-        <v>93.40000000000001</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="178">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8420,26 +8420,26 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F178" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G178" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H178" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I178" t="n">
         <v>35</v>
       </c>
       <c r="J178" t="n">
-        <v>49</v>
+        <v>34.1</v>
       </c>
       <c r="K178" t="n">
-        <v>140</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="179">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -8465,26 +8465,26 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F179" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G179" s="1" t="n">
-        <v>46277</v>
+        <v>46267</v>
       </c>
       <c r="H179" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I179" t="n">
         <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>49.6</v>
+        <v>33</v>
       </c>
       <c r="K179" t="n">
-        <v>141.7</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="180">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8510,26 +8510,26 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F180" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G180" s="1" t="n">
-        <v>46270</v>
+        <v>46274</v>
       </c>
       <c r="H180" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I180" t="n">
         <v>35</v>
       </c>
       <c r="J180" t="n">
-        <v>40.9</v>
+        <v>43.4</v>
       </c>
       <c r="K180" t="n">
-        <v>116.9</v>
+        <v>124</v>
       </c>
     </row>
     <row r="181">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -8555,26 +8555,26 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F181" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G181" s="1" t="n">
-        <v>46270</v>
+        <v>46274</v>
       </c>
       <c r="H181" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I181" t="n">
         <v>35</v>
       </c>
       <c r="J181" t="n">
-        <v>41.3</v>
+        <v>43.9</v>
       </c>
       <c r="K181" t="n">
-        <v>118</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="182">
@@ -8585,12 +8585,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -8600,14 +8600,14 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F182" s="1" t="n">
-        <v>46269</v>
+        <v>46260</v>
       </c>
       <c r="G182" s="1" t="n">
-        <v>46276</v>
+        <v>46267</v>
       </c>
       <c r="H182" t="n">
         <v>7</v>
@@ -8616,10 +8616,10 @@
         <v>35</v>
       </c>
       <c r="J182" t="n">
-        <v>36.6</v>
+        <v>37.8</v>
       </c>
       <c r="K182" t="n">
-        <v>104.6</v>
+        <v>108</v>
       </c>
     </row>
     <row r="183">
@@ -8630,12 +8630,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -8645,14 +8645,14 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F183" s="1" t="n">
-        <v>46269</v>
+        <v>46260</v>
       </c>
       <c r="G183" s="1" t="n">
-        <v>46276</v>
+        <v>46267</v>
       </c>
       <c r="H183" t="n">
         <v>7</v>
@@ -8661,10 +8661,10 @@
         <v>35</v>
       </c>
       <c r="J183" t="n">
-        <v>37.1</v>
+        <v>36.5</v>
       </c>
       <c r="K183" t="n">
-        <v>106</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="184">
@@ -8675,12 +8675,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -8690,26 +8690,26 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F184" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G184" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H184" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I184" t="n">
         <v>35</v>
       </c>
       <c r="J184" t="n">
-        <v>38.9</v>
+        <v>36.3</v>
       </c>
       <c r="K184" t="n">
-        <v>111.1</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="185">
@@ -8720,12 +8720,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -8735,26 +8735,26 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F185" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G185" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H185" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I185" t="n">
         <v>35</v>
       </c>
       <c r="J185" t="n">
-        <v>37.9</v>
+        <v>36.6</v>
       </c>
       <c r="K185" t="n">
-        <v>108.3</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="186">
@@ -8765,12 +8765,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -8780,14 +8780,14 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F186" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G186" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H186" t="n">
         <v>7</v>
@@ -8796,10 +8796,10 @@
         <v>35</v>
       </c>
       <c r="J186" t="n">
-        <v>40.3</v>
+        <v>31.6</v>
       </c>
       <c r="K186" t="n">
-        <v>115.1</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="187">
@@ -8810,12 +8810,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -8825,14 +8825,14 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F187" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G187" s="1" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="H187" t="n">
         <v>7</v>
@@ -8841,10 +8841,10 @@
         <v>35</v>
       </c>
       <c r="J187" t="n">
-        <v>40.8</v>
+        <v>30.2</v>
       </c>
       <c r="K187" t="n">
-        <v>116.6</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="188">
@@ -8855,12 +8855,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -8870,26 +8870,26 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F188" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G188" s="1" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H188" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I188" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>27.1</v>
+        <v>38.1</v>
       </c>
       <c r="K188" t="n">
-        <v>110.6</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="189">
@@ -8900,12 +8900,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -8915,26 +8915,26 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F189" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G189" s="1" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H189" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I189" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J189" t="n">
-        <v>25.8</v>
+        <v>38.6</v>
       </c>
       <c r="K189" t="n">
-        <v>105.3</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="190">
@@ -8945,12 +8945,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -8960,26 +8960,26 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F190" s="1" t="n">
-        <v>46273</v>
+        <v>46261</v>
       </c>
       <c r="G190" s="1" t="n">
-        <v>46280</v>
+        <v>46268</v>
       </c>
       <c r="H190" t="n">
         <v>7</v>
       </c>
       <c r="I190" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J190" t="n">
-        <v>24.8</v>
+        <v>32.1</v>
       </c>
       <c r="K190" t="n">
-        <v>101.2</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="191">
@@ -8990,12 +8990,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -9005,26 +9005,26 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F191" s="1" t="n">
-        <v>46273</v>
+        <v>46261</v>
       </c>
       <c r="G191" s="1" t="n">
-        <v>46280</v>
+        <v>46268</v>
       </c>
       <c r="H191" t="n">
         <v>7</v>
       </c>
       <c r="I191" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J191" t="n">
-        <v>24.6</v>
+        <v>32.7</v>
       </c>
       <c r="K191" t="n">
-        <v>100.4</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="192">
@@ -9035,12 +9035,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -9050,26 +9050,26 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F192" s="1" t="n">
-        <v>46274</v>
+        <v>46263</v>
       </c>
       <c r="G192" s="1" t="n">
-        <v>46281</v>
+        <v>46277</v>
       </c>
       <c r="H192" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I192" t="n">
         <v>35</v>
       </c>
       <c r="J192" t="n">
-        <v>35.9</v>
+        <v>49</v>
       </c>
       <c r="K192" t="n">
-        <v>102.6</v>
+        <v>140</v>
       </c>
     </row>
     <row r="193">
@@ -9080,40 +9080,850 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F193" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="G193" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H193" t="n">
+        <v>14</v>
+      </c>
+      <c r="I193" t="n">
+        <v>35</v>
+      </c>
+      <c r="J193" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="K193" t="n">
+        <v>141.7</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F194" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="G194" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="H194" t="n">
+        <v>7</v>
+      </c>
+      <c r="I194" t="n">
+        <v>35</v>
+      </c>
+      <c r="J194" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="K194" t="n">
+        <v>116.9</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F195" s="1" t="n">
+        <v>46263</v>
+      </c>
+      <c r="G195" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="H195" t="n">
+        <v>7</v>
+      </c>
+      <c r="I195" t="n">
+        <v>35</v>
+      </c>
+      <c r="J195" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="K195" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F196" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G196" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H196" t="n">
+        <v>14</v>
+      </c>
+      <c r="I196" t="n">
+        <v>35</v>
+      </c>
+      <c r="J196" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="K196" t="n">
+        <v>128.3</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F197" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G197" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H197" t="n">
+        <v>14</v>
+      </c>
+      <c r="I197" t="n">
+        <v>35</v>
+      </c>
+      <c r="J197" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="K197" t="n">
+        <v>124.3</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F198" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G198" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H198" t="n">
+        <v>7</v>
+      </c>
+      <c r="I198" t="n">
+        <v>35</v>
+      </c>
+      <c r="J198" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="K198" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>P36</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+        </is>
+      </c>
+      <c r="F199" s="1" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G199" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H199" t="n">
+        <v>7</v>
+      </c>
+      <c r="I199" t="n">
+        <v>35</v>
+      </c>
+      <c r="J199" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="K199" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F200" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G200" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H200" t="n">
+        <v>14</v>
+      </c>
+      <c r="I200" t="n">
+        <v>35</v>
+      </c>
+      <c r="J200" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="K200" t="n">
+        <v>134.9</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F201" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G201" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H201" t="n">
+        <v>14</v>
+      </c>
+      <c r="I201" t="n">
+        <v>35</v>
+      </c>
+      <c r="J201" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="K201" t="n">
+        <v>131.1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F202" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G202" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H202" t="n">
+        <v>7</v>
+      </c>
+      <c r="I202" t="n">
+        <v>35</v>
+      </c>
+      <c r="J202" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K202" t="n">
+        <v>111.1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F203" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G203" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H203" t="n">
+        <v>7</v>
+      </c>
+      <c r="I203" t="n">
+        <v>35</v>
+      </c>
+      <c r="J203" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="K203" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F204" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G204" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H204" t="n">
+        <v>7</v>
+      </c>
+      <c r="I204" t="n">
+        <v>35</v>
+      </c>
+      <c r="J204" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="K204" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F205" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G205" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H205" t="n">
+        <v>7</v>
+      </c>
+      <c r="I205" t="n">
+        <v>35</v>
+      </c>
+      <c r="J205" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K205" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F206" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G206" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H206" t="n">
+        <v>7</v>
+      </c>
+      <c r="I206" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J206" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K206" t="n">
+        <v>110.6</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F207" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G207" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H207" t="n">
+        <v>7</v>
+      </c>
+      <c r="I207" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J207" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K207" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F208" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G208" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H208" t="n">
+        <v>7</v>
+      </c>
+      <c r="I208" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J208" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K208" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F209" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G209" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H209" t="n">
+        <v>7</v>
+      </c>
+      <c r="I209" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J209" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="K209" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
           <t>P41</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No especificado </t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>Concreto</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
+      <c r="C210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
-      <c r="F193" s="1" t="n">
+      <c r="F210" s="1" t="n">
         <v>46274</v>
       </c>
-      <c r="G193" s="1" t="n">
+      <c r="G210" s="1" t="n">
         <v>46281</v>
       </c>
-      <c r="H193" t="n">
+      <c r="H210" t="n">
         <v>7</v>
       </c>
-      <c r="I193" t="n">
-        <v>35</v>
-      </c>
-      <c r="J193" t="n">
+      <c r="I210" t="n">
+        <v>35</v>
+      </c>
+      <c r="J210" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="K210" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F211" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G211" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H211" t="n">
+        <v>7</v>
+      </c>
+      <c r="I211" t="n">
+        <v>35</v>
+      </c>
+      <c r="J211" t="n">
         <v>36.7</v>
       </c>
-      <c r="K193" t="n">
+      <c r="K211" t="n">
         <v>104.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-09-22 16:21:26
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K211"/>
+  <dimension ref="A1:K220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7797,19 +7797,19 @@
         <v>46258</v>
       </c>
       <c r="G164" s="1" t="n">
-        <v>46272</v>
+        <v>46286</v>
       </c>
       <c r="H164" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I164" t="n">
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>31.9</v>
+        <v>38.6</v>
       </c>
       <c r="K164" t="n">
-        <v>91.09999999999999</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="165">
@@ -7842,19 +7842,19 @@
         <v>46258</v>
       </c>
       <c r="G165" s="1" t="n">
-        <v>46272</v>
+        <v>46286</v>
       </c>
       <c r="H165" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I165" t="n">
         <v>35</v>
       </c>
       <c r="J165" t="n">
-        <v>30.5</v>
+        <v>39.8</v>
       </c>
       <c r="K165" t="n">
-        <v>87.09999999999999</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="166">
@@ -7887,19 +7887,19 @@
         <v>46258</v>
       </c>
       <c r="G166" s="1" t="n">
-        <v>46265</v>
+        <v>46286</v>
       </c>
       <c r="H166" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I166" t="n">
         <v>35</v>
       </c>
       <c r="J166" t="n">
-        <v>26.9</v>
+        <v>37.9</v>
       </c>
       <c r="K166" t="n">
-        <v>76.90000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="167">
@@ -7932,19 +7932,19 @@
         <v>46258</v>
       </c>
       <c r="G167" s="1" t="n">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="H167" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I167" t="n">
         <v>35</v>
       </c>
       <c r="J167" t="n">
-        <v>26.5</v>
+        <v>31.9</v>
       </c>
       <c r="K167" t="n">
-        <v>75.7</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="168">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -7970,14 +7970,14 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F168" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G168" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="H168" t="n">
         <v>14</v>
@@ -7986,10 +7986,10 @@
         <v>35</v>
       </c>
       <c r="J168" t="n">
-        <v>37.9</v>
+        <v>30.5</v>
       </c>
       <c r="K168" t="n">
-        <v>108.3</v>
+        <v>87.09999999999999</v>
       </c>
     </row>
     <row r="169">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8015,26 +8015,26 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F169" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G169" s="1" t="n">
-        <v>46273</v>
+        <v>46265</v>
       </c>
       <c r="H169" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I169" t="n">
         <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>38</v>
+        <v>26.9</v>
       </c>
       <c r="K169" t="n">
-        <v>108.6</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="170">
@@ -8045,7 +8045,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>P20</t>
+          <t>P19</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8060,14 +8060,14 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 14 torre 1 tipo 1 , pilote 19 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F170" s="1" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="G170" s="1" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="H170" t="n">
         <v>7</v>
@@ -8076,10 +8076,10 @@
         <v>35</v>
       </c>
       <c r="J170" t="n">
-        <v>33.4</v>
+        <v>26.5</v>
       </c>
       <c r="K170" t="n">
-        <v>95.40000000000001</v>
+        <v>75.7</v>
       </c>
     </row>
     <row r="171">
@@ -8112,19 +8112,19 @@
         <v>46259</v>
       </c>
       <c r="G171" s="1" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="H171" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I171" t="n">
         <v>35</v>
       </c>
       <c r="J171" t="n">
-        <v>31.6</v>
+        <v>37.9</v>
       </c>
       <c r="K171" t="n">
-        <v>90.3</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="172">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F172" s="1" t="n">
@@ -8166,10 +8166,10 @@
         <v>35</v>
       </c>
       <c r="J172" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K172" t="n">
-        <v>94.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="173">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8195,26 +8195,26 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F173" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="G173" s="1" t="n">
-        <v>46273</v>
+        <v>46266</v>
       </c>
       <c r="H173" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I173" t="n">
         <v>35</v>
       </c>
       <c r="J173" t="n">
-        <v>32.6</v>
+        <v>33.4</v>
       </c>
       <c r="K173" t="n">
-        <v>93.09999999999999</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="174">
@@ -8225,7 +8225,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F174" s="1" t="n">
@@ -8256,10 +8256,10 @@
         <v>35</v>
       </c>
       <c r="J174" t="n">
-        <v>28.7</v>
+        <v>31.6</v>
       </c>
       <c r="K174" t="n">
-        <v>82</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="175">
@@ -8292,19 +8292,19 @@
         <v>46259</v>
       </c>
       <c r="G175" s="1" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="H175" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I175" t="n">
         <v>35</v>
       </c>
       <c r="J175" t="n">
-        <v>26.9</v>
+        <v>33</v>
       </c>
       <c r="K175" t="n">
-        <v>76.90000000000001</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="176">
@@ -8315,12 +8315,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -8330,14 +8330,14 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F176" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G176" s="1" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="H176" t="n">
         <v>14</v>
@@ -8346,10 +8346,10 @@
         <v>35</v>
       </c>
       <c r="J176" t="n">
-        <v>38.9</v>
+        <v>32.6</v>
       </c>
       <c r="K176" t="n">
-        <v>111.1</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="177">
@@ -8360,12 +8360,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -8375,26 +8375,26 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F177" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G177" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H177" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I177" t="n">
         <v>35</v>
       </c>
       <c r="J177" t="n">
-        <v>38</v>
+        <v>28.7</v>
       </c>
       <c r="K177" t="n">
-        <v>108.6</v>
+        <v>82</v>
       </c>
     </row>
     <row r="178">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -8420,14 +8420,14 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F178" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G178" s="1" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="H178" t="n">
         <v>7</v>
@@ -8436,10 +8436,10 @@
         <v>35</v>
       </c>
       <c r="J178" t="n">
-        <v>34.1</v>
+        <v>26.9</v>
       </c>
       <c r="K178" t="n">
-        <v>97.40000000000001</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="179">
@@ -8472,19 +8472,19 @@
         <v>46260</v>
       </c>
       <c r="G179" s="1" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="H179" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I179" t="n">
         <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>33</v>
+        <v>38.9</v>
       </c>
       <c r="K179" t="n">
-        <v>94.3</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="180">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8510,7 +8510,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F180" s="1" t="n">
@@ -8526,10 +8526,10 @@
         <v>35</v>
       </c>
       <c r="J180" t="n">
-        <v>43.4</v>
+        <v>38</v>
       </c>
       <c r="K180" t="n">
-        <v>124</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="181">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -8555,26 +8555,26 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F181" s="1" t="n">
         <v>46260</v>
       </c>
       <c r="G181" s="1" t="n">
-        <v>46274</v>
+        <v>46267</v>
       </c>
       <c r="H181" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I181" t="n">
         <v>35</v>
       </c>
       <c r="J181" t="n">
-        <v>43.9</v>
+        <v>34.1</v>
       </c>
       <c r="K181" t="n">
-        <v>125.4</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="182">
@@ -8585,7 +8585,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -8600,7 +8600,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F182" s="1" t="n">
@@ -8616,10 +8616,10 @@
         <v>35</v>
       </c>
       <c r="J182" t="n">
-        <v>37.8</v>
+        <v>33</v>
       </c>
       <c r="K182" t="n">
-        <v>108</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="183">
@@ -8652,19 +8652,19 @@
         <v>46260</v>
       </c>
       <c r="G183" s="1" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="H183" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I183" t="n">
         <v>35</v>
       </c>
       <c r="J183" t="n">
-        <v>36.5</v>
+        <v>43.4</v>
       </c>
       <c r="K183" t="n">
-        <v>104.3</v>
+        <v>124</v>
       </c>
     </row>
     <row r="184">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -8690,14 +8690,14 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F184" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G184" s="1" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="H184" t="n">
         <v>14</v>
@@ -8706,10 +8706,10 @@
         <v>35</v>
       </c>
       <c r="J184" t="n">
-        <v>36.3</v>
+        <v>43.9</v>
       </c>
       <c r="K184" t="n">
-        <v>103.7</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="185">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -8735,26 +8735,26 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F185" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G185" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H185" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I185" t="n">
         <v>35</v>
       </c>
       <c r="J185" t="n">
-        <v>36.6</v>
+        <v>37.8</v>
       </c>
       <c r="K185" t="n">
-        <v>104.6</v>
+        <v>108</v>
       </c>
     </row>
     <row r="186">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -8780,14 +8780,14 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F186" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G186" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="H186" t="n">
         <v>7</v>
@@ -8796,10 +8796,10 @@
         <v>35</v>
       </c>
       <c r="J186" t="n">
-        <v>31.6</v>
+        <v>36.5</v>
       </c>
       <c r="K186" t="n">
-        <v>90.3</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="187">
@@ -8832,19 +8832,19 @@
         <v>46261</v>
       </c>
       <c r="G187" s="1" t="n">
-        <v>46268</v>
+        <v>46275</v>
       </c>
       <c r="H187" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I187" t="n">
         <v>35</v>
       </c>
       <c r="J187" t="n">
-        <v>30.2</v>
+        <v>36.3</v>
       </c>
       <c r="K187" t="n">
-        <v>86.3</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="188">
@@ -8855,7 +8855,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -8870,7 +8870,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F188" s="1" t="n">
@@ -8886,10 +8886,10 @@
         <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>38.1</v>
+        <v>36.6</v>
       </c>
       <c r="K188" t="n">
-        <v>108.9</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="189">
@@ -8900,7 +8900,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8915,26 +8915,26 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F189" s="1" t="n">
         <v>46261</v>
       </c>
       <c r="G189" s="1" t="n">
-        <v>46275</v>
+        <v>46268</v>
       </c>
       <c r="H189" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I189" t="n">
         <v>35</v>
       </c>
       <c r="J189" t="n">
-        <v>38.6</v>
+        <v>31.6</v>
       </c>
       <c r="K189" t="n">
-        <v>110.3</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="190">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F190" s="1" t="n">
@@ -8976,10 +8976,10 @@
         <v>35</v>
       </c>
       <c r="J190" t="n">
-        <v>32.1</v>
+        <v>30.2</v>
       </c>
       <c r="K190" t="n">
-        <v>91.7</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="191">
@@ -9012,19 +9012,19 @@
         <v>46261</v>
       </c>
       <c r="G191" s="1" t="n">
-        <v>46268</v>
+        <v>46275</v>
       </c>
       <c r="H191" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I191" t="n">
         <v>35</v>
       </c>
       <c r="J191" t="n">
-        <v>32.7</v>
+        <v>38.1</v>
       </c>
       <c r="K191" t="n">
-        <v>93.40000000000001</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="192">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -9050,14 +9050,14 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F192" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G192" s="1" t="n">
-        <v>46277</v>
+        <v>46275</v>
       </c>
       <c r="H192" t="n">
         <v>14</v>
@@ -9066,10 +9066,10 @@
         <v>35</v>
       </c>
       <c r="J192" t="n">
-        <v>49</v>
+        <v>38.6</v>
       </c>
       <c r="K192" t="n">
-        <v>140</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="193">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -9095,26 +9095,26 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F193" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G193" s="1" t="n">
-        <v>46277</v>
+        <v>46268</v>
       </c>
       <c r="H193" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I193" t="n">
         <v>35</v>
       </c>
       <c r="J193" t="n">
-        <v>49.6</v>
+        <v>32.1</v>
       </c>
       <c r="K193" t="n">
-        <v>141.7</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="194">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -9140,14 +9140,14 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F194" s="1" t="n">
-        <v>46263</v>
+        <v>46261</v>
       </c>
       <c r="G194" s="1" t="n">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="H194" t="n">
         <v>7</v>
@@ -9156,10 +9156,10 @@
         <v>35</v>
       </c>
       <c r="J194" t="n">
-        <v>40.9</v>
+        <v>32.7</v>
       </c>
       <c r="K194" t="n">
-        <v>116.9</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="195">
@@ -9192,19 +9192,19 @@
         <v>46263</v>
       </c>
       <c r="G195" s="1" t="n">
-        <v>46270</v>
+        <v>46277</v>
       </c>
       <c r="H195" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I195" t="n">
         <v>35</v>
       </c>
       <c r="J195" t="n">
-        <v>41.3</v>
+        <v>49</v>
       </c>
       <c r="K195" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
     </row>
     <row r="196">
@@ -9215,12 +9215,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -9230,14 +9230,14 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F196" s="1" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="G196" s="1" t="n">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="H196" t="n">
         <v>14</v>
@@ -9246,10 +9246,10 @@
         <v>35</v>
       </c>
       <c r="J196" t="n">
-        <v>44.9</v>
+        <v>49.6</v>
       </c>
       <c r="K196" t="n">
-        <v>128.3</v>
+        <v>141.7</v>
       </c>
     </row>
     <row r="197">
@@ -9260,12 +9260,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -9275,26 +9275,26 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F197" s="1" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="G197" s="1" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
       <c r="H197" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I197" t="n">
         <v>35</v>
       </c>
       <c r="J197" t="n">
-        <v>43.5</v>
+        <v>40.9</v>
       </c>
       <c r="K197" t="n">
-        <v>124.3</v>
+        <v>116.9</v>
       </c>
     </row>
     <row r="198">
@@ -9305,12 +9305,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -9320,14 +9320,14 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F198" s="1" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="G198" s="1" t="n">
-        <v>46276</v>
+        <v>46270</v>
       </c>
       <c r="H198" t="n">
         <v>7</v>
@@ -9336,10 +9336,10 @@
         <v>35</v>
       </c>
       <c r="J198" t="n">
-        <v>36.6</v>
+        <v>41.3</v>
       </c>
       <c r="K198" t="n">
-        <v>104.6</v>
+        <v>118</v>
       </c>
     </row>
     <row r="199">
@@ -9372,19 +9372,19 @@
         <v>46269</v>
       </c>
       <c r="G199" s="1" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="H199" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I199" t="n">
         <v>35</v>
       </c>
       <c r="J199" t="n">
-        <v>37.1</v>
+        <v>44.9</v>
       </c>
       <c r="K199" t="n">
-        <v>106</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="200">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -9410,14 +9410,14 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F200" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="G200" s="1" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="H200" t="n">
         <v>14</v>
@@ -9426,10 +9426,10 @@
         <v>35</v>
       </c>
       <c r="J200" t="n">
-        <v>47.2</v>
+        <v>43.5</v>
       </c>
       <c r="K200" t="n">
-        <v>134.9</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="201">
@@ -9440,7 +9440,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -9455,26 +9455,26 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F201" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="G201" s="1" t="n">
-        <v>46284</v>
+        <v>46276</v>
       </c>
       <c r="H201" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I201" t="n">
         <v>35</v>
       </c>
       <c r="J201" t="n">
-        <v>45.9</v>
+        <v>36.6</v>
       </c>
       <c r="K201" t="n">
-        <v>131.1</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="202">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -9500,14 +9500,14 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F202" s="1" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="G202" s="1" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="H202" t="n">
         <v>7</v>
@@ -9516,10 +9516,10 @@
         <v>35</v>
       </c>
       <c r="J202" t="n">
-        <v>38.9</v>
+        <v>37.1</v>
       </c>
       <c r="K202" t="n">
-        <v>111.1</v>
+        <v>106</v>
       </c>
     </row>
     <row r="203">
@@ -9552,19 +9552,19 @@
         <v>46270</v>
       </c>
       <c r="G203" s="1" t="n">
-        <v>46277</v>
+        <v>46284</v>
       </c>
       <c r="H203" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I203" t="n">
         <v>35</v>
       </c>
       <c r="J203" t="n">
-        <v>37.9</v>
+        <v>47.2</v>
       </c>
       <c r="K203" t="n">
-        <v>108.3</v>
+        <v>134.9</v>
       </c>
     </row>
     <row r="204">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P37</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9590,26 +9590,26 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 33 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F204" s="1" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="G204" s="1" t="n">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="H204" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I204" t="n">
         <v>35</v>
       </c>
       <c r="J204" t="n">
-        <v>40.3</v>
+        <v>45.9</v>
       </c>
       <c r="K204" t="n">
-        <v>115.1</v>
+        <v>131.1</v>
       </c>
     </row>
     <row r="205">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P37</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -9635,14 +9635,14 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 33 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F205" s="1" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="G205" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H205" t="n">
         <v>7</v>
@@ -9651,10 +9651,10 @@
         <v>35</v>
       </c>
       <c r="J205" t="n">
-        <v>40.8</v>
+        <v>38.9</v>
       </c>
       <c r="K205" t="n">
-        <v>116.6</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="206">
@@ -9665,7 +9665,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P37</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -9680,26 +9680,26 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t>Pilote 33 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F206" s="1" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="G206" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H206" t="n">
         <v>7</v>
       </c>
       <c r="I206" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J206" t="n">
-        <v>27.1</v>
+        <v>37.9</v>
       </c>
       <c r="K206" t="n">
-        <v>110.6</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="207">
@@ -9710,7 +9710,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -9725,26 +9725,26 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F207" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="G207" s="1" t="n">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="H207" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I207" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J207" t="n">
-        <v>25.8</v>
+        <v>48.5</v>
       </c>
       <c r="K207" t="n">
-        <v>105.3</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="208">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -9770,26 +9770,26 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F208" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G208" s="1" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="H208" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I208" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J208" t="n">
-        <v>24.8</v>
+        <v>47.8</v>
       </c>
       <c r="K208" t="n">
-        <v>101.2</v>
+        <v>136.6</v>
       </c>
     </row>
     <row r="209">
@@ -9800,7 +9800,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -9815,26 +9815,26 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F209" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G209" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="H209" t="n">
         <v>7</v>
       </c>
       <c r="I209" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J209" t="n">
-        <v>24.6</v>
+        <v>40.3</v>
       </c>
       <c r="K209" t="n">
-        <v>100.4</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="210">
@@ -9845,7 +9845,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -9860,14 +9860,14 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F210" s="1" t="n">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="G210" s="1" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="H210" t="n">
         <v>7</v>
@@ -9876,10 +9876,10 @@
         <v>35</v>
       </c>
       <c r="J210" t="n">
-        <v>35.9</v>
+        <v>40.8</v>
       </c>
       <c r="K210" t="n">
-        <v>102.6</v>
+        <v>116.6</v>
       </c>
     </row>
     <row r="211">
@@ -9890,41 +9890,446 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F211" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G211" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H211" t="n">
+        <v>14</v>
+      </c>
+      <c r="I211" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J211" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="K211" t="n">
+        <v>131.8</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F212" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G212" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H212" t="n">
+        <v>14</v>
+      </c>
+      <c r="I212" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J212" t="n">
+        <v>32</v>
+      </c>
+      <c r="K212" t="n">
+        <v>130.6</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F213" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G213" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H213" t="n">
+        <v>7</v>
+      </c>
+      <c r="I213" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J213" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K213" t="n">
+        <v>110.6</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F214" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G214" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H214" t="n">
+        <v>7</v>
+      </c>
+      <c r="I214" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J214" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K214" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F215" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G215" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H215" t="n">
+        <v>7</v>
+      </c>
+      <c r="I215" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J215" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K215" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F216" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G216" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H216" t="n">
+        <v>7</v>
+      </c>
+      <c r="I216" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J216" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="K216" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
           <t>P41</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No especificado </t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>Concreto</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
+      <c r="C217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
-      <c r="F211" s="1" t="n">
+      <c r="F217" s="1" t="n">
         <v>46274</v>
       </c>
-      <c r="G211" s="1" t="n">
+      <c r="G217" s="1" t="n">
         <v>46281</v>
       </c>
-      <c r="H211" t="n">
+      <c r="H217" t="n">
         <v>7</v>
       </c>
-      <c r="I211" t="n">
-        <v>35</v>
-      </c>
-      <c r="J211" t="n">
+      <c r="I217" t="n">
+        <v>35</v>
+      </c>
+      <c r="J217" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="K217" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F218" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G218" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H218" t="n">
+        <v>7</v>
+      </c>
+      <c r="I218" t="n">
+        <v>35</v>
+      </c>
+      <c r="J218" t="n">
         <v>36.7</v>
       </c>
-      <c r="K211" t="n">
+      <c r="K218" t="n">
         <v>104.9</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>P42</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+        </is>
+      </c>
+      <c r="F219" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="G219" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H219" t="n">
+        <v>7</v>
+      </c>
+      <c r="I219" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J219" t="n">
+        <v>25</v>
+      </c>
+      <c r="K219" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>P42</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+        </is>
+      </c>
+      <c r="F220" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="G220" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H220" t="n">
+        <v>7</v>
+      </c>
+      <c r="I220" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J220" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="K220" t="n">
+        <v>103.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-09-24 21:04:19
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K220"/>
+  <dimension ref="A1:K246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8112,19 +8112,19 @@
         <v>46259</v>
       </c>
       <c r="G171" s="1" t="n">
-        <v>46273</v>
+        <v>46287</v>
       </c>
       <c r="H171" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I171" t="n">
         <v>35</v>
       </c>
       <c r="J171" t="n">
-        <v>37.9</v>
+        <v>46.1</v>
       </c>
       <c r="K171" t="n">
-        <v>108.3</v>
+        <v>131.7</v>
       </c>
     </row>
     <row r="172">
@@ -8157,19 +8157,19 @@
         <v>46259</v>
       </c>
       <c r="G172" s="1" t="n">
-        <v>46273</v>
+        <v>46287</v>
       </c>
       <c r="H172" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I172" t="n">
         <v>35</v>
       </c>
       <c r="J172" t="n">
-        <v>38</v>
+        <v>44.7</v>
       </c>
       <c r="K172" t="n">
-        <v>108.6</v>
+        <v>127.7</v>
       </c>
     </row>
     <row r="173">
@@ -8202,19 +8202,19 @@
         <v>46259</v>
       </c>
       <c r="G173" s="1" t="n">
-        <v>46266</v>
+        <v>46287</v>
       </c>
       <c r="H173" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I173" t="n">
         <v>35</v>
       </c>
       <c r="J173" t="n">
-        <v>33.4</v>
+        <v>45.5</v>
       </c>
       <c r="K173" t="n">
-        <v>95.40000000000001</v>
+        <v>130</v>
       </c>
     </row>
     <row r="174">
@@ -8247,19 +8247,19 @@
         <v>46259</v>
       </c>
       <c r="G174" s="1" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="H174" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I174" t="n">
         <v>35</v>
       </c>
       <c r="J174" t="n">
-        <v>31.6</v>
+        <v>37.9</v>
       </c>
       <c r="K174" t="n">
-        <v>90.3</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="175">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -8285,7 +8285,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F175" s="1" t="n">
@@ -8301,10 +8301,10 @@
         <v>35</v>
       </c>
       <c r="J175" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="K175" t="n">
-        <v>94.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="176">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8330,26 +8330,26 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F176" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="G176" s="1" t="n">
-        <v>46273</v>
+        <v>46266</v>
       </c>
       <c r="H176" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I176" t="n">
         <v>35</v>
       </c>
       <c r="J176" t="n">
-        <v>32.6</v>
+        <v>33.4</v>
       </c>
       <c r="K176" t="n">
-        <v>93.09999999999999</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="177">
@@ -8360,7 +8360,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>P21</t>
+          <t>P20</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8375,7 +8375,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 56 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F177" s="1" t="n">
@@ -8391,10 +8391,10 @@
         <v>35</v>
       </c>
       <c r="J177" t="n">
-        <v>28.7</v>
+        <v>31.6</v>
       </c>
       <c r="K177" t="n">
-        <v>82</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="178">
@@ -8427,19 +8427,19 @@
         <v>46259</v>
       </c>
       <c r="G178" s="1" t="n">
-        <v>46266</v>
+        <v>46287</v>
       </c>
       <c r="H178" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I178" t="n">
         <v>35</v>
       </c>
       <c r="J178" t="n">
-        <v>26.9</v>
+        <v>35.8</v>
       </c>
       <c r="K178" t="n">
-        <v>76.90000000000001</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="179">
@@ -8450,12 +8450,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -8465,26 +8465,26 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F179" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G179" s="1" t="n">
-        <v>46274</v>
+        <v>46287</v>
       </c>
       <c r="H179" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I179" t="n">
         <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>38.9</v>
+        <v>35.4</v>
       </c>
       <c r="K179" t="n">
-        <v>111.1</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="180">
@@ -8495,12 +8495,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -8510,26 +8510,26 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F180" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G180" s="1" t="n">
-        <v>46274</v>
+        <v>46287</v>
       </c>
       <c r="H180" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I180" t="n">
         <v>35</v>
       </c>
       <c r="J180" t="n">
-        <v>38</v>
+        <v>35.2</v>
       </c>
       <c r="K180" t="n">
-        <v>108.6</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="181">
@@ -8540,12 +8540,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -8555,26 +8555,26 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F181" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G181" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H181" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I181" t="n">
         <v>35</v>
       </c>
       <c r="J181" t="n">
-        <v>34.1</v>
+        <v>33</v>
       </c>
       <c r="K181" t="n">
-        <v>97.40000000000001</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="182">
@@ -8585,12 +8585,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>P22</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -8600,26 +8600,26 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F182" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G182" s="1" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="H182" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I182" t="n">
         <v>35</v>
       </c>
       <c r="J182" t="n">
-        <v>33</v>
+        <v>32.6</v>
       </c>
       <c r="K182" t="n">
-        <v>94.3</v>
+        <v>93.09999999999999</v>
       </c>
     </row>
     <row r="183">
@@ -8630,12 +8630,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -8645,26 +8645,26 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F183" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G183" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H183" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I183" t="n">
         <v>35</v>
       </c>
       <c r="J183" t="n">
-        <v>43.4</v>
+        <v>28.7</v>
       </c>
       <c r="K183" t="n">
-        <v>124</v>
+        <v>82</v>
       </c>
     </row>
     <row r="184">
@@ -8675,12 +8675,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P21</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -8690,26 +8690,26 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 2 torre 1 tipo 1 , pilote 57 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F184" s="1" t="n">
-        <v>46260</v>
+        <v>46259</v>
       </c>
       <c r="G184" s="1" t="n">
-        <v>46274</v>
+        <v>46266</v>
       </c>
       <c r="H184" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I184" t="n">
         <v>35</v>
       </c>
       <c r="J184" t="n">
-        <v>43.9</v>
+        <v>26.9</v>
       </c>
       <c r="K184" t="n">
-        <v>125.4</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="185">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -8735,26 +8735,26 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F185" s="1" t="n">
         <v>46260</v>
       </c>
       <c r="G185" s="1" t="n">
-        <v>46267</v>
+        <v>46288</v>
       </c>
       <c r="H185" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I185" t="n">
         <v>35</v>
       </c>
       <c r="J185" t="n">
-        <v>37.8</v>
+        <v>46.9</v>
       </c>
       <c r="K185" t="n">
-        <v>108</v>
+        <v>134</v>
       </c>
     </row>
     <row r="186">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>P23</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -8780,26 +8780,26 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Pilote 51 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F186" s="1" t="n">
         <v>46260</v>
       </c>
       <c r="G186" s="1" t="n">
-        <v>46267</v>
+        <v>46288</v>
       </c>
       <c r="H186" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I186" t="n">
         <v>35</v>
       </c>
       <c r="J186" t="n">
-        <v>36.5</v>
+        <v>45.4</v>
       </c>
       <c r="K186" t="n">
-        <v>104.3</v>
+        <v>129.7</v>
       </c>
     </row>
     <row r="187">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -8825,26 +8825,26 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F187" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G187" s="1" t="n">
-        <v>46275</v>
+        <v>46288</v>
       </c>
       <c r="H187" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I187" t="n">
         <v>35</v>
       </c>
       <c r="J187" t="n">
-        <v>36.3</v>
+        <v>46.3</v>
       </c>
       <c r="K187" t="n">
-        <v>103.7</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="188">
@@ -8855,7 +8855,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -8870,14 +8870,14 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F188" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G188" s="1" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="H188" t="n">
         <v>14</v>
@@ -8886,10 +8886,10 @@
         <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>36.6</v>
+        <v>38.9</v>
       </c>
       <c r="K188" t="n">
-        <v>104.6</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="189">
@@ -8900,7 +8900,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8915,26 +8915,26 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F189" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G189" s="1" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="H189" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I189" t="n">
         <v>35</v>
       </c>
       <c r="J189" t="n">
-        <v>31.6</v>
+        <v>38</v>
       </c>
       <c r="K189" t="n">
-        <v>90.3</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="190">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>P24</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -8960,14 +8960,14 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Pilote 6 torre 1 tipo 1</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F190" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G190" s="1" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="H190" t="n">
         <v>7</v>
@@ -8976,10 +8976,10 @@
         <v>35</v>
       </c>
       <c r="J190" t="n">
-        <v>30.2</v>
+        <v>34.1</v>
       </c>
       <c r="K190" t="n">
-        <v>86.3</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="191">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -9005,26 +9005,26 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 12 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F191" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G191" s="1" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="H191" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I191" t="n">
         <v>35</v>
       </c>
       <c r="J191" t="n">
-        <v>38.1</v>
+        <v>33</v>
       </c>
       <c r="K191" t="n">
-        <v>108.9</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="192">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -9050,26 +9050,26 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F192" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G192" s="1" t="n">
-        <v>46275</v>
+        <v>46288</v>
       </c>
       <c r="H192" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I192" t="n">
         <v>35</v>
       </c>
       <c r="J192" t="n">
-        <v>38.6</v>
+        <v>53.6</v>
       </c>
       <c r="K192" t="n">
-        <v>110.3</v>
+        <v>153.1</v>
       </c>
     </row>
     <row r="193">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -9095,26 +9095,26 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F193" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G193" s="1" t="n">
-        <v>46268</v>
+        <v>46288</v>
       </c>
       <c r="H193" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I193" t="n">
         <v>35</v>
       </c>
       <c r="J193" t="n">
-        <v>32.1</v>
+        <v>53.3</v>
       </c>
       <c r="K193" t="n">
-        <v>91.7</v>
+        <v>152.3</v>
       </c>
     </row>
     <row r="194">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>P25</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -9140,26 +9140,26 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F194" s="1" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="G194" s="1" t="n">
-        <v>46268</v>
+        <v>46288</v>
       </c>
       <c r="H194" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I194" t="n">
         <v>35</v>
       </c>
       <c r="J194" t="n">
-        <v>32.7</v>
+        <v>54.8</v>
       </c>
       <c r="K194" t="n">
-        <v>93.40000000000001</v>
+        <v>156.6</v>
       </c>
     </row>
     <row r="195">
@@ -9170,7 +9170,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -9185,14 +9185,14 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F195" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G195" s="1" t="n">
-        <v>46277</v>
+        <v>46274</v>
       </c>
       <c r="H195" t="n">
         <v>14</v>
@@ -9201,10 +9201,10 @@
         <v>35</v>
       </c>
       <c r="J195" t="n">
-        <v>49</v>
+        <v>43.4</v>
       </c>
       <c r="K195" t="n">
-        <v>140</v>
+        <v>124</v>
       </c>
     </row>
     <row r="196">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -9230,14 +9230,14 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F196" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G196" s="1" t="n">
-        <v>46277</v>
+        <v>46274</v>
       </c>
       <c r="H196" t="n">
         <v>14</v>
@@ -9246,10 +9246,10 @@
         <v>35</v>
       </c>
       <c r="J196" t="n">
-        <v>49.6</v>
+        <v>43.9</v>
       </c>
       <c r="K196" t="n">
-        <v>141.7</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="197">
@@ -9260,7 +9260,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -9275,14 +9275,14 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F197" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G197" s="1" t="n">
-        <v>46270</v>
+        <v>46267</v>
       </c>
       <c r="H197" t="n">
         <v>7</v>
@@ -9291,10 +9291,10 @@
         <v>35</v>
       </c>
       <c r="J197" t="n">
-        <v>40.9</v>
+        <v>37.8</v>
       </c>
       <c r="K197" t="n">
-        <v>116.9</v>
+        <v>108</v>
       </c>
     </row>
     <row r="198">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>P26</t>
+          <t>P23</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -9320,14 +9320,14 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
+          <t>Pilote 51 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F198" s="1" t="n">
-        <v>46263</v>
+        <v>46260</v>
       </c>
       <c r="G198" s="1" t="n">
-        <v>46270</v>
+        <v>46267</v>
       </c>
       <c r="H198" t="n">
         <v>7</v>
@@ -9336,10 +9336,10 @@
         <v>35</v>
       </c>
       <c r="J198" t="n">
-        <v>41.3</v>
+        <v>36.5</v>
       </c>
       <c r="K198" t="n">
-        <v>118</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="199">
@@ -9350,12 +9350,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -9365,26 +9365,26 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F199" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G199" s="1" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="H199" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I199" t="n">
         <v>35</v>
       </c>
       <c r="J199" t="n">
-        <v>44.9</v>
+        <v>44</v>
       </c>
       <c r="K199" t="n">
-        <v>128.3</v>
+        <v>125.7</v>
       </c>
     </row>
     <row r="200">
@@ -9395,12 +9395,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -9410,26 +9410,26 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F200" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G200" s="1" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="H200" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I200" t="n">
         <v>35</v>
       </c>
       <c r="J200" t="n">
-        <v>43.5</v>
+        <v>42.1</v>
       </c>
       <c r="K200" t="n">
-        <v>124.3</v>
+        <v>120.3</v>
       </c>
     </row>
     <row r="201">
@@ -9440,12 +9440,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -9455,26 +9455,26 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F201" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G201" s="1" t="n">
-        <v>46276</v>
+        <v>46289</v>
       </c>
       <c r="H201" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I201" t="n">
         <v>35</v>
       </c>
       <c r="J201" t="n">
-        <v>36.6</v>
+        <v>43.8</v>
       </c>
       <c r="K201" t="n">
-        <v>104.6</v>
+        <v>125.1</v>
       </c>
     </row>
     <row r="202">
@@ -9485,12 +9485,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>P36</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -9500,26 +9500,26 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F202" s="1" t="n">
-        <v>46269</v>
+        <v>46261</v>
       </c>
       <c r="G202" s="1" t="n">
-        <v>46276</v>
+        <v>46275</v>
       </c>
       <c r="H202" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I202" t="n">
         <v>35</v>
       </c>
       <c r="J202" t="n">
-        <v>37.1</v>
+        <v>36.3</v>
       </c>
       <c r="K202" t="n">
-        <v>106</v>
+        <v>103.7</v>
       </c>
     </row>
     <row r="203">
@@ -9530,12 +9530,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -9545,14 +9545,14 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F203" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G203" s="1" t="n">
-        <v>46284</v>
+        <v>46275</v>
       </c>
       <c r="H203" t="n">
         <v>14</v>
@@ -9561,10 +9561,10 @@
         <v>35</v>
       </c>
       <c r="J203" t="n">
-        <v>47.2</v>
+        <v>36.6</v>
       </c>
       <c r="K203" t="n">
-        <v>134.9</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="204">
@@ -9575,12 +9575,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -9590,26 +9590,26 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F204" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G204" s="1" t="n">
-        <v>46284</v>
+        <v>46268</v>
       </c>
       <c r="H204" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I204" t="n">
         <v>35</v>
       </c>
       <c r="J204" t="n">
-        <v>45.9</v>
+        <v>31.6</v>
       </c>
       <c r="K204" t="n">
-        <v>131.1</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="205">
@@ -9620,12 +9620,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P24</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -9635,14 +9635,14 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 6 torre 1 tipo 1</t>
         </is>
       </c>
       <c r="F205" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G205" s="1" t="n">
-        <v>46277</v>
+        <v>46268</v>
       </c>
       <c r="H205" t="n">
         <v>7</v>
@@ -9651,10 +9651,10 @@
         <v>35</v>
       </c>
       <c r="J205" t="n">
-        <v>38.9</v>
+        <v>30.2</v>
       </c>
       <c r="K205" t="n">
-        <v>111.1</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="206">
@@ -9665,12 +9665,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>P37</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -9680,26 +9680,26 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Pilote 33 torre 1 tipo 2</t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F206" s="1" t="n">
-        <v>46270</v>
+        <v>46261</v>
       </c>
       <c r="G206" s="1" t="n">
-        <v>46277</v>
+        <v>46289</v>
       </c>
       <c r="H206" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="I206" t="n">
         <v>35</v>
       </c>
       <c r="J206" t="n">
-        <v>37.9</v>
+        <v>46</v>
       </c>
       <c r="K206" t="n">
-        <v>108.3</v>
+        <v>131.4</v>
       </c>
     </row>
     <row r="207">
@@ -9710,12 +9710,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -9725,26 +9725,26 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F207" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G207" s="1" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="H207" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I207" t="n">
         <v>35</v>
       </c>
       <c r="J207" t="n">
-        <v>48.5</v>
+        <v>46.2</v>
       </c>
       <c r="K207" t="n">
-        <v>138.6</v>
+        <v>132</v>
       </c>
     </row>
     <row r="208">
@@ -9755,12 +9755,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -9770,26 +9770,26 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F208" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G208" s="1" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="H208" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I208" t="n">
         <v>35</v>
       </c>
       <c r="J208" t="n">
-        <v>47.8</v>
+        <v>47.3</v>
       </c>
       <c r="K208" t="n">
-        <v>136.6</v>
+        <v>135.1</v>
       </c>
     </row>
     <row r="209">
@@ -9800,12 +9800,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -9815,26 +9815,26 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F209" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G209" s="1" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H209" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I209" t="n">
         <v>35</v>
       </c>
       <c r="J209" t="n">
-        <v>40.3</v>
+        <v>38.1</v>
       </c>
       <c r="K209" t="n">
-        <v>115.1</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="210">
@@ -9845,12 +9845,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>P38</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -9860,26 +9860,26 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F210" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G210" s="1" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="H210" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I210" t="n">
         <v>35</v>
       </c>
       <c r="J210" t="n">
-        <v>40.8</v>
+        <v>38.6</v>
       </c>
       <c r="K210" t="n">
-        <v>116.6</v>
+        <v>110.3</v>
       </c>
     </row>
     <row r="211">
@@ -9890,12 +9890,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -9905,26 +9905,26 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F211" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G211" s="1" t="n">
-        <v>46286</v>
+        <v>46268</v>
       </c>
       <c r="H211" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I211" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J211" t="n">
-        <v>32.3</v>
+        <v>32.1</v>
       </c>
       <c r="K211" t="n">
-        <v>131.8</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="212">
@@ -9935,12 +9935,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P25</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -9950,26 +9950,26 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t>Pilote 8 torre 1 tipo 1 pilote 52 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F212" s="1" t="n">
-        <v>46272</v>
+        <v>46261</v>
       </c>
       <c r="G212" s="1" t="n">
-        <v>46286</v>
+        <v>46268</v>
       </c>
       <c r="H212" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I212" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J212" t="n">
-        <v>32</v>
+        <v>32.7</v>
       </c>
       <c r="K212" t="n">
-        <v>130.6</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="213">
@@ -9980,12 +9980,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -9995,26 +9995,26 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F213" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G213" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H213" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I213" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J213" t="n">
-        <v>27.1</v>
+        <v>49</v>
       </c>
       <c r="K213" t="n">
-        <v>110.6</v>
+        <v>140</v>
       </c>
     </row>
     <row r="214">
@@ -10025,12 +10025,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -10040,26 +10040,26 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F214" s="1" t="n">
-        <v>46272</v>
+        <v>46263</v>
       </c>
       <c r="G214" s="1" t="n">
-        <v>46279</v>
+        <v>46277</v>
       </c>
       <c r="H214" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I214" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J214" t="n">
-        <v>25.8</v>
+        <v>49.6</v>
       </c>
       <c r="K214" t="n">
-        <v>105.3</v>
+        <v>141.7</v>
       </c>
     </row>
     <row r="215">
@@ -10070,12 +10070,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -10085,26 +10085,26 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F215" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G215" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H215" t="n">
         <v>7</v>
       </c>
       <c r="I215" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J215" t="n">
-        <v>24.8</v>
+        <v>40.9</v>
       </c>
       <c r="K215" t="n">
-        <v>101.2</v>
+        <v>116.9</v>
       </c>
     </row>
     <row r="216">
@@ -10115,12 +10115,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P26</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -10130,26 +10130,26 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 1 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F216" s="1" t="n">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="G216" s="1" t="n">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="H216" t="n">
         <v>7</v>
       </c>
       <c r="I216" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J216" t="n">
-        <v>24.6</v>
+        <v>41.3</v>
       </c>
       <c r="K216" t="n">
-        <v>100.4</v>
+        <v>118</v>
       </c>
     </row>
     <row r="217">
@@ -10160,7 +10160,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -10175,26 +10175,26 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F217" s="1" t="n">
-        <v>46274</v>
+        <v>46269</v>
       </c>
       <c r="G217" s="1" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H217" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I217" t="n">
         <v>35</v>
       </c>
       <c r="J217" t="n">
-        <v>35.9</v>
+        <v>44.9</v>
       </c>
       <c r="K217" t="n">
-        <v>102.6</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="218">
@@ -10205,7 +10205,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -10220,26 +10220,26 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F218" s="1" t="n">
-        <v>46274</v>
+        <v>46269</v>
       </c>
       <c r="G218" s="1" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H218" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I218" t="n">
         <v>35</v>
       </c>
       <c r="J218" t="n">
-        <v>36.7</v>
+        <v>43.5</v>
       </c>
       <c r="K218" t="n">
-        <v>104.9</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="219">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -10265,26 +10265,26 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F219" s="1" t="n">
-        <v>46279</v>
+        <v>46269</v>
       </c>
       <c r="G219" s="1" t="n">
-        <v>46286</v>
+        <v>46276</v>
       </c>
       <c r="H219" t="n">
         <v>7</v>
       </c>
       <c r="I219" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="J219" t="n">
-        <v>25</v>
+        <v>36.6</v>
       </c>
       <c r="K219" t="n">
-        <v>102</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="220">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P36</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -10310,26 +10310,1196 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 40 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F220" s="1" t="n">
-        <v>46279</v>
+        <v>46269</v>
       </c>
       <c r="G220" s="1" t="n">
-        <v>46286</v>
+        <v>46276</v>
       </c>
       <c r="H220" t="n">
         <v>7</v>
       </c>
       <c r="I220" t="n">
+        <v>35</v>
+      </c>
+      <c r="J220" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="K220" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F221" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G221" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H221" t="n">
+        <v>14</v>
+      </c>
+      <c r="I221" t="n">
+        <v>35</v>
+      </c>
+      <c r="J221" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="K221" t="n">
+        <v>134.9</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F222" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G222" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H222" t="n">
+        <v>14</v>
+      </c>
+      <c r="I222" t="n">
+        <v>35</v>
+      </c>
+      <c r="J222" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="K222" t="n">
+        <v>131.1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F223" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G223" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H223" t="n">
+        <v>7</v>
+      </c>
+      <c r="I223" t="n">
+        <v>35</v>
+      </c>
+      <c r="J223" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K223" t="n">
+        <v>111.1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>P37</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Pilote 33 torre 1 tipo 2</t>
+        </is>
+      </c>
+      <c r="F224" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G224" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H224" t="n">
+        <v>7</v>
+      </c>
+      <c r="I224" t="n">
+        <v>35</v>
+      </c>
+      <c r="J224" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="K224" t="n">
+        <v>108.3</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F225" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G225" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H225" t="n">
+        <v>14</v>
+      </c>
+      <c r="I225" t="n">
+        <v>35</v>
+      </c>
+      <c r="J225" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K225" t="n">
+        <v>138.6</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F226" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G226" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H226" t="n">
+        <v>14</v>
+      </c>
+      <c r="I226" t="n">
+        <v>35</v>
+      </c>
+      <c r="J226" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="K226" t="n">
+        <v>136.6</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F227" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G227" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H227" t="n">
+        <v>7</v>
+      </c>
+      <c r="I227" t="n">
+        <v>35</v>
+      </c>
+      <c r="J227" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="K227" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F228" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G228" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H228" t="n">
+        <v>7</v>
+      </c>
+      <c r="I228" t="n">
+        <v>35</v>
+      </c>
+      <c r="J228" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K228" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F229" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G229" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H229" t="n">
+        <v>14</v>
+      </c>
+      <c r="I229" t="n">
         <v>24.5</v>
       </c>
-      <c r="J220" t="n">
+      <c r="J229" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="K229" t="n">
+        <v>131.8</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F230" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G230" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H230" t="n">
+        <v>14</v>
+      </c>
+      <c r="I230" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J230" t="n">
+        <v>32</v>
+      </c>
+      <c r="K230" t="n">
+        <v>130.6</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F231" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G231" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H231" t="n">
+        <v>7</v>
+      </c>
+      <c r="I231" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J231" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K231" t="n">
+        <v>110.6</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+        </is>
+      </c>
+      <c r="F232" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G232" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H232" t="n">
+        <v>7</v>
+      </c>
+      <c r="I232" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J232" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K232" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F233" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G233" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H233" t="n">
+        <v>14</v>
+      </c>
+      <c r="I233" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J233" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="K233" t="n">
+        <v>123.7</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F234" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G234" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H234" t="n">
+        <v>14</v>
+      </c>
+      <c r="I234" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J234" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="K234" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F235" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G235" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H235" t="n">
+        <v>7</v>
+      </c>
+      <c r="I235" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J235" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K235" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>P40</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+        </is>
+      </c>
+      <c r="F236" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G236" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H236" t="n">
+        <v>7</v>
+      </c>
+      <c r="I236" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J236" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="K236" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F237" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G237" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H237" t="n">
+        <v>14</v>
+      </c>
+      <c r="I237" t="n">
+        <v>35</v>
+      </c>
+      <c r="J237" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="K237" t="n">
+        <v>124.6</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F238" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G238" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H238" t="n">
+        <v>14</v>
+      </c>
+      <c r="I238" t="n">
+        <v>35</v>
+      </c>
+      <c r="J238" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="K238" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F239" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G239" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H239" t="n">
+        <v>7</v>
+      </c>
+      <c r="I239" t="n">
+        <v>35</v>
+      </c>
+      <c r="J239" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="K239" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>P41</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F240" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="G240" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H240" t="n">
+        <v>7</v>
+      </c>
+      <c r="I240" t="n">
+        <v>35</v>
+      </c>
+      <c r="J240" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K240" t="n">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>P42</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+        </is>
+      </c>
+      <c r="F241" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="G241" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H241" t="n">
+        <v>7</v>
+      </c>
+      <c r="I241" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J241" t="n">
+        <v>25</v>
+      </c>
+      <c r="K241" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>P42</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+        </is>
+      </c>
+      <c r="F242" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="G242" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H242" t="n">
+        <v>7</v>
+      </c>
+      <c r="I242" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J242" t="n">
         <v>25.3</v>
       </c>
-      <c r="K220" t="n">
+      <c r="K242" t="n">
         <v>103.3</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>P43</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+        </is>
+      </c>
+      <c r="F243" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="G243" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H243" t="n">
+        <v>7</v>
+      </c>
+      <c r="I243" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J243" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="K243" t="n">
+        <v>78.40000000000001</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>P43</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+        </is>
+      </c>
+      <c r="F244" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="G244" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H244" t="n">
+        <v>7</v>
+      </c>
+      <c r="I244" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J244" t="n">
+        <v>18</v>
+      </c>
+      <c r="K244" t="n">
+        <v>73.5</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>P44</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F245" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="G245" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H245" t="n">
+        <v>7</v>
+      </c>
+      <c r="I245" t="n">
+        <v>35</v>
+      </c>
+      <c r="J245" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="K245" t="n">
+        <v>113.7</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>P44</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F246" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="G246" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H246" t="n">
+        <v>7</v>
+      </c>
+      <c r="I246" t="n">
+        <v>35</v>
+      </c>
+      <c r="J246" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="K246" t="n">
+        <v>108.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-07 18:31:26
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L328"/>
+  <dimension ref="A1:L354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12944,22 +12944,22 @@
         <v>46272</v>
       </c>
       <c r="G261" s="1" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="H261" s="1" t="n">
-        <v>46287</v>
+        <v>46302</v>
       </c>
       <c r="I261" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J261" t="n">
         <v>35</v>
       </c>
       <c r="K261" t="n">
-        <v>48.5</v>
+        <v>56.5</v>
       </c>
       <c r="L261" t="n">
-        <v>138.6</v>
+        <v>161.4</v>
       </c>
     </row>
     <row r="262">
@@ -12992,22 +12992,22 @@
         <v>46272</v>
       </c>
       <c r="G262" s="1" t="n">
-        <v>46286</v>
+        <v>46300</v>
       </c>
       <c r="H262" s="1" t="n">
-        <v>46287</v>
+        <v>46302</v>
       </c>
       <c r="I262" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J262" t="n">
         <v>35</v>
       </c>
       <c r="K262" t="n">
-        <v>47.8</v>
+        <v>57.8</v>
       </c>
       <c r="L262" t="n">
-        <v>136.6</v>
+        <v>165.1</v>
       </c>
     </row>
     <row r="263">
@@ -13040,22 +13040,22 @@
         <v>46272</v>
       </c>
       <c r="G263" s="1" t="n">
-        <v>46279</v>
+        <v>46300</v>
       </c>
       <c r="H263" s="1" t="n">
-        <v>46280</v>
+        <v>46302</v>
       </c>
       <c r="I263" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J263" t="n">
         <v>35</v>
       </c>
       <c r="K263" t="n">
-        <v>40.3</v>
+        <v>57.2</v>
       </c>
       <c r="L263" t="n">
-        <v>115.1</v>
+        <v>163.4</v>
       </c>
     </row>
     <row r="264">
@@ -13088,22 +13088,22 @@
         <v>46272</v>
       </c>
       <c r="G264" s="1" t="n">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="H264" s="1" t="n">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="I264" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J264" t="n">
         <v>35</v>
       </c>
       <c r="K264" t="n">
-        <v>40.8</v>
+        <v>48.5</v>
       </c>
       <c r="L264" t="n">
-        <v>116.6</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="265">
@@ -13114,7 +13114,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F265" s="1" t="n">
@@ -13145,13 +13145,13 @@
         <v>14</v>
       </c>
       <c r="J265" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K265" t="n">
-        <v>32.3</v>
+        <v>47.8</v>
       </c>
       <c r="L265" t="n">
-        <v>131.8</v>
+        <v>136.6</v>
       </c>
     </row>
     <row r="266">
@@ -13162,7 +13162,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -13177,29 +13177,29 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F266" s="1" t="n">
         <v>46272</v>
       </c>
       <c r="G266" s="1" t="n">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="H266" s="1" t="n">
-        <v>46287</v>
+        <v>46280</v>
       </c>
       <c r="I266" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J266" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K266" t="n">
-        <v>32</v>
+        <v>40.3</v>
       </c>
       <c r="L266" t="n">
-        <v>130.6</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="267">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>P39</t>
+          <t>P38</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -13225,7 +13225,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
+          <t xml:space="preserve">Pilote 36 torre 1 tipo 2 , pilote 37 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F267" s="1" t="n">
@@ -13241,13 +13241,13 @@
         <v>7</v>
       </c>
       <c r="J267" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K267" t="n">
-        <v>27.1</v>
+        <v>40.8</v>
       </c>
       <c r="L267" t="n">
-        <v>110.6</v>
+        <v>116.6</v>
       </c>
     </row>
     <row r="268">
@@ -13280,22 +13280,22 @@
         <v>46272</v>
       </c>
       <c r="G268" s="1" t="n">
-        <v>46279</v>
+        <v>46300</v>
       </c>
       <c r="H268" s="1" t="n">
-        <v>46280</v>
+        <v>46302</v>
       </c>
       <c r="I268" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J268" t="n">
         <v>24.5</v>
       </c>
       <c r="K268" t="n">
-        <v>25.8</v>
+        <v>38.5</v>
       </c>
       <c r="L268" t="n">
-        <v>105.3</v>
+        <v>157.1</v>
       </c>
     </row>
     <row r="269">
@@ -13306,7 +13306,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -13321,29 +13321,29 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F269" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G269" s="1" t="n">
-        <v>46287</v>
+        <v>46300</v>
       </c>
       <c r="H269" s="1" t="n">
-        <v>46289</v>
+        <v>46302</v>
       </c>
       <c r="I269" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J269" t="n">
         <v>24.5</v>
       </c>
       <c r="K269" t="n">
-        <v>30.3</v>
+        <v>39.3</v>
       </c>
       <c r="L269" t="n">
-        <v>123.7</v>
+        <v>160.4</v>
       </c>
     </row>
     <row r="270">
@@ -13354,7 +13354,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -13369,29 +13369,29 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F270" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G270" s="1" t="n">
-        <v>46287</v>
+        <v>46300</v>
       </c>
       <c r="H270" s="1" t="n">
-        <v>46289</v>
+        <v>46302</v>
       </c>
       <c r="I270" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J270" t="n">
         <v>24.5</v>
       </c>
       <c r="K270" t="n">
-        <v>29.9</v>
+        <v>38.3</v>
       </c>
       <c r="L270" t="n">
-        <v>122</v>
+        <v>156.3</v>
       </c>
     </row>
     <row r="271">
@@ -13402,7 +13402,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -13417,29 +13417,29 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F271" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G271" s="1" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="H271" s="1" t="n">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="I271" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J271" t="n">
         <v>24.5</v>
       </c>
       <c r="K271" t="n">
-        <v>24.8</v>
+        <v>32.3</v>
       </c>
       <c r="L271" t="n">
-        <v>101.2</v>
+        <v>131.8</v>
       </c>
     </row>
     <row r="272">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>P40</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -13465,29 +13465,29 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F272" s="1" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G272" s="1" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="H272" s="1" t="n">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="I272" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J272" t="n">
         <v>24.5</v>
       </c>
       <c r="K272" t="n">
-        <v>24.6</v>
+        <v>32</v>
       </c>
       <c r="L272" t="n">
-        <v>100.4</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="273">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -13513,29 +13513,29 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F273" s="1" t="n">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="G273" s="1" t="n">
-        <v>46288</v>
+        <v>46279</v>
       </c>
       <c r="H273" s="1" t="n">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="I273" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J273" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K273" t="n">
-        <v>43.6</v>
+        <v>27.1</v>
       </c>
       <c r="L273" t="n">
-        <v>124.6</v>
+        <v>110.6</v>
       </c>
     </row>
     <row r="274">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P39</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -13561,29 +13561,29 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 133 salón comunal , pilote 121 salón comunal </t>
         </is>
       </c>
       <c r="F274" s="1" t="n">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="G274" s="1" t="n">
-        <v>46288</v>
+        <v>46279</v>
       </c>
       <c r="H274" s="1" t="n">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="I274" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J274" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K274" t="n">
-        <v>45.5</v>
+        <v>25.8</v>
       </c>
       <c r="L274" t="n">
-        <v>130</v>
+        <v>105.3</v>
       </c>
     </row>
     <row r="275">
@@ -13594,7 +13594,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -13609,29 +13609,29 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F275" s="1" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="G275" s="1" t="n">
-        <v>46281</v>
+        <v>46301</v>
       </c>
       <c r="H275" s="1" t="n">
-        <v>46283</v>
+        <v>46302</v>
       </c>
       <c r="I275" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J275" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K275" t="n">
-        <v>35.9</v>
+        <v>36.1</v>
       </c>
       <c r="L275" t="n">
-        <v>102.6</v>
+        <v>147.3</v>
       </c>
     </row>
     <row r="276">
@@ -13642,7 +13642,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>P41</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -13657,29 +13657,29 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F276" s="1" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="G276" s="1" t="n">
-        <v>46281</v>
+        <v>46301</v>
       </c>
       <c r="H276" s="1" t="n">
-        <v>46283</v>
+        <v>46302</v>
       </c>
       <c r="I276" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J276" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K276" t="n">
-        <v>36.7</v>
+        <v>35.6</v>
       </c>
       <c r="L276" t="n">
-        <v>104.9</v>
+        <v>145.3</v>
       </c>
     </row>
     <row r="277">
@@ -13690,7 +13690,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -13705,29 +13705,29 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F277" s="1" t="n">
-        <v>46279</v>
+        <v>46273</v>
       </c>
       <c r="G277" s="1" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="H277" s="1" t="n">
-        <v>46294</v>
+        <v>46302</v>
       </c>
       <c r="I277" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J277" t="n">
         <v>24.5</v>
       </c>
       <c r="K277" t="n">
-        <v>30.6</v>
+        <v>37.1</v>
       </c>
       <c r="L277" t="n">
-        <v>124.9</v>
+        <v>151.4</v>
       </c>
     </row>
     <row r="278">
@@ -13738,7 +13738,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -13753,17 +13753,17 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F278" s="1" t="n">
-        <v>46279</v>
+        <v>46273</v>
       </c>
       <c r="G278" s="1" t="n">
-        <v>46293</v>
+        <v>46287</v>
       </c>
       <c r="H278" s="1" t="n">
-        <v>46294</v>
+        <v>46289</v>
       </c>
       <c r="I278" t="n">
         <v>14</v>
@@ -13772,10 +13772,10 @@
         <v>24.5</v>
       </c>
       <c r="K278" t="n">
-        <v>29.7</v>
+        <v>30.3</v>
       </c>
       <c r="L278" t="n">
-        <v>121.2</v>
+        <v>123.7</v>
       </c>
     </row>
     <row r="279">
@@ -13786,7 +13786,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -13801,29 +13801,29 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F279" s="1" t="n">
-        <v>46279</v>
+        <v>46273</v>
       </c>
       <c r="G279" s="1" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H279" s="1" t="n">
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="I279" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J279" t="n">
         <v>24.5</v>
       </c>
       <c r="K279" t="n">
-        <v>25</v>
+        <v>29.9</v>
       </c>
       <c r="L279" t="n">
-        <v>102</v>
+        <v>122</v>
       </c>
     </row>
     <row r="280">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>P42</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -13849,17 +13849,17 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F280" s="1" t="n">
-        <v>46279</v>
+        <v>46273</v>
       </c>
       <c r="G280" s="1" t="n">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="H280" s="1" t="n">
-        <v>46287</v>
+        <v>46280</v>
       </c>
       <c r="I280" t="n">
         <v>7</v>
@@ -13868,10 +13868,10 @@
         <v>24.5</v>
       </c>
       <c r="K280" t="n">
-        <v>25.3</v>
+        <v>24.8</v>
       </c>
       <c r="L280" t="n">
-        <v>103.3</v>
+        <v>101.2</v>
       </c>
     </row>
     <row r="281">
@@ -13882,7 +13882,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>P43</t>
+          <t>P40</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -13897,29 +13897,29 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+          <t xml:space="preserve">Pilote 143 salón comunal , Pilote 125 salón comunal , Pilote 115 salón comunal , Pilote 136 salón comunal </t>
         </is>
       </c>
       <c r="F281" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G281" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="G281" s="1" t="n">
-        <v>46294</v>
-      </c>
       <c r="H281" s="1" t="n">
-        <v>46301</v>
+        <v>46280</v>
       </c>
       <c r="I281" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J281" t="n">
         <v>24.5</v>
       </c>
       <c r="K281" t="n">
-        <v>21.4</v>
+        <v>24.6</v>
       </c>
       <c r="L281" t="n">
-        <v>87.3</v>
+        <v>100.4</v>
       </c>
     </row>
     <row r="282">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>P43</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -13945,29 +13945,29 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F282" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G282" s="1" t="n">
-        <v>46294</v>
+        <v>46302</v>
       </c>
       <c r="H282" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I282" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J282" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K282" t="n">
-        <v>21.6</v>
+        <v>52.1</v>
       </c>
       <c r="L282" t="n">
-        <v>88.2</v>
+        <v>148.9</v>
       </c>
     </row>
     <row r="283">
@@ -13978,7 +13978,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>P43</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -13993,29 +13993,29 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F283" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G283" s="1" t="n">
-        <v>46287</v>
+        <v>46302</v>
       </c>
       <c r="H283" s="1" t="n">
-        <v>46289</v>
+        <v>46302</v>
       </c>
       <c r="I283" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J283" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K283" t="n">
-        <v>19.2</v>
+        <v>53.1</v>
       </c>
       <c r="L283" t="n">
-        <v>78.40000000000001</v>
+        <v>151.7</v>
       </c>
     </row>
     <row r="284">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>P43</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -14041,29 +14041,29 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F284" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G284" s="1" t="n">
-        <v>46287</v>
+        <v>46302</v>
       </c>
       <c r="H284" s="1" t="n">
-        <v>46289</v>
+        <v>46302</v>
       </c>
       <c r="I284" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J284" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K284" t="n">
-        <v>18</v>
+        <v>52.7</v>
       </c>
       <c r="L284" t="n">
-        <v>73.5</v>
+        <v>150.6</v>
       </c>
     </row>
     <row r="285">
@@ -14074,7 +14074,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>P44</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -14089,17 +14089,17 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F285" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G285" s="1" t="n">
-        <v>46294</v>
+        <v>46288</v>
       </c>
       <c r="H285" s="1" t="n">
-        <v>46301</v>
+        <v>46289</v>
       </c>
       <c r="I285" t="n">
         <v>14</v>
@@ -14108,10 +14108,10 @@
         <v>35</v>
       </c>
       <c r="K285" t="n">
-        <v>45.5</v>
+        <v>43.6</v>
       </c>
       <c r="L285" t="n">
-        <v>130</v>
+        <v>124.6</v>
       </c>
     </row>
     <row r="286">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>P44</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -14137,17 +14137,17 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F286" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G286" s="1" t="n">
-        <v>46294</v>
+        <v>46288</v>
       </c>
       <c r="H286" s="1" t="n">
-        <v>46301</v>
+        <v>46289</v>
       </c>
       <c r="I286" t="n">
         <v>14</v>
@@ -14156,10 +14156,10 @@
         <v>35</v>
       </c>
       <c r="K286" t="n">
-        <v>46.3</v>
+        <v>45.5</v>
       </c>
       <c r="L286" t="n">
-        <v>132.3</v>
+        <v>130</v>
       </c>
     </row>
     <row r="287">
@@ -14170,7 +14170,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>P44</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -14185,17 +14185,17 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F287" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G287" s="1" t="n">
-        <v>46287</v>
+        <v>46281</v>
       </c>
       <c r="H287" s="1" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
       <c r="I287" t="n">
         <v>7</v>
@@ -14204,10 +14204,10 @@
         <v>35</v>
       </c>
       <c r="K287" t="n">
-        <v>39.8</v>
+        <v>35.9</v>
       </c>
       <c r="L287" t="n">
-        <v>113.7</v>
+        <v>102.6</v>
       </c>
     </row>
     <row r="288">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>P44</t>
+          <t>P41</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -14233,17 +14233,17 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
+          <t xml:space="preserve">Pilote 39 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F288" s="1" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="G288" s="1" t="n">
-        <v>46287</v>
+        <v>46281</v>
       </c>
       <c r="H288" s="1" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
       <c r="I288" t="n">
         <v>7</v>
@@ -14252,10 +14252,10 @@
         <v>35</v>
       </c>
       <c r="K288" t="n">
-        <v>38.1</v>
+        <v>36.7</v>
       </c>
       <c r="L288" t="n">
-        <v>108.9</v>
+        <v>104.9</v>
       </c>
     </row>
     <row r="289">
@@ -14266,7 +14266,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>P45</t>
+          <t>P42</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -14281,17 +14281,17 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
         </is>
       </c>
       <c r="F289" s="1" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="G289" s="1" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="H289" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I289" t="n">
         <v>14</v>
@@ -14300,10 +14300,10 @@
         <v>24.5</v>
       </c>
       <c r="K289" t="n">
-        <v>33.5</v>
+        <v>30.6</v>
       </c>
       <c r="L289" t="n">
-        <v>136.7</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="290">
@@ -14314,7 +14314,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>P45</t>
+          <t>P42</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -14329,17 +14329,17 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
         </is>
       </c>
       <c r="F290" s="1" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="G290" s="1" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="H290" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I290" t="n">
         <v>14</v>
@@ -14348,10 +14348,10 @@
         <v>24.5</v>
       </c>
       <c r="K290" t="n">
-        <v>32</v>
+        <v>29.7</v>
       </c>
       <c r="L290" t="n">
-        <v>130.6</v>
+        <v>121.2</v>
       </c>
     </row>
     <row r="291">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>P45</t>
+          <t>P42</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -14377,29 +14377,29 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
         </is>
       </c>
       <c r="F291" s="1" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="G291" s="1" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="H291" s="1" t="n">
-        <v>46294</v>
+        <v>46287</v>
       </c>
       <c r="I291" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J291" t="n">
         <v>24.5</v>
       </c>
       <c r="K291" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L291" t="n">
-        <v>110.2</v>
+        <v>102</v>
       </c>
     </row>
     <row r="292">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>P45</t>
+          <t>P42</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -14425,29 +14425,29 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
+          <t xml:space="preserve">Pilote 131 - 130 - 129 salón comunal </t>
         </is>
       </c>
       <c r="F292" s="1" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="G292" s="1" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="H292" s="1" t="n">
-        <v>46294</v>
+        <v>46287</v>
       </c>
       <c r="I292" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J292" t="n">
         <v>24.5</v>
       </c>
       <c r="K292" t="n">
-        <v>27.4</v>
+        <v>25.3</v>
       </c>
       <c r="L292" t="n">
-        <v>111.8</v>
+        <v>103.3</v>
       </c>
     </row>
     <row r="293">
@@ -14458,7 +14458,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>P46</t>
+          <t>P43</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -14473,14 +14473,14 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
         </is>
       </c>
       <c r="F293" s="1" t="n">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="G293" s="1" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="H293" s="1" t="n">
         <v>46301</v>
@@ -14492,10 +14492,10 @@
         <v>24.5</v>
       </c>
       <c r="K293" t="n">
-        <v>27.1</v>
+        <v>21.4</v>
       </c>
       <c r="L293" t="n">
-        <v>110.6</v>
+        <v>87.3</v>
       </c>
     </row>
     <row r="294">
@@ -14506,7 +14506,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>P46</t>
+          <t>P43</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -14521,14 +14521,14 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
         </is>
       </c>
       <c r="F294" s="1" t="n">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="G294" s="1" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="H294" s="1" t="n">
         <v>46301</v>
@@ -14540,10 +14540,10 @@
         <v>24.5</v>
       </c>
       <c r="K294" t="n">
-        <v>27.5</v>
+        <v>21.6</v>
       </c>
       <c r="L294" t="n">
-        <v>112.2</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="295">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>P46</t>
+          <t>P43</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -14569,17 +14569,17 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
         </is>
       </c>
       <c r="F295" s="1" t="n">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="G295" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H295" s="1" t="n">
         <v>46289</v>
-      </c>
-      <c r="H295" s="1" t="n">
-        <v>46294</v>
       </c>
       <c r="I295" t="n">
         <v>7</v>
@@ -14588,10 +14588,10 @@
         <v>24.5</v>
       </c>
       <c r="K295" t="n">
-        <v>21.8</v>
+        <v>19.2</v>
       </c>
       <c r="L295" t="n">
-        <v>89</v>
+        <v>78.40000000000001</v>
       </c>
     </row>
     <row r="296">
@@ -14602,7 +14602,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>P46</t>
+          <t>P43</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -14617,17 +14617,17 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
+          <t xml:space="preserve">Pilote 128 - 118 - 140 salón comunal </t>
         </is>
       </c>
       <c r="F296" s="1" t="n">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="G296" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H296" s="1" t="n">
         <v>46289</v>
-      </c>
-      <c r="H296" s="1" t="n">
-        <v>46294</v>
       </c>
       <c r="I296" t="n">
         <v>7</v>
@@ -14636,10 +14636,10 @@
         <v>24.5</v>
       </c>
       <c r="K296" t="n">
-        <v>21.7</v>
+        <v>18</v>
       </c>
       <c r="L296" t="n">
-        <v>88.59999999999999</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="297">
@@ -14650,7 +14650,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>P47</t>
+          <t>P44</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -14665,14 +14665,14 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Pilote 41 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F297" s="1" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="G297" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="H297" s="1" t="n">
         <v>46301</v>
@@ -14684,10 +14684,10 @@
         <v>35</v>
       </c>
       <c r="K297" t="n">
-        <v>36.6</v>
+        <v>45.5</v>
       </c>
       <c r="L297" t="n">
-        <v>104.6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="298">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>P47</t>
+          <t>P44</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -14713,14 +14713,14 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Pilote 41 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F298" s="1" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="G298" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="H298" s="1" t="n">
         <v>46301</v>
@@ -14732,10 +14732,10 @@
         <v>35</v>
       </c>
       <c r="K298" t="n">
-        <v>36.9</v>
+        <v>46.3</v>
       </c>
       <c r="L298" t="n">
-        <v>105.4</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="299">
@@ -14746,7 +14746,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>P47</t>
+          <t>P44</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -14761,17 +14761,17 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Pilote 41 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F299" s="1" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="G299" s="1" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="H299" s="1" t="n">
-        <v>46294</v>
+        <v>46289</v>
       </c>
       <c r="I299" t="n">
         <v>7</v>
@@ -14780,10 +14780,10 @@
         <v>35</v>
       </c>
       <c r="K299" t="n">
-        <v>31.7</v>
+        <v>39.8</v>
       </c>
       <c r="L299" t="n">
-        <v>90.59999999999999</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="300">
@@ -14794,7 +14794,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>P47</t>
+          <t>P44</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -14809,17 +14809,17 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Pilote 41 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 32 torre 1 tipo 2 </t>
         </is>
       </c>
       <c r="F300" s="1" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="G300" s="1" t="n">
-        <v>46290</v>
+        <v>46287</v>
       </c>
       <c r="H300" s="1" t="n">
-        <v>46294</v>
+        <v>46289</v>
       </c>
       <c r="I300" t="n">
         <v>7</v>
@@ -14828,10 +14828,10 @@
         <v>35</v>
       </c>
       <c r="K300" t="n">
-        <v>30.3</v>
+        <v>38.1</v>
       </c>
       <c r="L300" t="n">
-        <v>86.59999999999999</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="301">
@@ -14842,7 +14842,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>P48</t>
+          <t>P45</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -14857,14 +14857,14 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
+          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
         </is>
       </c>
       <c r="F301" s="1" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="G301" s="1" t="n">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="H301" s="1" t="n">
         <v>46301</v>
@@ -14876,10 +14876,10 @@
         <v>24.5</v>
       </c>
       <c r="K301" t="n">
-        <v>27.1</v>
+        <v>33.5</v>
       </c>
       <c r="L301" t="n">
-        <v>110.6</v>
+        <v>136.7</v>
       </c>
     </row>
     <row r="302">
@@ -14890,7 +14890,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>P48</t>
+          <t>P45</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -14905,14 +14905,14 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
+          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
         </is>
       </c>
       <c r="F302" s="1" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="G302" s="1" t="n">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="H302" s="1" t="n">
         <v>46301</v>
@@ -14924,10 +14924,10 @@
         <v>24.5</v>
       </c>
       <c r="K302" t="n">
-        <v>26.3</v>
+        <v>32</v>
       </c>
       <c r="L302" t="n">
-        <v>107.3</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="303">
@@ -14938,7 +14938,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>P48</t>
+          <t>P45</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -14953,29 +14953,29 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
+          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
         </is>
       </c>
       <c r="F303" s="1" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="G303" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="H303" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="I303" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J303" t="n">
         <v>24.5</v>
       </c>
       <c r="K303" t="n">
-        <v>23.5</v>
+        <v>27</v>
       </c>
       <c r="L303" t="n">
-        <v>95.90000000000001</v>
+        <v>110.2</v>
       </c>
     </row>
     <row r="304">
@@ -14986,7 +14986,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>P48</t>
+          <t>P45</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -15001,29 +15001,29 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
+          <t xml:space="preserve">Pilote 142 - 108 - 109 salón comunal </t>
         </is>
       </c>
       <c r="F304" s="1" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="G304" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="H304" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="I304" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J304" t="n">
         <v>24.5</v>
       </c>
       <c r="K304" t="n">
-        <v>22.7</v>
+        <v>27.4</v>
       </c>
       <c r="L304" t="n">
-        <v>92.7</v>
+        <v>111.8</v>
       </c>
     </row>
     <row r="305">
@@ -15034,7 +15034,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>P49</t>
+          <t>P46</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -15049,14 +15049,14 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
+          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
         </is>
       </c>
       <c r="F305" s="1" t="n">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="G305" s="1" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="H305" s="1" t="n">
         <v>46301</v>
@@ -15068,10 +15068,10 @@
         <v>24.5</v>
       </c>
       <c r="K305" t="n">
-        <v>32</v>
+        <v>27.1</v>
       </c>
       <c r="L305" t="n">
-        <v>130.6</v>
+        <v>110.6</v>
       </c>
     </row>
     <row r="306">
@@ -15082,7 +15082,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>P49</t>
+          <t>P46</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -15097,14 +15097,14 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
+          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
         </is>
       </c>
       <c r="F306" s="1" t="n">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="G306" s="1" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="H306" s="1" t="n">
         <v>46301</v>
@@ -15116,10 +15116,10 @@
         <v>24.5</v>
       </c>
       <c r="K306" t="n">
-        <v>33.3</v>
+        <v>27.5</v>
       </c>
       <c r="L306" t="n">
-        <v>135.9</v>
+        <v>112.2</v>
       </c>
     </row>
     <row r="307">
@@ -15130,7 +15130,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>P49</t>
+          <t>P46</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -15145,14 +15145,14 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
+          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
         </is>
       </c>
       <c r="F307" s="1" t="n">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="G307" s="1" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="H307" s="1" t="n">
         <v>46294</v>
@@ -15164,10 +15164,10 @@
         <v>24.5</v>
       </c>
       <c r="K307" t="n">
-        <v>26.5</v>
+        <v>21.8</v>
       </c>
       <c r="L307" t="n">
-        <v>108.2</v>
+        <v>89</v>
       </c>
     </row>
     <row r="308">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>P49</t>
+          <t>P46</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -15193,14 +15193,14 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
+          <t xml:space="preserve">Pilote 144 - 134 - 138 - 132 salón comunal </t>
         </is>
       </c>
       <c r="F308" s="1" t="n">
-        <v>46284</v>
+        <v>46282</v>
       </c>
       <c r="G308" s="1" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="H308" s="1" t="n">
         <v>46294</v>
@@ -15212,10 +15212,10 @@
         <v>24.5</v>
       </c>
       <c r="K308" t="n">
-        <v>26.9</v>
+        <v>21.7</v>
       </c>
       <c r="L308" t="n">
-        <v>109.8</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="309">
@@ -15226,7 +15226,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P47</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -15241,29 +15241,29 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
+          <t>Pilote 41 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F309" s="1" t="n">
-        <v>46286</v>
+        <v>46283</v>
       </c>
       <c r="G309" s="1" t="n">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="H309" s="1" t="n">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="I309" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J309" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K309" t="n">
-        <v>23.9</v>
+        <v>36.6</v>
       </c>
       <c r="L309" t="n">
-        <v>97.59999999999999</v>
+        <v>104.6</v>
       </c>
     </row>
     <row r="310">
@@ -15274,7 +15274,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P47</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -15289,29 +15289,29 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
+          <t>Pilote 41 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F310" s="1" t="n">
-        <v>46286</v>
+        <v>46283</v>
       </c>
       <c r="G310" s="1" t="n">
-        <v>46293</v>
+        <v>46297</v>
       </c>
       <c r="H310" s="1" t="n">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="I310" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J310" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K310" t="n">
-        <v>24.1</v>
+        <v>36.9</v>
       </c>
       <c r="L310" t="n">
-        <v>98.40000000000001</v>
+        <v>105.4</v>
       </c>
     </row>
     <row r="311">
@@ -15322,7 +15322,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P47</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -15337,29 +15337,29 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t>Pilote 41 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F311" s="1" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="G311" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H311" s="1" t="n">
         <v>46294</v>
-      </c>
-      <c r="H311" s="1" t="n">
-        <v>46301</v>
       </c>
       <c r="I311" t="n">
         <v>7</v>
       </c>
       <c r="J311" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K311" t="n">
-        <v>22.6</v>
+        <v>31.7</v>
       </c>
       <c r="L311" t="n">
-        <v>92.2</v>
+        <v>90.59999999999999</v>
       </c>
     </row>
     <row r="312">
@@ -15370,7 +15370,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P47</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -15385,29 +15385,29 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t>Pilote 41 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F312" s="1" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="G312" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H312" s="1" t="n">
         <v>46294</v>
-      </c>
-      <c r="H312" s="1" t="n">
-        <v>46301</v>
       </c>
       <c r="I312" t="n">
         <v>7</v>
       </c>
       <c r="J312" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K312" t="n">
-        <v>23.4</v>
+        <v>30.3</v>
       </c>
       <c r="L312" t="n">
-        <v>95.5</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="313">
@@ -15418,12 +15418,12 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P48</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -15433,29 +15433,29 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
         </is>
       </c>
       <c r="F313" s="1" t="n">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="G313" s="1" t="n">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="H313" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="I313" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J313" t="n">
         <v>24.5</v>
       </c>
       <c r="K313" t="n">
-        <v>21.4</v>
+        <v>27.1</v>
       </c>
       <c r="L313" t="n">
-        <v>87.3</v>
+        <v>110.6</v>
       </c>
     </row>
     <row r="314">
@@ -15466,12 +15466,12 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P48</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -15481,29 +15481,29 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
         </is>
       </c>
       <c r="F314" s="1" t="n">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="G314" s="1" t="n">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="H314" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="I314" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J314" t="n">
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>21.6</v>
+        <v>26.3</v>
       </c>
       <c r="L314" t="n">
-        <v>88.2</v>
+        <v>107.3</v>
       </c>
     </row>
     <row r="315">
@@ -15514,12 +15514,12 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P48</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -15529,29 +15529,29 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
         </is>
       </c>
       <c r="F315" s="1" t="n">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="G315" s="1" t="n">
-        <v>46295</v>
+        <v>46290</v>
       </c>
       <c r="H315" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I315" t="n">
         <v>7</v>
       </c>
       <c r="J315" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K315" t="n">
-        <v>34.8</v>
+        <v>23.5</v>
       </c>
       <c r="L315" t="n">
-        <v>99.40000000000001</v>
+        <v>95.90000000000001</v>
       </c>
     </row>
     <row r="316">
@@ -15562,12 +15562,12 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P48</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -15577,29 +15577,29 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 119 - 114 - 116 salón comunal </t>
         </is>
       </c>
       <c r="F316" s="1" t="n">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="G316" s="1" t="n">
-        <v>46295</v>
+        <v>46290</v>
       </c>
       <c r="H316" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I316" t="n">
         <v>7</v>
       </c>
       <c r="J316" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K316" t="n">
-        <v>33.8</v>
+        <v>22.7</v>
       </c>
       <c r="L316" t="n">
-        <v>96.59999999999999</v>
+        <v>92.7</v>
       </c>
     </row>
     <row r="317">
@@ -15610,12 +15610,12 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -15625,29 +15625,29 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F317" s="1" t="n">
-        <v>46289</v>
+        <v>46284</v>
       </c>
       <c r="G317" s="1" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="H317" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="I317" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J317" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K317" t="n">
-        <v>35.7</v>
+        <v>32</v>
       </c>
       <c r="L317" t="n">
-        <v>102</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="318">
@@ -15658,12 +15658,12 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -15673,29 +15673,29 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F318" s="1" t="n">
-        <v>46289</v>
+        <v>46284</v>
       </c>
       <c r="G318" s="1" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="H318" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="I318" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J318" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>36.9</v>
+        <v>33.3</v>
       </c>
       <c r="L318" t="n">
-        <v>105.4</v>
+        <v>135.9</v>
       </c>
     </row>
     <row r="319">
@@ -15706,12 +15706,12 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -15721,29 +15721,29 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F319" s="1" t="n">
-        <v>46289</v>
+        <v>46284</v>
       </c>
       <c r="G319" s="1" t="n">
-        <v>46296</v>
+        <v>46291</v>
       </c>
       <c r="H319" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I319" t="n">
         <v>7</v>
       </c>
       <c r="J319" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>36.5</v>
+        <v>26.5</v>
       </c>
       <c r="L319" t="n">
-        <v>104.3</v>
+        <v>108.2</v>
       </c>
     </row>
     <row r="320">
@@ -15754,12 +15754,12 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -15769,29 +15769,29 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F320" s="1" t="n">
-        <v>46289</v>
+        <v>46284</v>
       </c>
       <c r="G320" s="1" t="n">
-        <v>46296</v>
+        <v>46291</v>
       </c>
       <c r="H320" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I320" t="n">
         <v>7</v>
       </c>
       <c r="J320" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K320" t="n">
-        <v>37</v>
+        <v>26.9</v>
       </c>
       <c r="L320" t="n">
-        <v>105.7</v>
+        <v>109.8</v>
       </c>
     </row>
     <row r="321">
@@ -15802,12 +15802,12 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -15817,29 +15817,29 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F321" s="1" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="G321" s="1" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="H321" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I321" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J321" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K321" t="n">
-        <v>42.8</v>
+        <v>28.4</v>
       </c>
       <c r="L321" t="n">
-        <v>122.3</v>
+        <v>115.9</v>
       </c>
     </row>
     <row r="322">
@@ -15850,12 +15850,12 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -15865,29 +15865,29 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F322" s="1" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="G322" s="1" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="H322" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I322" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J322" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K322" t="n">
-        <v>43.5</v>
+        <v>27.6</v>
       </c>
       <c r="L322" t="n">
-        <v>124.3</v>
+        <v>112.7</v>
       </c>
     </row>
     <row r="323">
@@ -15898,7 +15898,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -15913,17 +15913,17 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F323" s="1" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="G323" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="H323" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I323" t="n">
         <v>7</v>
@@ -15932,10 +15932,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>27.8</v>
+        <v>23.9</v>
       </c>
       <c r="L323" t="n">
-        <v>113.5</v>
+        <v>97.59999999999999</v>
       </c>
     </row>
     <row r="324">
@@ -15946,7 +15946,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -15961,17 +15961,17 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F324" s="1" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="G324" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="H324" s="1" t="n">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="I324" t="n">
         <v>7</v>
@@ -15980,10 +15980,10 @@
         <v>24.5</v>
       </c>
       <c r="K324" t="n">
-        <v>28.1</v>
+        <v>24.1</v>
       </c>
       <c r="L324" t="n">
-        <v>114.7</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="325">
@@ -15994,7 +15994,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -16009,29 +16009,29 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F325" s="1" t="n">
-        <v>46291</v>
+        <v>46287</v>
       </c>
       <c r="G325" s="1" t="n">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="H325" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I325" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J325" t="n">
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>28.9</v>
+        <v>28.8</v>
       </c>
       <c r="L325" t="n">
-        <v>118</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="326">
@@ -16042,7 +16042,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -16057,29 +16057,29 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F326" s="1" t="n">
-        <v>46291</v>
+        <v>46287</v>
       </c>
       <c r="G326" s="1" t="n">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="H326" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I326" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J326" t="n">
         <v>24.5</v>
       </c>
       <c r="K326" t="n">
-        <v>29.4</v>
+        <v>29.8</v>
       </c>
       <c r="L326" t="n">
-        <v>120</v>
+        <v>121.6</v>
       </c>
     </row>
     <row r="327">
@@ -16090,7 +16090,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -16105,14 +16105,14 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F327" s="1" t="n">
-        <v>46291</v>
+        <v>46287</v>
       </c>
       <c r="G327" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="H327" s="1" t="n">
         <v>46301</v>
@@ -16121,13 +16121,13 @@
         <v>7</v>
       </c>
       <c r="J327" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K327" t="n">
-        <v>36.4</v>
+        <v>22.6</v>
       </c>
       <c r="L327" t="n">
-        <v>104</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="328">
@@ -16138,7 +16138,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -16153,14 +16153,14 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F328" s="1" t="n">
-        <v>46291</v>
+        <v>46287</v>
       </c>
       <c r="G328" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="H328" s="1" t="n">
         <v>46301</v>
@@ -16169,13 +16169,1261 @@
         <v>7</v>
       </c>
       <c r="J328" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K328" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="L328" t="n">
+        <v>95.5</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Pilote 145 salón comunal</t>
+        </is>
+      </c>
+      <c r="F329" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G329" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H329" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I329" t="n">
+        <v>14</v>
+      </c>
+      <c r="J329" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K329" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="L329" t="n">
+        <v>109.8</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Pilote 145 salón comunal</t>
+        </is>
+      </c>
+      <c r="F330" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G330" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H330" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I330" t="n">
+        <v>14</v>
+      </c>
+      <c r="J330" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K330" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="L330" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Pilote 145 salón comunal</t>
+        </is>
+      </c>
+      <c r="F331" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G331" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H331" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I331" t="n">
+        <v>7</v>
+      </c>
+      <c r="J331" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K331" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="L331" t="n">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Pilote 145 salón comunal</t>
+        </is>
+      </c>
+      <c r="F332" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G332" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H332" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I332" t="n">
+        <v>7</v>
+      </c>
+      <c r="J332" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K332" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="L332" t="n">
+        <v>88.2</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Pilote 95 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F333" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G333" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H333" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I333" t="n">
+        <v>14</v>
+      </c>
+      <c r="J333" t="n">
+        <v>35</v>
+      </c>
+      <c r="K333" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="L333" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Pilote 95 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F334" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G334" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H334" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I334" t="n">
+        <v>14</v>
+      </c>
+      <c r="J334" t="n">
+        <v>35</v>
+      </c>
+      <c r="K334" t="n">
+        <v>39</v>
+      </c>
+      <c r="L334" t="n">
+        <v>111.4</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Pilote 95 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F335" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G335" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H335" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I335" t="n">
+        <v>7</v>
+      </c>
+      <c r="J335" t="n">
+        <v>35</v>
+      </c>
+      <c r="K335" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="L335" t="n">
+        <v>99.40000000000001</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>P53</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Pilote 95 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F336" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G336" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H336" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I336" t="n">
+        <v>7</v>
+      </c>
+      <c r="J336" t="n">
+        <v>35</v>
+      </c>
+      <c r="K336" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="L336" t="n">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>P54</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Pilote 67 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F337" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G337" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H337" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I337" t="n">
+        <v>7</v>
+      </c>
+      <c r="J337" t="n">
+        <v>35</v>
+      </c>
+      <c r="K337" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="L337" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>P54</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Pilote 67 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F338" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G338" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H338" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I338" t="n">
+        <v>7</v>
+      </c>
+      <c r="J338" t="n">
+        <v>35</v>
+      </c>
+      <c r="K338" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="L338" t="n">
+        <v>105.4</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>P55</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Pilote 65 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F339" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G339" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H339" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I339" t="n">
+        <v>7</v>
+      </c>
+      <c r="J339" t="n">
+        <v>35</v>
+      </c>
+      <c r="K339" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="L339" t="n">
+        <v>104.3</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>P55</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Pilote 65 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F340" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G340" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H340" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I340" t="n">
+        <v>7</v>
+      </c>
+      <c r="J340" t="n">
+        <v>35</v>
+      </c>
+      <c r="K340" t="n">
+        <v>37</v>
+      </c>
+      <c r="L340" t="n">
+        <v>105.7</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>P56</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Pilote 76 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F341" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G341" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H341" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I341" t="n">
+        <v>7</v>
+      </c>
+      <c r="J341" t="n">
+        <v>35</v>
+      </c>
+      <c r="K341" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="L341" t="n">
+        <v>122.3</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>P56</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Pilote 76 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F342" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G342" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H342" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I342" t="n">
+        <v>7</v>
+      </c>
+      <c r="J342" t="n">
+        <v>35</v>
+      </c>
+      <c r="K342" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="L342" t="n">
+        <v>124.3</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>P57</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+        </is>
+      </c>
+      <c r="F343" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G343" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H343" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I343" t="n">
+        <v>7</v>
+      </c>
+      <c r="J343" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K343" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="L343" t="n">
+        <v>113.5</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>P57</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+        </is>
+      </c>
+      <c r="F344" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G344" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H344" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I344" t="n">
+        <v>7</v>
+      </c>
+      <c r="J344" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K344" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="L344" t="n">
+        <v>114.7</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>P58</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
+        </is>
+      </c>
+      <c r="F345" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G345" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H345" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I345" t="n">
+        <v>7</v>
+      </c>
+      <c r="J345" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K345" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="L345" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>P58</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
+        </is>
+      </c>
+      <c r="F346" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G346" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H346" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I346" t="n">
+        <v>7</v>
+      </c>
+      <c r="J346" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K346" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="L346" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>P59</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Pilote 60 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F347" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G347" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H347" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I347" t="n">
+        <v>7</v>
+      </c>
+      <c r="J347" t="n">
+        <v>35</v>
+      </c>
+      <c r="K347" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="L347" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>P59</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Pilote 60 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F348" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G348" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H348" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="I348" t="n">
+        <v>7</v>
+      </c>
+      <c r="J348" t="n">
+        <v>35</v>
+      </c>
+      <c r="K348" t="n">
         <v>35.2</v>
       </c>
-      <c r="L328" t="n">
+      <c r="L348" t="n">
         <v>100.6</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>P60</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F349" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="G349" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="H349" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I349" t="n">
+        <v>7</v>
+      </c>
+      <c r="J349" t="n">
+        <v>35</v>
+      </c>
+      <c r="K349" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="L349" t="n">
+        <v>118.3</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>P60</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F350" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="G350" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="H350" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I350" t="n">
+        <v>7</v>
+      </c>
+      <c r="J350" t="n">
+        <v>35</v>
+      </c>
+      <c r="K350" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="L350" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>P61</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F351" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G351" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H351" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I351" t="n">
+        <v>7</v>
+      </c>
+      <c r="J351" t="n">
+        <v>35</v>
+      </c>
+      <c r="K351" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="L351" t="n">
+        <v>107.1</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>P61</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F352" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G352" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H352" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I352" t="n">
+        <v>7</v>
+      </c>
+      <c r="J352" t="n">
+        <v>35</v>
+      </c>
+      <c r="K352" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="L352" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>P62</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F353" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G353" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H353" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I353" t="n">
+        <v>7</v>
+      </c>
+      <c r="J353" t="n">
+        <v>35</v>
+      </c>
+      <c r="K353" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="L353" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>P62</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>No Especificado</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+        </is>
+      </c>
+      <c r="F354" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G354" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H354" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I354" t="n">
+        <v>7</v>
+      </c>
+      <c r="J354" t="n">
+        <v>35</v>
+      </c>
+      <c r="K354" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="L354" t="n">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-20 16:24:52
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L439"/>
+  <dimension ref="A1:L451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17600,22 +17600,22 @@
         <v>46284</v>
       </c>
       <c r="G358" s="1" t="n">
-        <v>46298</v>
+        <v>46312</v>
       </c>
       <c r="H358" s="1" t="n">
-        <v>46301</v>
+        <v>46315</v>
       </c>
       <c r="I358" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J358" t="n">
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>32</v>
+        <v>38.9</v>
       </c>
       <c r="L358" t="n">
-        <v>130.6</v>
+        <v>158.8</v>
       </c>
     </row>
     <row r="359">
@@ -17648,22 +17648,22 @@
         <v>46284</v>
       </c>
       <c r="G359" s="1" t="n">
-        <v>46298</v>
+        <v>46312</v>
       </c>
       <c r="H359" s="1" t="n">
-        <v>46301</v>
+        <v>46315</v>
       </c>
       <c r="I359" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J359" t="n">
         <v>24.5</v>
       </c>
       <c r="K359" t="n">
-        <v>33.3</v>
+        <v>39.8</v>
       </c>
       <c r="L359" t="n">
-        <v>135.9</v>
+        <v>162.4</v>
       </c>
     </row>
     <row r="360">
@@ -17696,22 +17696,22 @@
         <v>46284</v>
       </c>
       <c r="G360" s="1" t="n">
-        <v>46291</v>
+        <v>46312</v>
       </c>
       <c r="H360" s="1" t="n">
-        <v>46294</v>
+        <v>46315</v>
       </c>
       <c r="I360" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J360" t="n">
         <v>24.5</v>
       </c>
       <c r="K360" t="n">
-        <v>26.5</v>
+        <v>38.6</v>
       </c>
       <c r="L360" t="n">
-        <v>108.2</v>
+        <v>157.6</v>
       </c>
     </row>
     <row r="361">
@@ -17744,22 +17744,22 @@
         <v>46284</v>
       </c>
       <c r="G361" s="1" t="n">
-        <v>46291</v>
+        <v>46298</v>
       </c>
       <c r="H361" s="1" t="n">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="I361" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J361" t="n">
         <v>24.5</v>
       </c>
       <c r="K361" t="n">
-        <v>26.9</v>
+        <v>32</v>
       </c>
       <c r="L361" t="n">
-        <v>109.8</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="362">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -17785,17 +17785,17 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F362" s="1" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="G362" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="H362" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="I362" t="n">
         <v>14</v>
@@ -17804,10 +17804,10 @@
         <v>24.5</v>
       </c>
       <c r="K362" t="n">
-        <v>28.4</v>
+        <v>33.3</v>
       </c>
       <c r="L362" t="n">
-        <v>115.9</v>
+        <v>135.9</v>
       </c>
     </row>
     <row r="363">
@@ -17818,7 +17818,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -17833,29 +17833,29 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F363" s="1" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="G363" s="1" t="n">
-        <v>46300</v>
+        <v>46291</v>
       </c>
       <c r="H363" s="1" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="I363" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J363" t="n">
         <v>24.5</v>
       </c>
       <c r="K363" t="n">
-        <v>27.6</v>
+        <v>26.5</v>
       </c>
       <c r="L363" t="n">
-        <v>112.7</v>
+        <v>108.2</v>
       </c>
     </row>
     <row r="364">
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>P50</t>
+          <t>P49</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -17881,14 +17881,14 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
+          <t xml:space="preserve">Pilote 127 - 123 salón comunal </t>
         </is>
       </c>
       <c r="F364" s="1" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="G364" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="H364" s="1" t="n">
         <v>46294</v>
@@ -17900,10 +17900,10 @@
         <v>24.5</v>
       </c>
       <c r="K364" t="n">
-        <v>23.9</v>
+        <v>26.9</v>
       </c>
       <c r="L364" t="n">
-        <v>97.59999999999999</v>
+        <v>109.8</v>
       </c>
     </row>
     <row r="365">
@@ -17936,22 +17936,22 @@
         <v>46286</v>
       </c>
       <c r="G365" s="1" t="n">
-        <v>46293</v>
+        <v>46314</v>
       </c>
       <c r="H365" s="1" t="n">
-        <v>46294</v>
+        <v>46315</v>
       </c>
       <c r="I365" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J365" t="n">
         <v>24.5</v>
       </c>
       <c r="K365" t="n">
-        <v>24.1</v>
+        <v>34.1</v>
       </c>
       <c r="L365" t="n">
-        <v>98.40000000000001</v>
+        <v>139.2</v>
       </c>
     </row>
     <row r="366">
@@ -17962,7 +17962,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -17977,29 +17977,29 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F366" s="1" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="G366" s="1" t="n">
-        <v>46301</v>
+        <v>46314</v>
       </c>
       <c r="H366" s="1" t="n">
-        <v>46302</v>
+        <v>46315</v>
       </c>
       <c r="I366" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J366" t="n">
         <v>24.5</v>
       </c>
       <c r="K366" t="n">
-        <v>28.8</v>
+        <v>32.6</v>
       </c>
       <c r="L366" t="n">
-        <v>117.6</v>
+        <v>133.1</v>
       </c>
     </row>
     <row r="367">
@@ -18010,7 +18010,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -18025,29 +18025,29 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F367" s="1" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="G367" s="1" t="n">
-        <v>46301</v>
+        <v>46314</v>
       </c>
       <c r="H367" s="1" t="n">
-        <v>46302</v>
+        <v>46315</v>
       </c>
       <c r="I367" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J367" t="n">
         <v>24.5</v>
       </c>
       <c r="K367" t="n">
-        <v>29.8</v>
+        <v>33.7</v>
       </c>
       <c r="L367" t="n">
-        <v>121.6</v>
+        <v>137.6</v>
       </c>
     </row>
     <row r="368">
@@ -18058,7 +18058,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -18073,29 +18073,29 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F368" s="1" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="G368" s="1" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="H368" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I368" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J368" t="n">
         <v>24.5</v>
       </c>
       <c r="K368" t="n">
-        <v>22.6</v>
+        <v>28.4</v>
       </c>
       <c r="L368" t="n">
-        <v>92.2</v>
+        <v>115.9</v>
       </c>
     </row>
     <row r="369">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>P51</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -18121,29 +18121,29 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F369" s="1" t="n">
-        <v>46287</v>
+        <v>46286</v>
       </c>
       <c r="G369" s="1" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="H369" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I369" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J369" t="n">
         <v>24.5</v>
       </c>
       <c r="K369" t="n">
-        <v>23.4</v>
+        <v>27.6</v>
       </c>
       <c r="L369" t="n">
-        <v>95.5</v>
+        <v>112.7</v>
       </c>
     </row>
     <row r="370">
@@ -18154,12 +18154,12 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -18169,29 +18169,29 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F370" s="1" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="G370" s="1" t="n">
-        <v>46302</v>
+        <v>46293</v>
       </c>
       <c r="H370" s="1" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="I370" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J370" t="n">
         <v>24.5</v>
       </c>
       <c r="K370" t="n">
-        <v>26.9</v>
+        <v>23.9</v>
       </c>
       <c r="L370" t="n">
-        <v>109.8</v>
+        <v>97.59999999999999</v>
       </c>
     </row>
     <row r="371">
@@ -18202,12 +18202,12 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P50</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -18217,29 +18217,29 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 120 - 122 - 126 salón comunal </t>
         </is>
       </c>
       <c r="F371" s="1" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="G371" s="1" t="n">
-        <v>46302</v>
+        <v>46293</v>
       </c>
       <c r="H371" s="1" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="I371" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J371" t="n">
         <v>24.5</v>
       </c>
       <c r="K371" t="n">
-        <v>27.2</v>
+        <v>24.1</v>
       </c>
       <c r="L371" t="n">
-        <v>111</v>
+        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="372">
@@ -18250,12 +18250,12 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -18265,29 +18265,29 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F372" s="1" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="G372" s="1" t="n">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="H372" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I372" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J372" t="n">
         <v>24.5</v>
       </c>
       <c r="K372" t="n">
-        <v>21.4</v>
+        <v>28.8</v>
       </c>
       <c r="L372" t="n">
-        <v>87.3</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="373">
@@ -18298,12 +18298,12 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>P52</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -18313,29 +18313,29 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Pilote 145 salón comunal</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F373" s="1" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="G373" s="1" t="n">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="H373" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I373" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J373" t="n">
         <v>24.5</v>
       </c>
       <c r="K373" t="n">
-        <v>21.6</v>
+        <v>29.8</v>
       </c>
       <c r="L373" t="n">
-        <v>88.2</v>
+        <v>121.6</v>
       </c>
     </row>
     <row r="374">
@@ -18346,12 +18346,12 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
@@ -18361,29 +18361,29 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F374" s="1" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="G374" s="1" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="H374" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="I374" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J374" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K374" t="n">
-        <v>37.8</v>
+        <v>22.6</v>
       </c>
       <c r="L374" t="n">
-        <v>108</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="375">
@@ -18394,12 +18394,12 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P51</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -18409,29 +18409,29 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 113 - 112 - 139 - 124 salón comunal </t>
         </is>
       </c>
       <c r="F375" s="1" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="G375" s="1" t="n">
-        <v>46302</v>
+        <v>46294</v>
       </c>
       <c r="H375" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="I375" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J375" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K375" t="n">
-        <v>39</v>
+        <v>23.4</v>
       </c>
       <c r="L375" t="n">
-        <v>111.4</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="376">
@@ -18442,7 +18442,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P52</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -18457,29 +18457,29 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t>Pilote 145 salón comunal</t>
         </is>
       </c>
       <c r="F376" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="G376" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="H376" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I376" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J376" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K376" t="n">
-        <v>34.8</v>
+        <v>26.9</v>
       </c>
       <c r="L376" t="n">
-        <v>99.40000000000001</v>
+        <v>109.8</v>
       </c>
     </row>
     <row r="377">
@@ -18490,7 +18490,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>P53</t>
+          <t>P52</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -18505,29 +18505,29 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Pilote 95 torre 2 tipo 2</t>
+          <t>Pilote 145 salón comunal</t>
         </is>
       </c>
       <c r="F377" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="G377" s="1" t="n">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="H377" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I377" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J377" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K377" t="n">
-        <v>33.8</v>
+        <v>27.2</v>
       </c>
       <c r="L377" t="n">
-        <v>96.59999999999999</v>
+        <v>111</v>
       </c>
     </row>
     <row r="378">
@@ -18538,7 +18538,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P52</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -18553,29 +18553,29 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t>Pilote 145 salón comunal</t>
         </is>
       </c>
       <c r="F378" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G378" s="1" t="n">
-        <v>46303</v>
+        <v>46295</v>
       </c>
       <c r="H378" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I378" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J378" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K378" t="n">
-        <v>44.7</v>
+        <v>21.4</v>
       </c>
       <c r="L378" t="n">
-        <v>127.7</v>
+        <v>87.3</v>
       </c>
     </row>
     <row r="379">
@@ -18586,7 +18586,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P52</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -18601,29 +18601,29 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t>Pilote 145 salón comunal</t>
         </is>
       </c>
       <c r="F379" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G379" s="1" t="n">
-        <v>46303</v>
+        <v>46295</v>
       </c>
       <c r="H379" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I379" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J379" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K379" t="n">
-        <v>44.2</v>
+        <v>21.6</v>
       </c>
       <c r="L379" t="n">
-        <v>126.3</v>
+        <v>88.2</v>
       </c>
     </row>
     <row r="380">
@@ -18634,7 +18634,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P53</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -18649,29 +18649,29 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t>Pilote 95 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F380" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G380" s="1" t="n">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="H380" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I380" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J380" t="n">
         <v>35</v>
       </c>
       <c r="K380" t="n">
-        <v>35.7</v>
+        <v>37.8</v>
       </c>
       <c r="L380" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="381">
@@ -18682,7 +18682,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>P54</t>
+          <t>P53</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -18697,29 +18697,29 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Pilote 67 torre 2 tipo 2</t>
+          <t>Pilote 95 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F381" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G381" s="1" t="n">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="H381" s="1" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="I381" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J381" t="n">
         <v>35</v>
       </c>
       <c r="K381" t="n">
-        <v>36.9</v>
+        <v>39</v>
       </c>
       <c r="L381" t="n">
-        <v>105.4</v>
+        <v>111.4</v>
       </c>
     </row>
     <row r="382">
@@ -18730,7 +18730,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P53</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -18745,29 +18745,29 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 95 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F382" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G382" s="1" t="n">
-        <v>46303</v>
+        <v>46295</v>
       </c>
       <c r="H382" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I382" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J382" t="n">
         <v>35</v>
       </c>
       <c r="K382" t="n">
-        <v>43.2</v>
+        <v>34.8</v>
       </c>
       <c r="L382" t="n">
-        <v>123.4</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="383">
@@ -18778,7 +18778,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P53</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -18793,29 +18793,29 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 95 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F383" s="1" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="G383" s="1" t="n">
-        <v>46303</v>
+        <v>46295</v>
       </c>
       <c r="H383" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I383" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J383" t="n">
         <v>35</v>
       </c>
       <c r="K383" t="n">
-        <v>43.9</v>
+        <v>33.8</v>
       </c>
       <c r="L383" t="n">
-        <v>125.4</v>
+        <v>96.59999999999999</v>
       </c>
     </row>
     <row r="384">
@@ -18826,7 +18826,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -18841,29 +18841,29 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F384" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="G384" s="1" t="n">
-        <v>46296</v>
+        <v>46303</v>
       </c>
       <c r="H384" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I384" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J384" t="n">
         <v>35</v>
       </c>
       <c r="K384" t="n">
-        <v>36.5</v>
+        <v>44.7</v>
       </c>
       <c r="L384" t="n">
-        <v>104.3</v>
+        <v>127.7</v>
       </c>
     </row>
     <row r="385">
@@ -18874,7 +18874,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -18889,29 +18889,29 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F385" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="G385" s="1" t="n">
-        <v>46296</v>
+        <v>46303</v>
       </c>
       <c r="H385" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I385" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J385" t="n">
         <v>35</v>
       </c>
       <c r="K385" t="n">
-        <v>37</v>
+        <v>44.2</v>
       </c>
       <c r="L385" t="n">
-        <v>105.7</v>
+        <v>126.3</v>
       </c>
     </row>
     <row r="386">
@@ -18922,7 +18922,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -18937,29 +18937,29 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F386" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G386" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H386" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I386" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J386" t="n">
         <v>35</v>
       </c>
       <c r="K386" t="n">
-        <v>51.1</v>
+        <v>35.7</v>
       </c>
       <c r="L386" t="n">
-        <v>146</v>
+        <v>102</v>
       </c>
     </row>
     <row r="387">
@@ -18970,7 +18970,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -18985,29 +18985,29 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F387" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G387" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H387" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I387" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J387" t="n">
         <v>35</v>
       </c>
       <c r="K387" t="n">
-        <v>52.8</v>
+        <v>36.9</v>
       </c>
       <c r="L387" t="n">
-        <v>150.9</v>
+        <v>105.4</v>
       </c>
     </row>
     <row r="388">
@@ -19018,7 +19018,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -19033,29 +19033,29 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F388" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G388" s="1" t="n">
-        <v>46297</v>
+        <v>46303</v>
       </c>
       <c r="H388" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I388" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J388" t="n">
         <v>35</v>
       </c>
       <c r="K388" t="n">
-        <v>42.8</v>
+        <v>43.2</v>
       </c>
       <c r="L388" t="n">
-        <v>122.3</v>
+        <v>123.4</v>
       </c>
     </row>
     <row r="389">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -19081,29 +19081,29 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F389" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G389" s="1" t="n">
-        <v>46297</v>
+        <v>46303</v>
       </c>
       <c r="H389" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I389" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J389" t="n">
         <v>35</v>
       </c>
       <c r="K389" t="n">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
       <c r="L389" t="n">
-        <v>124.3</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="390">
@@ -19114,12 +19114,12 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
@@ -19129,29 +19129,29 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F390" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G390" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H390" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I390" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J390" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K390" t="n">
-        <v>33.6</v>
+        <v>36.5</v>
       </c>
       <c r="L390" t="n">
-        <v>137.1</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="391">
@@ -19162,12 +19162,12 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
@@ -19177,29 +19177,29 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F391" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G391" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H391" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I391" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J391" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K391" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="L391" t="n">
-        <v>134.7</v>
+        <v>105.7</v>
       </c>
     </row>
     <row r="392">
@@ -19210,12 +19210,12 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
@@ -19225,29 +19225,29 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F392" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="G392" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="H392" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I392" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J392" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K392" t="n">
-        <v>27.8</v>
+        <v>51.1</v>
       </c>
       <c r="L392" t="n">
-        <v>113.5</v>
+        <v>146</v>
       </c>
     </row>
     <row r="393">
@@ -19258,12 +19258,12 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -19273,29 +19273,29 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F393" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="G393" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="H393" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I393" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J393" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K393" t="n">
-        <v>28.1</v>
+        <v>52.8</v>
       </c>
       <c r="L393" t="n">
-        <v>114.7</v>
+        <v>150.9</v>
       </c>
     </row>
     <row r="394">
@@ -19306,12 +19306,12 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
@@ -19321,29 +19321,29 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F394" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G394" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H394" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I394" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J394" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K394" t="n">
-        <v>34.8</v>
+        <v>42.8</v>
       </c>
       <c r="L394" t="n">
-        <v>142</v>
+        <v>122.3</v>
       </c>
     </row>
     <row r="395">
@@ -19354,12 +19354,12 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
@@ -19369,29 +19369,29 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F395" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G395" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H395" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I395" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J395" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K395" t="n">
-        <v>35.8</v>
+        <v>43.5</v>
       </c>
       <c r="L395" t="n">
-        <v>146.1</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="396">
@@ -19402,7 +19402,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -19417,29 +19417,29 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F396" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G396" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H396" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I396" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J396" t="n">
         <v>24.5</v>
       </c>
       <c r="K396" t="n">
-        <v>28.9</v>
+        <v>33.6</v>
       </c>
       <c r="L396" t="n">
-        <v>118</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="397">
@@ -19450,7 +19450,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -19465,29 +19465,29 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F397" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G397" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H397" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I397" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J397" t="n">
         <v>24.5</v>
       </c>
       <c r="K397" t="n">
-        <v>29.4</v>
+        <v>33</v>
       </c>
       <c r="L397" t="n">
-        <v>120</v>
+        <v>134.7</v>
       </c>
     </row>
     <row r="398">
@@ -19498,7 +19498,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -19513,29 +19513,29 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F398" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G398" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H398" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I398" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J398" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K398" t="n">
-        <v>42.6</v>
+        <v>27.8</v>
       </c>
       <c r="L398" t="n">
-        <v>121.7</v>
+        <v>113.5</v>
       </c>
     </row>
     <row r="399">
@@ -19546,7 +19546,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -19561,29 +19561,29 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F399" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G399" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H399" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I399" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J399" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K399" t="n">
-        <v>43.5</v>
+        <v>28.1</v>
       </c>
       <c r="L399" t="n">
-        <v>124.3</v>
+        <v>114.7</v>
       </c>
     </row>
     <row r="400">
@@ -19594,7 +19594,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -19609,29 +19609,29 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F400" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G400" s="1" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="H400" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I400" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J400" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K400" t="n">
-        <v>36.4</v>
+        <v>34.8</v>
       </c>
       <c r="L400" t="n">
-        <v>104</v>
+        <v>142</v>
       </c>
     </row>
     <row r="401">
@@ -19642,7 +19642,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -19657,29 +19657,29 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F401" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G401" s="1" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="H401" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I401" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J401" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K401" t="n">
-        <v>35.2</v>
+        <v>35.8</v>
       </c>
       <c r="L401" t="n">
-        <v>100.6</v>
+        <v>146.1</v>
       </c>
     </row>
     <row r="402">
@@ -19690,12 +19690,12 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
@@ -19705,29 +19705,29 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F402" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G402" s="1" t="n">
-        <v>46307</v>
+        <v>46298</v>
       </c>
       <c r="H402" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I402" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J402" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K402" t="n">
-        <v>49</v>
+        <v>28.9</v>
       </c>
       <c r="L402" t="n">
-        <v>140</v>
+        <v>118</v>
       </c>
     </row>
     <row r="403">
@@ -19738,12 +19738,12 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
@@ -19753,29 +19753,29 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F403" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G403" s="1" t="n">
-        <v>46307</v>
+        <v>46298</v>
       </c>
       <c r="H403" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I403" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J403" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K403" t="n">
-        <v>47.9</v>
+        <v>29.4</v>
       </c>
       <c r="L403" t="n">
-        <v>136.9</v>
+        <v>120</v>
       </c>
     </row>
     <row r="404">
@@ -19786,12 +19786,12 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
@@ -19801,29 +19801,29 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F404" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G404" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="H404" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I404" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J404" t="n">
         <v>35</v>
       </c>
       <c r="K404" t="n">
-        <v>41.4</v>
+        <v>42.6</v>
       </c>
       <c r="L404" t="n">
-        <v>118.3</v>
+        <v>121.7</v>
       </c>
     </row>
     <row r="405">
@@ -19834,12 +19834,12 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
@@ -19849,29 +19849,29 @@
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F405" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G405" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="H405" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I405" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J405" t="n">
         <v>35</v>
       </c>
       <c r="K405" t="n">
-        <v>40.3</v>
+        <v>43.5</v>
       </c>
       <c r="L405" t="n">
-        <v>115.1</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="406">
@@ -19882,12 +19882,12 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
@@ -19897,29 +19897,29 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F406" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G406" s="1" t="n">
-        <v>46308</v>
+        <v>46298</v>
       </c>
       <c r="H406" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I406" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J406" t="n">
         <v>35</v>
       </c>
       <c r="K406" t="n">
-        <v>44.3</v>
+        <v>36.4</v>
       </c>
       <c r="L406" t="n">
-        <v>126.6</v>
+        <v>104</v>
       </c>
     </row>
     <row r="407">
@@ -19930,12 +19930,12 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -19945,29 +19945,29 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F407" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G407" s="1" t="n">
-        <v>46308</v>
+        <v>46298</v>
       </c>
       <c r="H407" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I407" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J407" t="n">
         <v>35</v>
       </c>
       <c r="K407" t="n">
-        <v>44.9</v>
+        <v>35.2</v>
       </c>
       <c r="L407" t="n">
-        <v>128.3</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="408">
@@ -19978,7 +19978,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -19993,29 +19993,29 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F408" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G408" s="1" t="n">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="H408" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I408" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J408" t="n">
         <v>35</v>
       </c>
       <c r="K408" t="n">
-        <v>37.5</v>
+        <v>49</v>
       </c>
       <c r="L408" t="n">
-        <v>107.1</v>
+        <v>140</v>
       </c>
     </row>
     <row r="409">
@@ -20026,7 +20026,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -20041,29 +20041,29 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F409" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G409" s="1" t="n">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="H409" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I409" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J409" t="n">
         <v>35</v>
       </c>
       <c r="K409" t="n">
-        <v>36.4</v>
+        <v>47.9</v>
       </c>
       <c r="L409" t="n">
-        <v>104</v>
+        <v>136.9</v>
       </c>
     </row>
     <row r="410">
@@ -20074,7 +20074,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -20089,29 +20089,29 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F410" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G410" s="1" t="n">
-        <v>46308</v>
+        <v>46300</v>
       </c>
       <c r="H410" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I410" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J410" t="n">
         <v>35</v>
       </c>
       <c r="K410" t="n">
-        <v>43.9</v>
+        <v>41.4</v>
       </c>
       <c r="L410" t="n">
-        <v>125.4</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="411">
@@ -20122,7 +20122,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -20137,29 +20137,29 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F411" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G411" s="1" t="n">
-        <v>46308</v>
+        <v>46300</v>
       </c>
       <c r="H411" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I411" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J411" t="n">
         <v>35</v>
       </c>
       <c r="K411" t="n">
-        <v>43.7</v>
+        <v>40.3</v>
       </c>
       <c r="L411" t="n">
-        <v>124.9</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="412">
@@ -20170,7 +20170,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -20185,29 +20185,29 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F412" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="G412" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H412" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I412" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J412" t="n">
         <v>35</v>
       </c>
       <c r="K412" t="n">
-        <v>38.5</v>
+        <v>44.3</v>
       </c>
       <c r="L412" t="n">
-        <v>110</v>
+        <v>126.6</v>
       </c>
     </row>
     <row r="413">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -20233,29 +20233,29 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F413" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="G413" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H413" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I413" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J413" t="n">
         <v>35</v>
       </c>
       <c r="K413" t="n">
-        <v>37.1</v>
+        <v>44.9</v>
       </c>
       <c r="L413" t="n">
-        <v>106</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="414">
@@ -20266,12 +20266,12 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
@@ -20281,29 +20281,29 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F414" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G414" s="1" t="n">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="H414" s="1" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="I414" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J414" t="n">
         <v>35</v>
       </c>
       <c r="K414" t="n">
-        <v>33.5</v>
+        <v>37.5</v>
       </c>
       <c r="L414" t="n">
-        <v>95.7</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="415">
@@ -20314,12 +20314,12 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -20329,29 +20329,29 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F415" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G415" s="1" t="n">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="H415" s="1" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="I415" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J415" t="n">
         <v>35</v>
       </c>
       <c r="K415" t="n">
-        <v>32</v>
+        <v>36.4</v>
       </c>
       <c r="L415" t="n">
-        <v>91.40000000000001</v>
+        <v>104</v>
       </c>
     </row>
     <row r="416">
@@ -20362,12 +20362,12 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
@@ -20377,29 +20377,29 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F416" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G416" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H416" s="1" t="n">
         <v>46309</v>
       </c>
       <c r="I416" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J416" t="n">
         <v>35</v>
       </c>
       <c r="K416" t="n">
-        <v>24.4</v>
+        <v>43.9</v>
       </c>
       <c r="L416" t="n">
-        <v>69.7</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="417">
@@ -20410,12 +20410,12 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
@@ -20425,29 +20425,29 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F417" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G417" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H417" s="1" t="n">
         <v>46309</v>
       </c>
       <c r="I417" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J417" t="n">
         <v>35</v>
       </c>
       <c r="K417" t="n">
-        <v>24.6</v>
+        <v>43.7</v>
       </c>
       <c r="L417" t="n">
-        <v>70.3</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="418">
@@ -20458,12 +20458,12 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
@@ -20473,17 +20473,17 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F418" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G418" s="1" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="H418" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I418" t="n">
         <v>7</v>
@@ -20492,10 +20492,10 @@
         <v>35</v>
       </c>
       <c r="K418" t="n">
-        <v>22.8</v>
+        <v>38.5</v>
       </c>
       <c r="L418" t="n">
-        <v>65.09999999999999</v>
+        <v>110</v>
       </c>
     </row>
     <row r="419">
@@ -20506,12 +20506,12 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -20521,17 +20521,17 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F419" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G419" s="1" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="H419" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I419" t="n">
         <v>7</v>
@@ -20540,10 +20540,10 @@
         <v>35</v>
       </c>
       <c r="K419" t="n">
-        <v>23.3</v>
+        <v>37.1</v>
       </c>
       <c r="L419" t="n">
-        <v>66.59999999999999</v>
+        <v>106</v>
       </c>
     </row>
     <row r="420">
@@ -20554,7 +20554,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -20569,29 +20569,29 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F420" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G420" s="1" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="H420" s="1" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I420" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J420" t="n">
         <v>35</v>
       </c>
       <c r="K420" t="n">
-        <v>34.3</v>
+        <v>33.5</v>
       </c>
       <c r="L420" t="n">
-        <v>98</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="421">
@@ -20602,7 +20602,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -20617,29 +20617,29 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F421" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G421" s="1" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="H421" s="1" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I421" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J421" t="n">
         <v>35</v>
       </c>
       <c r="K421" t="n">
-        <v>34.7</v>
+        <v>32</v>
       </c>
       <c r="L421" t="n">
-        <v>99.09999999999999</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="422">
@@ -20650,7 +20650,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -20665,14 +20665,14 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F422" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G422" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="H422" s="1" t="n">
         <v>46309</v>
@@ -20684,10 +20684,10 @@
         <v>35</v>
       </c>
       <c r="K422" t="n">
-        <v>33.4</v>
+        <v>24.4</v>
       </c>
       <c r="L422" t="n">
-        <v>95.40000000000001</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="423">
@@ -20698,7 +20698,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -20713,14 +20713,14 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F423" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G423" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="H423" s="1" t="n">
         <v>46309</v>
@@ -20732,10 +20732,10 @@
         <v>35</v>
       </c>
       <c r="K423" t="n">
-        <v>32.4</v>
+        <v>24.6</v>
       </c>
       <c r="L423" t="n">
-        <v>92.59999999999999</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="424">
@@ -20746,7 +20746,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -20761,29 +20761,29 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F424" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G424" s="1" t="n">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="H424" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I424" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J424" t="n">
         <v>35</v>
       </c>
       <c r="K424" t="n">
-        <v>37.9</v>
+        <v>35.4</v>
       </c>
       <c r="L424" t="n">
-        <v>108.3</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="425">
@@ -20794,7 +20794,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -20809,29 +20809,29 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F425" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G425" s="1" t="n">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="H425" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I425" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J425" t="n">
         <v>35</v>
       </c>
       <c r="K425" t="n">
-        <v>38.4</v>
+        <v>35.8</v>
       </c>
       <c r="L425" t="n">
-        <v>109.7</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="426">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -20857,14 +20857,14 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F426" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G426" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H426" s="1" t="n">
         <v>46309</v>
@@ -20876,10 +20876,10 @@
         <v>35</v>
       </c>
       <c r="K426" t="n">
-        <v>38.9</v>
+        <v>22.8</v>
       </c>
       <c r="L426" t="n">
-        <v>111.1</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="427">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -20905,14 +20905,14 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F427" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G427" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H427" s="1" t="n">
         <v>46309</v>
@@ -20924,10 +20924,10 @@
         <v>35</v>
       </c>
       <c r="K427" t="n">
-        <v>38</v>
+        <v>23.3</v>
       </c>
       <c r="L427" t="n">
-        <v>108.6</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="428">
@@ -20938,12 +20938,12 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -20953,29 +20953,29 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F428" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G428" s="1" t="n">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="H428" s="1" t="n">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="I428" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J428" t="n">
         <v>35</v>
       </c>
       <c r="K428" t="n">
-        <v>41.2</v>
+        <v>37.8</v>
       </c>
       <c r="L428" t="n">
-        <v>117.7</v>
+        <v>108</v>
       </c>
     </row>
     <row r="429">
@@ -20986,12 +20986,12 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -21001,29 +21001,29 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F429" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G429" s="1" t="n">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="H429" s="1" t="n">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="I429" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J429" t="n">
         <v>35</v>
       </c>
       <c r="K429" t="n">
-        <v>41.7</v>
+        <v>38.9</v>
       </c>
       <c r="L429" t="n">
-        <v>119.1</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="430">
@@ -21034,12 +21034,12 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -21049,17 +21049,17 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F430" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G430" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H430" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H430" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I430" t="n">
         <v>7</v>
@@ -21068,10 +21068,10 @@
         <v>35</v>
       </c>
       <c r="K430" t="n">
-        <v>32.8</v>
+        <v>34.3</v>
       </c>
       <c r="L430" t="n">
-        <v>93.7</v>
+        <v>98</v>
       </c>
     </row>
     <row r="431">
@@ -21082,12 +21082,12 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -21097,17 +21097,17 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F431" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G431" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H431" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H431" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I431" t="n">
         <v>7</v>
@@ -21116,10 +21116,10 @@
         <v>35</v>
       </c>
       <c r="K431" t="n">
-        <v>31.8</v>
+        <v>34.7</v>
       </c>
       <c r="L431" t="n">
-        <v>90.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="432">
@@ -21130,12 +21130,12 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
@@ -21145,29 +21145,29 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F432" s="1" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="G432" s="1" t="n">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="H432" s="1" t="n">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="I432" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J432" t="n">
         <v>35</v>
       </c>
       <c r="K432" t="n">
-        <v>35.7</v>
+        <v>38.8</v>
       </c>
       <c r="L432" t="n">
-        <v>102</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="433">
@@ -21178,12 +21178,12 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -21193,29 +21193,29 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F433" s="1" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="G433" s="1" t="n">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="H433" s="1" t="n">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="I433" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J433" t="n">
         <v>35</v>
       </c>
       <c r="K433" t="n">
-        <v>36.2</v>
+        <v>38.3</v>
       </c>
       <c r="L433" t="n">
-        <v>103.4</v>
+        <v>109.4</v>
       </c>
     </row>
     <row r="434">
@@ -21226,12 +21226,12 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
@@ -21241,29 +21241,29 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F434" s="1" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="G434" s="1" t="n">
-        <v>46310</v>
+        <v>46307</v>
       </c>
       <c r="H434" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="I434" t="n">
         <v>7</v>
       </c>
       <c r="J434" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K434" t="n">
-        <v>24.4</v>
+        <v>33.4</v>
       </c>
       <c r="L434" t="n">
-        <v>99.59999999999999</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="435">
@@ -21274,12 +21274,12 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -21289,29 +21289,29 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F435" s="1" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="G435" s="1" t="n">
-        <v>46310</v>
+        <v>46307</v>
       </c>
       <c r="H435" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="I435" t="n">
         <v>7</v>
       </c>
       <c r="J435" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K435" t="n">
-        <v>23.6</v>
+        <v>32.4</v>
       </c>
       <c r="L435" t="n">
-        <v>96.3</v>
+        <v>92.59999999999999</v>
       </c>
     </row>
     <row r="436">
@@ -21322,12 +21322,12 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
@@ -21337,17 +21337,17 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F436" s="1" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="G436" s="1" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H436" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I436" t="n">
         <v>7</v>
@@ -21356,10 +21356,10 @@
         <v>35</v>
       </c>
       <c r="K436" t="n">
-        <v>34.6</v>
+        <v>37.9</v>
       </c>
       <c r="L436" t="n">
-        <v>98.90000000000001</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="437">
@@ -21370,12 +21370,12 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -21385,17 +21385,17 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F437" s="1" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="G437" s="1" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H437" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I437" t="n">
         <v>7</v>
@@ -21404,10 +21404,10 @@
         <v>35</v>
       </c>
       <c r="K437" t="n">
-        <v>34.7</v>
+        <v>38.4</v>
       </c>
       <c r="L437" t="n">
-        <v>99.09999999999999</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="438">
@@ -21418,7 +21418,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -21433,17 +21433,17 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F438" s="1" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="G438" s="1" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H438" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I438" t="n">
         <v>7</v>
@@ -21452,10 +21452,10 @@
         <v>35</v>
       </c>
       <c r="K438" t="n">
-        <v>32.5</v>
+        <v>38.9</v>
       </c>
       <c r="L438" t="n">
-        <v>92.90000000000001</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="439">
@@ -21466,7 +21466,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -21481,17 +21481,17 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F439" s="1" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="G439" s="1" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H439" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I439" t="n">
         <v>7</v>
@@ -21500,9 +21500,585 @@
         <v>35</v>
       </c>
       <c r="K439" t="n">
+        <v>38</v>
+      </c>
+      <c r="L439" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>P74</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F440" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G440" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H440" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I440" t="n">
+        <v>7</v>
+      </c>
+      <c r="J440" t="n">
+        <v>35</v>
+      </c>
+      <c r="K440" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="L440" t="n">
+        <v>117.7</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>P74</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F441" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G441" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H441" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I441" t="n">
+        <v>7</v>
+      </c>
+      <c r="J441" t="n">
+        <v>35</v>
+      </c>
+      <c r="K441" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="L441" t="n">
+        <v>119.1</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Pilote 99 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F442" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G442" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H442" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I442" t="n">
+        <v>7</v>
+      </c>
+      <c r="J442" t="n">
+        <v>35</v>
+      </c>
+      <c r="K442" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="L442" t="n">
+        <v>93.7</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Pilote 99 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F443" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="G443" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H443" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I443" t="n">
+        <v>7</v>
+      </c>
+      <c r="J443" t="n">
+        <v>35</v>
+      </c>
+      <c r="K443" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="L443" t="n">
+        <v>90.90000000000001</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F444" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G444" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H444" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I444" t="n">
+        <v>7</v>
+      </c>
+      <c r="J444" t="n">
+        <v>35</v>
+      </c>
+      <c r="K444" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="L444" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F445" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G445" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H445" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I445" t="n">
+        <v>7</v>
+      </c>
+      <c r="J445" t="n">
+        <v>35</v>
+      </c>
+      <c r="K445" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="L445" t="n">
+        <v>103.4</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F446" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G446" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H446" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I446" t="n">
+        <v>7</v>
+      </c>
+      <c r="J446" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K446" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="L446" t="n">
+        <v>99.59999999999999</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F447" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G447" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H447" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I447" t="n">
+        <v>7</v>
+      </c>
+      <c r="J447" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K447" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L447" t="n">
+        <v>96.3</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>P78</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F448" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G448" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H448" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I448" t="n">
+        <v>7</v>
+      </c>
+      <c r="J448" t="n">
+        <v>35</v>
+      </c>
+      <c r="K448" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="L448" t="n">
+        <v>98.90000000000001</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>P78</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F449" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G449" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H449" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I449" t="n">
+        <v>7</v>
+      </c>
+      <c r="J449" t="n">
+        <v>35</v>
+      </c>
+      <c r="K449" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="L449" t="n">
+        <v>99.09999999999999</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F450" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G450" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H450" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I450" t="n">
+        <v>7</v>
+      </c>
+      <c r="J450" t="n">
+        <v>35</v>
+      </c>
+      <c r="K450" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="L450" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F451" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G451" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H451" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I451" t="n">
+        <v>7</v>
+      </c>
+      <c r="J451" t="n">
+        <v>35</v>
+      </c>
+      <c r="K451" t="n">
         <v>32.2</v>
       </c>
-      <c r="L439" t="n">
+      <c r="L451" t="n">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-22 19:53:23
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L470"/>
+  <dimension ref="A1:L480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19376,22 +19376,22 @@
         <v>46289</v>
       </c>
       <c r="G395" s="1" t="n">
-        <v>46303</v>
+        <v>46317</v>
       </c>
       <c r="H395" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="I395" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J395" t="n">
         <v>35</v>
       </c>
       <c r="K395" t="n">
-        <v>44.7</v>
+        <v>53.7</v>
       </c>
       <c r="L395" t="n">
-        <v>127.7</v>
+        <v>153.4</v>
       </c>
     </row>
     <row r="396">
@@ -19424,22 +19424,22 @@
         <v>46289</v>
       </c>
       <c r="G396" s="1" t="n">
-        <v>46303</v>
+        <v>46317</v>
       </c>
       <c r="H396" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="I396" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J396" t="n">
         <v>35</v>
       </c>
       <c r="K396" t="n">
-        <v>44.2</v>
+        <v>52.6</v>
       </c>
       <c r="L396" t="n">
-        <v>126.3</v>
+        <v>150.3</v>
       </c>
     </row>
     <row r="397">
@@ -19472,22 +19472,22 @@
         <v>46289</v>
       </c>
       <c r="G397" s="1" t="n">
-        <v>46296</v>
+        <v>46317</v>
       </c>
       <c r="H397" s="1" t="n">
-        <v>46301</v>
+        <v>46317</v>
       </c>
       <c r="I397" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J397" t="n">
         <v>35</v>
       </c>
       <c r="K397" t="n">
-        <v>35.7</v>
+        <v>52.9</v>
       </c>
       <c r="L397" t="n">
-        <v>102</v>
+        <v>151.1</v>
       </c>
     </row>
     <row r="398">
@@ -19520,22 +19520,22 @@
         <v>46289</v>
       </c>
       <c r="G398" s="1" t="n">
-        <v>46296</v>
+        <v>46303</v>
       </c>
       <c r="H398" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I398" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J398" t="n">
         <v>35</v>
       </c>
       <c r="K398" t="n">
-        <v>36.9</v>
+        <v>44.7</v>
       </c>
       <c r="L398" t="n">
-        <v>105.4</v>
+        <v>127.7</v>
       </c>
     </row>
     <row r="399">
@@ -19546,7 +19546,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F399" s="1" t="n">
@@ -19580,10 +19580,10 @@
         <v>35</v>
       </c>
       <c r="K399" t="n">
-        <v>43.2</v>
+        <v>44.2</v>
       </c>
       <c r="L399" t="n">
-        <v>123.4</v>
+        <v>126.3</v>
       </c>
     </row>
     <row r="400">
@@ -19594,7 +19594,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -19609,29 +19609,29 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F400" s="1" t="n">
         <v>46289</v>
       </c>
       <c r="G400" s="1" t="n">
-        <v>46303</v>
+        <v>46296</v>
       </c>
       <c r="H400" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I400" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J400" t="n">
         <v>35</v>
       </c>
       <c r="K400" t="n">
-        <v>43.9</v>
+        <v>35.7</v>
       </c>
       <c r="L400" t="n">
-        <v>125.4</v>
+        <v>102</v>
       </c>
     </row>
     <row r="401">
@@ -19642,7 +19642,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>P55</t>
+          <t>P54</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -19657,7 +19657,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Pilote 65 torre 2 tipo 2</t>
+          <t>Pilote 67 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F401" s="1" t="n">
@@ -19676,10 +19676,10 @@
         <v>35</v>
       </c>
       <c r="K401" t="n">
-        <v>36.5</v>
+        <v>36.9</v>
       </c>
       <c r="L401" t="n">
-        <v>104.3</v>
+        <v>105.4</v>
       </c>
     </row>
     <row r="402">
@@ -19712,22 +19712,22 @@
         <v>46289</v>
       </c>
       <c r="G402" s="1" t="n">
-        <v>46296</v>
+        <v>46317</v>
       </c>
       <c r="H402" s="1" t="n">
-        <v>46301</v>
+        <v>46317</v>
       </c>
       <c r="I402" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J402" t="n">
         <v>35</v>
       </c>
       <c r="K402" t="n">
-        <v>37</v>
+        <v>52.8</v>
       </c>
       <c r="L402" t="n">
-        <v>105.7</v>
+        <v>150.9</v>
       </c>
     </row>
     <row r="403">
@@ -19738,7 +19738,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -19753,29 +19753,29 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F403" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G403" s="1" t="n">
-        <v>46304</v>
+        <v>46317</v>
       </c>
       <c r="H403" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="I403" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J403" t="n">
         <v>35</v>
       </c>
       <c r="K403" t="n">
-        <v>51.1</v>
+        <v>53.9</v>
       </c>
       <c r="L403" t="n">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="404">
@@ -19786,7 +19786,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -19801,29 +19801,29 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F404" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G404" s="1" t="n">
-        <v>46304</v>
+        <v>46317</v>
       </c>
       <c r="H404" s="1" t="n">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="I404" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J404" t="n">
         <v>35</v>
       </c>
       <c r="K404" t="n">
-        <v>52.8</v>
+        <v>53.5</v>
       </c>
       <c r="L404" t="n">
-        <v>150.9</v>
+        <v>152.9</v>
       </c>
     </row>
     <row r="405">
@@ -19834,7 +19834,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -19849,29 +19849,29 @@
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F405" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G405" s="1" t="n">
-        <v>46297</v>
+        <v>46303</v>
       </c>
       <c r="H405" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I405" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J405" t="n">
         <v>35</v>
       </c>
       <c r="K405" t="n">
-        <v>42.8</v>
+        <v>43.2</v>
       </c>
       <c r="L405" t="n">
-        <v>122.3</v>
+        <v>123.4</v>
       </c>
     </row>
     <row r="406">
@@ -19882,7 +19882,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>P56</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -19897,29 +19897,29 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Pilote 76 torre 2 tipo 2</t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F406" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G406" s="1" t="n">
-        <v>46297</v>
+        <v>46303</v>
       </c>
       <c r="H406" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I406" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J406" t="n">
         <v>35</v>
       </c>
       <c r="K406" t="n">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
       <c r="L406" t="n">
-        <v>124.3</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="407">
@@ -19930,12 +19930,12 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -19945,29 +19945,29 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F407" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G407" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H407" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I407" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J407" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K407" t="n">
-        <v>33.6</v>
+        <v>36.5</v>
       </c>
       <c r="L407" t="n">
-        <v>137.1</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="408">
@@ -19978,12 +19978,12 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P55</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -19993,29 +19993,29 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 65 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F408" s="1" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="G408" s="1" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="H408" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I408" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J408" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K408" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="L408" t="n">
-        <v>134.7</v>
+        <v>105.7</v>
       </c>
     </row>
     <row r="409">
@@ -20026,12 +20026,12 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
@@ -20041,29 +20041,29 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F409" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="G409" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="H409" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I409" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J409" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K409" t="n">
-        <v>27.8</v>
+        <v>51.1</v>
       </c>
       <c r="L409" t="n">
-        <v>113.5</v>
+        <v>146</v>
       </c>
     </row>
     <row r="410">
@@ -20074,12 +20074,12 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -20089,29 +20089,29 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F410" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="G410" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="H410" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I410" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J410" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K410" t="n">
-        <v>28.1</v>
+        <v>52.8</v>
       </c>
       <c r="L410" t="n">
-        <v>114.7</v>
+        <v>150.9</v>
       </c>
     </row>
     <row r="411">
@@ -20122,12 +20122,12 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
@@ -20137,29 +20137,29 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F411" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G411" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H411" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I411" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J411" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K411" t="n">
-        <v>34.8</v>
+        <v>42.8</v>
       </c>
       <c r="L411" t="n">
-        <v>142</v>
+        <v>122.3</v>
       </c>
     </row>
     <row r="412">
@@ -20170,12 +20170,12 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
@@ -20185,29 +20185,29 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F412" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G412" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H412" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I412" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J412" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K412" t="n">
-        <v>35.8</v>
+        <v>43.5</v>
       </c>
       <c r="L412" t="n">
-        <v>146.1</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="413">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -20233,29 +20233,29 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F413" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G413" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H413" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I413" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J413" t="n">
         <v>24.5</v>
       </c>
       <c r="K413" t="n">
-        <v>28.9</v>
+        <v>33.6</v>
       </c>
       <c r="L413" t="n">
-        <v>118</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="414">
@@ -20266,7 +20266,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -20281,29 +20281,29 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F414" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G414" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H414" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I414" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J414" t="n">
         <v>24.5</v>
       </c>
       <c r="K414" t="n">
-        <v>29.4</v>
+        <v>33</v>
       </c>
       <c r="L414" t="n">
-        <v>120</v>
+        <v>134.7</v>
       </c>
     </row>
     <row r="415">
@@ -20314,7 +20314,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -20329,29 +20329,29 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F415" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G415" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H415" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I415" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J415" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K415" t="n">
-        <v>42.6</v>
+        <v>27.8</v>
       </c>
       <c r="L415" t="n">
-        <v>121.7</v>
+        <v>113.5</v>
       </c>
     </row>
     <row r="416">
@@ -20362,7 +20362,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -20377,29 +20377,29 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F416" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G416" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H416" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I416" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J416" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K416" t="n">
-        <v>43.5</v>
+        <v>28.1</v>
       </c>
       <c r="L416" t="n">
-        <v>124.3</v>
+        <v>114.7</v>
       </c>
     </row>
     <row r="417">
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -20425,29 +20425,29 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F417" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G417" s="1" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="H417" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I417" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J417" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K417" t="n">
-        <v>36.4</v>
+        <v>34.8</v>
       </c>
       <c r="L417" t="n">
-        <v>104</v>
+        <v>142</v>
       </c>
     </row>
     <row r="418">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -20473,29 +20473,29 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F418" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G418" s="1" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="H418" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I418" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J418" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K418" t="n">
-        <v>35.2</v>
+        <v>35.8</v>
       </c>
       <c r="L418" t="n">
-        <v>100.6</v>
+        <v>146.1</v>
       </c>
     </row>
     <row r="419">
@@ -20506,12 +20506,12 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
@@ -20521,29 +20521,29 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F419" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G419" s="1" t="n">
-        <v>46307</v>
+        <v>46298</v>
       </c>
       <c r="H419" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I419" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J419" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K419" t="n">
-        <v>49</v>
+        <v>28.9</v>
       </c>
       <c r="L419" t="n">
-        <v>140</v>
+        <v>118</v>
       </c>
     </row>
     <row r="420">
@@ -20554,12 +20554,12 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
@@ -20569,29 +20569,29 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F420" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G420" s="1" t="n">
-        <v>46307</v>
+        <v>46298</v>
       </c>
       <c r="H420" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I420" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J420" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K420" t="n">
-        <v>47.9</v>
+        <v>29.4</v>
       </c>
       <c r="L420" t="n">
-        <v>136.9</v>
+        <v>120</v>
       </c>
     </row>
     <row r="421">
@@ -20602,12 +20602,12 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
@@ -20617,29 +20617,29 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F421" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G421" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="H421" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I421" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J421" t="n">
         <v>35</v>
       </c>
       <c r="K421" t="n">
-        <v>41.4</v>
+        <v>42.6</v>
       </c>
       <c r="L421" t="n">
-        <v>118.3</v>
+        <v>121.7</v>
       </c>
     </row>
     <row r="422">
@@ -20650,12 +20650,12 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
@@ -20665,29 +20665,29 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F422" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G422" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="H422" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I422" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J422" t="n">
         <v>35</v>
       </c>
       <c r="K422" t="n">
-        <v>40.3</v>
+        <v>43.5</v>
       </c>
       <c r="L422" t="n">
-        <v>115.1</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="423">
@@ -20698,12 +20698,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -20713,29 +20713,29 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F423" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G423" s="1" t="n">
-        <v>46308</v>
+        <v>46298</v>
       </c>
       <c r="H423" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I423" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J423" t="n">
         <v>35</v>
       </c>
       <c r="K423" t="n">
-        <v>44.3</v>
+        <v>36.4</v>
       </c>
       <c r="L423" t="n">
-        <v>126.6</v>
+        <v>104</v>
       </c>
     </row>
     <row r="424">
@@ -20746,12 +20746,12 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
@@ -20761,29 +20761,29 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F424" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G424" s="1" t="n">
-        <v>46308</v>
+        <v>46298</v>
       </c>
       <c r="H424" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I424" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J424" t="n">
         <v>35</v>
       </c>
       <c r="K424" t="n">
-        <v>44.9</v>
+        <v>35.2</v>
       </c>
       <c r="L424" t="n">
-        <v>128.3</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="425">
@@ -20794,7 +20794,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -20809,29 +20809,29 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F425" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G425" s="1" t="n">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="H425" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I425" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J425" t="n">
         <v>35</v>
       </c>
       <c r="K425" t="n">
-        <v>37.5</v>
+        <v>49</v>
       </c>
       <c r="L425" t="n">
-        <v>107.1</v>
+        <v>140</v>
       </c>
     </row>
     <row r="426">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -20857,29 +20857,29 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F426" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G426" s="1" t="n">
-        <v>46301</v>
+        <v>46307</v>
       </c>
       <c r="H426" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I426" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J426" t="n">
         <v>35</v>
       </c>
       <c r="K426" t="n">
-        <v>36.4</v>
+        <v>47.9</v>
       </c>
       <c r="L426" t="n">
-        <v>104</v>
+        <v>136.9</v>
       </c>
     </row>
     <row r="427">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -20905,29 +20905,29 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F427" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G427" s="1" t="n">
-        <v>46308</v>
+        <v>46300</v>
       </c>
       <c r="H427" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I427" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J427" t="n">
         <v>35</v>
       </c>
       <c r="K427" t="n">
-        <v>43.9</v>
+        <v>41.4</v>
       </c>
       <c r="L427" t="n">
-        <v>125.4</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="428">
@@ -20938,7 +20938,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -20953,29 +20953,29 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F428" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G428" s="1" t="n">
-        <v>46308</v>
+        <v>46300</v>
       </c>
       <c r="H428" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I428" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J428" t="n">
         <v>35</v>
       </c>
       <c r="K428" t="n">
-        <v>43.7</v>
+        <v>40.3</v>
       </c>
       <c r="L428" t="n">
-        <v>124.9</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="429">
@@ -20986,7 +20986,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -21001,29 +21001,29 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F429" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="G429" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H429" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I429" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J429" t="n">
         <v>35</v>
       </c>
       <c r="K429" t="n">
-        <v>38.5</v>
+        <v>44.3</v>
       </c>
       <c r="L429" t="n">
-        <v>110</v>
+        <v>126.6</v>
       </c>
     </row>
     <row r="430">
@@ -21034,7 +21034,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -21049,29 +21049,29 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F430" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="G430" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H430" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I430" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J430" t="n">
         <v>35</v>
       </c>
       <c r="K430" t="n">
-        <v>37.1</v>
+        <v>44.9</v>
       </c>
       <c r="L430" t="n">
-        <v>106</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="431">
@@ -21082,12 +21082,12 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -21097,29 +21097,29 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F431" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G431" s="1" t="n">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="H431" s="1" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="I431" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J431" t="n">
         <v>35</v>
       </c>
       <c r="K431" t="n">
-        <v>33.5</v>
+        <v>37.5</v>
       </c>
       <c r="L431" t="n">
-        <v>95.7</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="432">
@@ -21130,12 +21130,12 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
@@ -21145,29 +21145,29 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F432" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G432" s="1" t="n">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="H432" s="1" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="I432" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J432" t="n">
         <v>35</v>
       </c>
       <c r="K432" t="n">
-        <v>32</v>
+        <v>36.4</v>
       </c>
       <c r="L432" t="n">
-        <v>91.40000000000001</v>
+        <v>104</v>
       </c>
     </row>
     <row r="433">
@@ -21178,12 +21178,12 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -21193,29 +21193,29 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F433" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G433" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H433" s="1" t="n">
         <v>46309</v>
       </c>
       <c r="I433" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J433" t="n">
         <v>35</v>
       </c>
       <c r="K433" t="n">
-        <v>24.4</v>
+        <v>43.9</v>
       </c>
       <c r="L433" t="n">
-        <v>69.7</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="434">
@@ -21226,12 +21226,12 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
@@ -21241,29 +21241,29 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F434" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G434" s="1" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="H434" s="1" t="n">
         <v>46309</v>
       </c>
       <c r="I434" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J434" t="n">
         <v>35</v>
       </c>
       <c r="K434" t="n">
-        <v>24.6</v>
+        <v>43.7</v>
       </c>
       <c r="L434" t="n">
-        <v>70.3</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="435">
@@ -21274,12 +21274,12 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -21289,29 +21289,29 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F435" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G435" s="1" t="n">
-        <v>46312</v>
+        <v>46301</v>
       </c>
       <c r="H435" s="1" t="n">
-        <v>46315</v>
+        <v>46302</v>
       </c>
       <c r="I435" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J435" t="n">
         <v>35</v>
       </c>
       <c r="K435" t="n">
-        <v>35.4</v>
+        <v>38.5</v>
       </c>
       <c r="L435" t="n">
-        <v>101.1</v>
+        <v>110</v>
       </c>
     </row>
     <row r="436">
@@ -21322,12 +21322,12 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
@@ -21337,29 +21337,29 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F436" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G436" s="1" t="n">
-        <v>46312</v>
+        <v>46301</v>
       </c>
       <c r="H436" s="1" t="n">
-        <v>46315</v>
+        <v>46302</v>
       </c>
       <c r="I436" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J436" t="n">
         <v>35</v>
       </c>
       <c r="K436" t="n">
-        <v>35.8</v>
+        <v>37.1</v>
       </c>
       <c r="L436" t="n">
-        <v>102.3</v>
+        <v>106</v>
       </c>
     </row>
     <row r="437">
@@ -21370,7 +21370,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -21385,29 +21385,29 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F437" s="1" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="G437" s="1" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="H437" s="1" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I437" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J437" t="n">
         <v>35</v>
       </c>
       <c r="K437" t="n">
-        <v>22.8</v>
+        <v>33.5</v>
       </c>
       <c r="L437" t="n">
-        <v>65.09999999999999</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="438">
@@ -21418,7 +21418,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -21433,29 +21433,29 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F438" s="1" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="G438" s="1" t="n">
-        <v>46305</v>
+        <v>46311</v>
       </c>
       <c r="H438" s="1" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I438" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J438" t="n">
         <v>35</v>
       </c>
       <c r="K438" t="n">
-        <v>23.3</v>
+        <v>32</v>
       </c>
       <c r="L438" t="n">
-        <v>66.59999999999999</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="439">
@@ -21466,7 +21466,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -21481,29 +21481,29 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F439" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G439" s="1" t="n">
-        <v>46314</v>
+        <v>46304</v>
       </c>
       <c r="H439" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I439" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J439" t="n">
         <v>35</v>
       </c>
       <c r="K439" t="n">
-        <v>37.8</v>
+        <v>24.4</v>
       </c>
       <c r="L439" t="n">
-        <v>108</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="440">
@@ -21514,7 +21514,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -21529,29 +21529,29 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F440" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G440" s="1" t="n">
-        <v>46314</v>
+        <v>46304</v>
       </c>
       <c r="H440" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I440" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J440" t="n">
         <v>35</v>
       </c>
       <c r="K440" t="n">
-        <v>38.9</v>
+        <v>24.6</v>
       </c>
       <c r="L440" t="n">
-        <v>111.1</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="441">
@@ -21562,7 +21562,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -21577,29 +21577,29 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F441" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G441" s="1" t="n">
-        <v>46307</v>
+        <v>46312</v>
       </c>
       <c r="H441" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I441" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J441" t="n">
         <v>35</v>
       </c>
       <c r="K441" t="n">
-        <v>34.3</v>
+        <v>35.4</v>
       </c>
       <c r="L441" t="n">
-        <v>98</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="442">
@@ -21610,7 +21610,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -21625,29 +21625,29 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F442" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G442" s="1" t="n">
-        <v>46307</v>
+        <v>46312</v>
       </c>
       <c r="H442" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I442" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J442" t="n">
         <v>35</v>
       </c>
       <c r="K442" t="n">
-        <v>34.7</v>
+        <v>35.8</v>
       </c>
       <c r="L442" t="n">
-        <v>99.09999999999999</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="443">
@@ -21658,7 +21658,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -21673,29 +21673,29 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F443" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G443" s="1" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="H443" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I443" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J443" t="n">
         <v>35</v>
       </c>
       <c r="K443" t="n">
-        <v>38.8</v>
+        <v>22.8</v>
       </c>
       <c r="L443" t="n">
-        <v>110.9</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="444">
@@ -21706,7 +21706,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
@@ -21721,29 +21721,29 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F444" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G444" s="1" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="H444" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I444" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J444" t="n">
         <v>35</v>
       </c>
       <c r="K444" t="n">
-        <v>38.3</v>
+        <v>23.3</v>
       </c>
       <c r="L444" t="n">
-        <v>109.4</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="445">
@@ -21754,7 +21754,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -21769,29 +21769,29 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F445" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="G445" s="1" t="n">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="H445" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I445" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J445" t="n">
         <v>35</v>
       </c>
       <c r="K445" t="n">
-        <v>33.4</v>
+        <v>37.8</v>
       </c>
       <c r="L445" t="n">
-        <v>95.40000000000001</v>
+        <v>108</v>
       </c>
     </row>
     <row r="446">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -21817,29 +21817,29 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F446" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="G446" s="1" t="n">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="H446" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I446" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J446" t="n">
         <v>35</v>
       </c>
       <c r="K446" t="n">
-        <v>32.4</v>
+        <v>38.9</v>
       </c>
       <c r="L446" t="n">
-        <v>92.59999999999999</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="447">
@@ -21850,7 +21850,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -21865,29 +21865,29 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F447" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G447" s="1" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="H447" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I447" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J447" t="n">
         <v>35</v>
       </c>
       <c r="K447" t="n">
-        <v>45.8</v>
+        <v>34.3</v>
       </c>
       <c r="L447" t="n">
-        <v>130.9</v>
+        <v>98</v>
       </c>
     </row>
     <row r="448">
@@ -21898,7 +21898,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -21913,29 +21913,29 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F448" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G448" s="1" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="H448" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I448" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J448" t="n">
         <v>35</v>
       </c>
       <c r="K448" t="n">
-        <v>47</v>
+        <v>34.7</v>
       </c>
       <c r="L448" t="n">
-        <v>134.3</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="449">
@@ -21946,7 +21946,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -21961,29 +21961,29 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F449" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G449" s="1" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="H449" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I449" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J449" t="n">
         <v>35</v>
       </c>
       <c r="K449" t="n">
-        <v>37.9</v>
+        <v>38.8</v>
       </c>
       <c r="L449" t="n">
-        <v>108.3</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="450">
@@ -21994,7 +21994,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -22009,29 +22009,29 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F450" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G450" s="1" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="H450" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I450" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J450" t="n">
         <v>35</v>
       </c>
       <c r="K450" t="n">
-        <v>38.4</v>
+        <v>38.3</v>
       </c>
       <c r="L450" t="n">
-        <v>109.7</v>
+        <v>109.4</v>
       </c>
     </row>
     <row r="451">
@@ -22042,7 +22042,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -22057,29 +22057,29 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F451" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G451" s="1" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="H451" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I451" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J451" t="n">
         <v>35</v>
       </c>
       <c r="K451" t="n">
-        <v>46.3</v>
+        <v>33.4</v>
       </c>
       <c r="L451" t="n">
-        <v>132.3</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="452">
@@ -22090,7 +22090,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -22105,29 +22105,29 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F452" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G452" s="1" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="H452" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I452" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J452" t="n">
         <v>35</v>
       </c>
       <c r="K452" t="n">
-        <v>45.7</v>
+        <v>32.4</v>
       </c>
       <c r="L452" t="n">
-        <v>130.6</v>
+        <v>92.59999999999999</v>
       </c>
     </row>
     <row r="453">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -22153,29 +22153,29 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F453" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="G453" s="1" t="n">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="H453" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="I453" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J453" t="n">
         <v>35</v>
       </c>
       <c r="K453" t="n">
-        <v>38.9</v>
+        <v>45.8</v>
       </c>
       <c r="L453" t="n">
-        <v>111.1</v>
+        <v>130.9</v>
       </c>
     </row>
     <row r="454">
@@ -22186,7 +22186,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -22201,29 +22201,29 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F454" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="G454" s="1" t="n">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="H454" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="I454" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J454" t="n">
         <v>35</v>
       </c>
       <c r="K454" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="L454" t="n">
-        <v>108.6</v>
+        <v>134.3</v>
       </c>
     </row>
     <row r="455">
@@ -22234,12 +22234,12 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
@@ -22249,29 +22249,29 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F455" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G455" s="1" t="n">
-        <v>46316</v>
+        <v>46308</v>
       </c>
       <c r="H455" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I455" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J455" t="n">
         <v>35</v>
       </c>
       <c r="K455" t="n">
-        <v>48</v>
+        <v>37.9</v>
       </c>
       <c r="L455" t="n">
-        <v>137.1</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="456">
@@ -22282,12 +22282,12 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
@@ -22297,29 +22297,29 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F456" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G456" s="1" t="n">
-        <v>46316</v>
+        <v>46308</v>
       </c>
       <c r="H456" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I456" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J456" t="n">
         <v>35</v>
       </c>
       <c r="K456" t="n">
-        <v>48.7</v>
+        <v>38.4</v>
       </c>
       <c r="L456" t="n">
-        <v>139.1</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="457">
@@ -22330,12 +22330,12 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
@@ -22345,29 +22345,29 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F457" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G457" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="H457" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I457" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J457" t="n">
         <v>35</v>
       </c>
       <c r="K457" t="n">
-        <v>41.2</v>
+        <v>46.3</v>
       </c>
       <c r="L457" t="n">
-        <v>117.7</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="458">
@@ -22378,12 +22378,12 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -22393,29 +22393,29 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F458" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G458" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="H458" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I458" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J458" t="n">
         <v>35</v>
       </c>
       <c r="K458" t="n">
-        <v>41.7</v>
+        <v>45.7</v>
       </c>
       <c r="L458" t="n">
-        <v>119.1</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="459">
@@ -22426,12 +22426,12 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -22441,29 +22441,29 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F459" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G459" s="1" t="n">
-        <v>46316</v>
+        <v>46308</v>
       </c>
       <c r="H459" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I459" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J459" t="n">
         <v>35</v>
       </c>
       <c r="K459" t="n">
-        <v>39.8</v>
+        <v>38.9</v>
       </c>
       <c r="L459" t="n">
-        <v>113.7</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="460">
@@ -22474,12 +22474,12 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -22489,29 +22489,29 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F460" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G460" s="1" t="n">
-        <v>46316</v>
+        <v>46308</v>
       </c>
       <c r="H460" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I460" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J460" t="n">
         <v>35</v>
       </c>
       <c r="K460" t="n">
-        <v>38.2</v>
+        <v>38</v>
       </c>
       <c r="L460" t="n">
-        <v>109.1</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="461">
@@ -22522,7 +22522,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -22537,29 +22537,29 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F461" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="G461" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="H461" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I461" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J461" t="n">
         <v>35</v>
       </c>
       <c r="K461" t="n">
-        <v>32.8</v>
+        <v>48</v>
       </c>
       <c r="L461" t="n">
-        <v>93.7</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="462">
@@ -22570,7 +22570,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -22585,29 +22585,29 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F462" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="G462" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="H462" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I462" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J462" t="n">
         <v>35</v>
       </c>
       <c r="K462" t="n">
-        <v>31.8</v>
+        <v>48.7</v>
       </c>
       <c r="L462" t="n">
-        <v>90.90000000000001</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="463">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -22633,14 +22633,14 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F463" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G463" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H463" s="1" t="n">
         <v>46310</v>
@@ -22652,10 +22652,10 @@
         <v>35</v>
       </c>
       <c r="K463" t="n">
-        <v>35.7</v>
+        <v>41.2</v>
       </c>
       <c r="L463" t="n">
-        <v>102</v>
+        <v>117.7</v>
       </c>
     </row>
     <row r="464">
@@ -22666,7 +22666,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -22681,14 +22681,14 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F464" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G464" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H464" s="1" t="n">
         <v>46310</v>
@@ -22700,10 +22700,10 @@
         <v>35</v>
       </c>
       <c r="K464" t="n">
-        <v>36.2</v>
+        <v>41.7</v>
       </c>
       <c r="L464" t="n">
-        <v>103.4</v>
+        <v>119.1</v>
       </c>
     </row>
     <row r="465">
@@ -22714,7 +22714,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -22729,29 +22729,29 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F465" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G465" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="H465" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I465" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J465" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K465" t="n">
-        <v>24.4</v>
+        <v>39.8</v>
       </c>
       <c r="L465" t="n">
-        <v>99.59999999999999</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="466">
@@ -22762,7 +22762,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -22777,29 +22777,29 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F466" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G466" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="H466" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I466" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J466" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K466" t="n">
-        <v>23.6</v>
+        <v>38.2</v>
       </c>
       <c r="L466" t="n">
-        <v>96.3</v>
+        <v>109.1</v>
       </c>
     </row>
     <row r="467">
@@ -22810,7 +22810,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -22825,17 +22825,17 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F467" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G467" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="H467" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="I467" t="n">
         <v>7</v>
@@ -22844,10 +22844,10 @@
         <v>35</v>
       </c>
       <c r="K467" t="n">
-        <v>34.6</v>
+        <v>32.8</v>
       </c>
       <c r="L467" t="n">
-        <v>98.90000000000001</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="468">
@@ -22858,7 +22858,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -22873,17 +22873,17 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F468" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G468" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="H468" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="I468" t="n">
         <v>7</v>
@@ -22892,10 +22892,10 @@
         <v>35</v>
       </c>
       <c r="K468" t="n">
-        <v>34.7</v>
+        <v>31.8</v>
       </c>
       <c r="L468" t="n">
-        <v>99.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="469">
@@ -22906,12 +22906,12 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -22921,29 +22921,29 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F469" s="1" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="G469" s="1" t="n">
-        <v>46311</v>
+        <v>46317</v>
       </c>
       <c r="H469" s="1" t="n">
-        <v>46311</v>
+        <v>46317</v>
       </c>
       <c r="I469" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J469" t="n">
         <v>35</v>
       </c>
       <c r="K469" t="n">
-        <v>32.5</v>
+        <v>43.2</v>
       </c>
       <c r="L469" t="n">
-        <v>92.90000000000001</v>
+        <v>123.4</v>
       </c>
     </row>
     <row r="470">
@@ -22954,43 +22954,523 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F470" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G470" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H470" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I470" t="n">
+        <v>14</v>
+      </c>
+      <c r="J470" t="n">
+        <v>35</v>
+      </c>
+      <c r="K470" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="L470" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F471" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G471" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H471" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I471" t="n">
+        <v>7</v>
+      </c>
+      <c r="J471" t="n">
+        <v>35</v>
+      </c>
+      <c r="K471" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="L471" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>P76</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F472" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G472" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H472" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I472" t="n">
+        <v>7</v>
+      </c>
+      <c r="J472" t="n">
+        <v>35</v>
+      </c>
+      <c r="K472" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="L472" t="n">
+        <v>103.4</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F473" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G473" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H473" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I473" t="n">
+        <v>14</v>
+      </c>
+      <c r="J473" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K473" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="L473" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F474" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G474" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H474" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I474" t="n">
+        <v>14</v>
+      </c>
+      <c r="J474" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K474" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="L474" t="n">
+        <v>117.6</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F475" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G475" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H475" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I475" t="n">
+        <v>7</v>
+      </c>
+      <c r="J475" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K475" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="L475" t="n">
+        <v>99.59999999999999</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>P77</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Pilote 111 salón comunal</t>
+        </is>
+      </c>
+      <c r="F476" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G476" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H476" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I476" t="n">
+        <v>7</v>
+      </c>
+      <c r="J476" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="K476" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L476" t="n">
+        <v>96.3</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>P78</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F477" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G477" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H477" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I477" t="n">
+        <v>7</v>
+      </c>
+      <c r="J477" t="n">
+        <v>35</v>
+      </c>
+      <c r="K477" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="L477" t="n">
+        <v>98.90000000000001</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>P78</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F478" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G478" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H478" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I478" t="n">
+        <v>7</v>
+      </c>
+      <c r="J478" t="n">
+        <v>35</v>
+      </c>
+      <c r="K478" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="L478" t="n">
+        <v>99.09999999999999</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
           <t>P79</t>
         </is>
       </c>
-      <c r="C470" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No especificado </t>
-        </is>
-      </c>
-      <c r="D470" t="inlineStr">
-        <is>
-          <t>Concreto</t>
-        </is>
-      </c>
-      <c r="E470" t="inlineStr">
+      <c r="C479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
         </is>
       </c>
-      <c r="F470" s="1" t="n">
+      <c r="F479" s="1" t="n">
         <v>46304</v>
       </c>
-      <c r="G470" s="1" t="n">
+      <c r="G479" s="1" t="n">
         <v>46311</v>
       </c>
-      <c r="H470" s="1" t="n">
+      <c r="H479" s="1" t="n">
         <v>46311</v>
       </c>
-      <c r="I470" t="n">
+      <c r="I479" t="n">
         <v>7</v>
       </c>
-      <c r="J470" t="n">
-        <v>35</v>
-      </c>
-      <c r="K470" t="n">
+      <c r="J479" t="n">
+        <v>35</v>
+      </c>
+      <c r="K479" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="L479" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F480" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G480" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H480" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I480" t="n">
+        <v>7</v>
+      </c>
+      <c r="J480" t="n">
+        <v>35</v>
+      </c>
+      <c r="K480" t="n">
         <v>32.2</v>
       </c>
-      <c r="L470" t="n">
+      <c r="L480" t="n">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-23 19:52:01
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L480"/>
+  <dimension ref="A1:L491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23474,6 +23474,534 @@
         <v>92</v>
       </c>
     </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F481" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G481" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H481" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I481" t="n">
+        <v>7</v>
+      </c>
+      <c r="J481" t="n">
+        <v>35</v>
+      </c>
+      <c r="K481" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L481" t="n">
+        <v>121.4</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F482" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G482" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H482" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I482" t="n">
+        <v>7</v>
+      </c>
+      <c r="J482" t="n">
+        <v>35</v>
+      </c>
+      <c r="K482" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="L482" t="n">
+        <v>119.7</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F483" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G483" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H483" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I483" t="n">
+        <v>7</v>
+      </c>
+      <c r="J483" t="n">
+        <v>35</v>
+      </c>
+      <c r="K483" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="L483" t="n">
+        <v>116.3</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>P82</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F484" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G484" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H484" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I484" t="n">
+        <v>7</v>
+      </c>
+      <c r="J484" t="n">
+        <v>35</v>
+      </c>
+      <c r="K484" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="L484" t="n">
+        <v>92.3</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>P82</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F485" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G485" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H485" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I485" t="n">
+        <v>7</v>
+      </c>
+      <c r="J485" t="n">
+        <v>35</v>
+      </c>
+      <c r="K485" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="L485" t="n">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>P83</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Pilote 103 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F486" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G486" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H486" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I486" t="n">
+        <v>7</v>
+      </c>
+      <c r="J486" t="n">
+        <v>35</v>
+      </c>
+      <c r="K486" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="L486" t="n">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>P83</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Pilote 103 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F487" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G487" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H487" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I487" t="n">
+        <v>7</v>
+      </c>
+      <c r="J487" t="n">
+        <v>35</v>
+      </c>
+      <c r="K487" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="L487" t="n">
+        <v>58.9</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>P84</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F488" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G488" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H488" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I488" t="n">
+        <v>7</v>
+      </c>
+      <c r="J488" t="n">
+        <v>35</v>
+      </c>
+      <c r="K488" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="L488" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>P84</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F489" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G489" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H489" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I489" t="n">
+        <v>7</v>
+      </c>
+      <c r="J489" t="n">
+        <v>35</v>
+      </c>
+      <c r="K489" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="L489" t="n">
+        <v>100.3</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>P85</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Pilote 73 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F490" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G490" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H490" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I490" t="n">
+        <v>7</v>
+      </c>
+      <c r="J490" t="n">
+        <v>35</v>
+      </c>
+      <c r="K490" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L490" t="n">
+        <v>121.4</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>P85</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Pilote 73 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F491" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G491" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H491" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I491" t="n">
+        <v>7</v>
+      </c>
+      <c r="J491" t="n">
+        <v>35</v>
+      </c>
+      <c r="K491" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="L491" t="n">
+        <v>118.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-26 19:59:33
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L491"/>
+  <dimension ref="A1:L513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20048,22 +20048,22 @@
         <v>46290</v>
       </c>
       <c r="G409" s="1" t="n">
-        <v>46304</v>
+        <v>46318</v>
       </c>
       <c r="H409" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I409" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J409" t="n">
         <v>35</v>
       </c>
       <c r="K409" t="n">
-        <v>51.1</v>
+        <v>61.9</v>
       </c>
       <c r="L409" t="n">
-        <v>146</v>
+        <v>176.9</v>
       </c>
     </row>
     <row r="410">
@@ -20096,22 +20096,22 @@
         <v>46290</v>
       </c>
       <c r="G410" s="1" t="n">
-        <v>46304</v>
+        <v>46318</v>
       </c>
       <c r="H410" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I410" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J410" t="n">
         <v>35</v>
       </c>
       <c r="K410" t="n">
-        <v>52.8</v>
+        <v>61.6</v>
       </c>
       <c r="L410" t="n">
-        <v>150.9</v>
+        <v>176</v>
       </c>
     </row>
     <row r="411">
@@ -20144,22 +20144,22 @@
         <v>46290</v>
       </c>
       <c r="G411" s="1" t="n">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="H411" s="1" t="n">
-        <v>46301</v>
+        <v>46321</v>
       </c>
       <c r="I411" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J411" t="n">
         <v>35</v>
       </c>
       <c r="K411" t="n">
-        <v>42.8</v>
+        <v>61</v>
       </c>
       <c r="L411" t="n">
-        <v>122.3</v>
+        <v>174.3</v>
       </c>
     </row>
     <row r="412">
@@ -20192,22 +20192,22 @@
         <v>46290</v>
       </c>
       <c r="G412" s="1" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="H412" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I412" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J412" t="n">
         <v>35</v>
       </c>
       <c r="K412" t="n">
-        <v>43.5</v>
+        <v>51.1</v>
       </c>
       <c r="L412" t="n">
-        <v>124.3</v>
+        <v>146</v>
       </c>
     </row>
     <row r="413">
@@ -20218,12 +20218,12 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
@@ -20233,7 +20233,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F413" s="1" t="n">
@@ -20249,13 +20249,13 @@
         <v>14</v>
       </c>
       <c r="J413" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K413" t="n">
-        <v>33.6</v>
+        <v>52.8</v>
       </c>
       <c r="L413" t="n">
-        <v>137.1</v>
+        <v>150.9</v>
       </c>
     </row>
     <row r="414">
@@ -20266,12 +20266,12 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
@@ -20281,29 +20281,29 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F414" s="1" t="n">
         <v>46290</v>
       </c>
       <c r="G414" s="1" t="n">
-        <v>46304</v>
+        <v>46297</v>
       </c>
       <c r="H414" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I414" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J414" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K414" t="n">
-        <v>33</v>
+        <v>42.8</v>
       </c>
       <c r="L414" t="n">
-        <v>134.7</v>
+        <v>122.3</v>
       </c>
     </row>
     <row r="415">
@@ -20314,12 +20314,12 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>P57</t>
+          <t>P56</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
@@ -20329,7 +20329,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
+          <t>Pilote 76 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F415" s="1" t="n">
@@ -20345,13 +20345,13 @@
         <v>7</v>
       </c>
       <c r="J415" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K415" t="n">
-        <v>27.8</v>
+        <v>43.5</v>
       </c>
       <c r="L415" t="n">
-        <v>113.5</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="416">
@@ -20384,22 +20384,22 @@
         <v>46290</v>
       </c>
       <c r="G416" s="1" t="n">
-        <v>46297</v>
+        <v>46318</v>
       </c>
       <c r="H416" s="1" t="n">
-        <v>46301</v>
+        <v>46321</v>
       </c>
       <c r="I416" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J416" t="n">
         <v>24.5</v>
       </c>
       <c r="K416" t="n">
-        <v>28.1</v>
+        <v>40.2</v>
       </c>
       <c r="L416" t="n">
-        <v>114.7</v>
+        <v>164.1</v>
       </c>
     </row>
     <row r="417">
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -20425,29 +20425,29 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F417" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G417" s="1" t="n">
-        <v>46305</v>
+        <v>46318</v>
       </c>
       <c r="H417" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I417" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J417" t="n">
         <v>24.5</v>
       </c>
       <c r="K417" t="n">
-        <v>34.8</v>
+        <v>39</v>
       </c>
       <c r="L417" t="n">
-        <v>142</v>
+        <v>159.2</v>
       </c>
     </row>
     <row r="418">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -20473,29 +20473,29 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F418" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G418" s="1" t="n">
-        <v>46305</v>
+        <v>46318</v>
       </c>
       <c r="H418" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I418" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J418" t="n">
         <v>24.5</v>
       </c>
       <c r="K418" t="n">
-        <v>35.8</v>
+        <v>38.8</v>
       </c>
       <c r="L418" t="n">
-        <v>146.1</v>
+        <v>158.4</v>
       </c>
     </row>
     <row r="419">
@@ -20506,7 +20506,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -20521,29 +20521,29 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F419" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G419" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H419" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I419" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J419" t="n">
         <v>24.5</v>
       </c>
       <c r="K419" t="n">
-        <v>28.9</v>
+        <v>33.6</v>
       </c>
       <c r="L419" t="n">
-        <v>118</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="420">
@@ -20554,7 +20554,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>P58</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -20569,29 +20569,29 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 141 salón comunal </t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F420" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G420" s="1" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="H420" s="1" t="n">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="I420" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J420" t="n">
         <v>24.5</v>
       </c>
       <c r="K420" t="n">
-        <v>29.4</v>
+        <v>33</v>
       </c>
       <c r="L420" t="n">
-        <v>120</v>
+        <v>134.7</v>
       </c>
     </row>
     <row r="421">
@@ -20602,7 +20602,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -20617,29 +20617,29 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F421" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G421" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H421" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I421" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J421" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K421" t="n">
-        <v>42.6</v>
+        <v>27.8</v>
       </c>
       <c r="L421" t="n">
-        <v>121.7</v>
+        <v>113.5</v>
       </c>
     </row>
     <row r="422">
@@ -20650,7 +20650,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P57</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -20665,29 +20665,29 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 117 - 110 - 137 salón comunal </t>
         </is>
       </c>
       <c r="F422" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="G422" s="1" t="n">
-        <v>46305</v>
+        <v>46297</v>
       </c>
       <c r="H422" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I422" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J422" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K422" t="n">
-        <v>43.5</v>
+        <v>28.1</v>
       </c>
       <c r="L422" t="n">
-        <v>124.3</v>
+        <v>114.7</v>
       </c>
     </row>
     <row r="423">
@@ -20698,7 +20698,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -20713,29 +20713,29 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F423" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G423" s="1" t="n">
-        <v>46298</v>
+        <v>46319</v>
       </c>
       <c r="H423" s="1" t="n">
-        <v>46301</v>
+        <v>46321</v>
       </c>
       <c r="I423" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J423" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K423" t="n">
-        <v>36.4</v>
+        <v>41.8</v>
       </c>
       <c r="L423" t="n">
-        <v>104</v>
+        <v>170.6</v>
       </c>
     </row>
     <row r="424">
@@ -20746,7 +20746,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>P59</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -20761,29 +20761,29 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Pilote 60 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F424" s="1" t="n">
         <v>46291</v>
       </c>
       <c r="G424" s="1" t="n">
-        <v>46298</v>
+        <v>46319</v>
       </c>
       <c r="H424" s="1" t="n">
-        <v>46301</v>
+        <v>46321</v>
       </c>
       <c r="I424" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J424" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K424" t="n">
-        <v>35.2</v>
+        <v>42</v>
       </c>
       <c r="L424" t="n">
-        <v>100.6</v>
+        <v>171.4</v>
       </c>
     </row>
     <row r="425">
@@ -20794,12 +20794,12 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
@@ -20809,29 +20809,29 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F425" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G425" s="1" t="n">
-        <v>46307</v>
+        <v>46319</v>
       </c>
       <c r="H425" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I425" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J425" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K425" t="n">
-        <v>49</v>
+        <v>41.4</v>
       </c>
       <c r="L425" t="n">
-        <v>140</v>
+        <v>169</v>
       </c>
     </row>
     <row r="426">
@@ -20842,12 +20842,12 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
@@ -20857,14 +20857,14 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F426" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G426" s="1" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="H426" s="1" t="n">
         <v>46309</v>
@@ -20873,13 +20873,13 @@
         <v>14</v>
       </c>
       <c r="J426" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K426" t="n">
-        <v>47.9</v>
+        <v>34.8</v>
       </c>
       <c r="L426" t="n">
-        <v>136.9</v>
+        <v>142</v>
       </c>
     </row>
     <row r="427">
@@ -20890,12 +20890,12 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
@@ -20905,29 +20905,29 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F427" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G427" s="1" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="H427" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I427" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J427" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K427" t="n">
-        <v>41.4</v>
+        <v>35.8</v>
       </c>
       <c r="L427" t="n">
-        <v>118.3</v>
+        <v>146.1</v>
       </c>
     </row>
     <row r="428">
@@ -20938,12 +20938,12 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>P60</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -20953,29 +20953,29 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Pilote 106 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F428" s="1" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="G428" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="H428" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="I428" t="n">
         <v>7</v>
       </c>
       <c r="J428" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K428" t="n">
-        <v>40.3</v>
+        <v>28.9</v>
       </c>
       <c r="L428" t="n">
-        <v>115.1</v>
+        <v>118</v>
       </c>
     </row>
     <row r="429">
@@ -20986,12 +20986,12 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P58</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -21001,29 +21001,29 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t xml:space="preserve">Pilote 141 salón comunal </t>
         </is>
       </c>
       <c r="F429" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G429" s="1" t="n">
-        <v>46308</v>
+        <v>46298</v>
       </c>
       <c r="H429" s="1" t="n">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="I429" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J429" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K429" t="n">
-        <v>44.3</v>
+        <v>29.4</v>
       </c>
       <c r="L429" t="n">
-        <v>126.6</v>
+        <v>120</v>
       </c>
     </row>
     <row r="430">
@@ -21034,12 +21034,12 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -21049,29 +21049,29 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F430" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G430" s="1" t="n">
-        <v>46308</v>
+        <v>46319</v>
       </c>
       <c r="H430" s="1" t="n">
-        <v>46309</v>
+        <v>46321</v>
       </c>
       <c r="I430" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J430" t="n">
         <v>35</v>
       </c>
       <c r="K430" t="n">
-        <v>44.9</v>
+        <v>51.7</v>
       </c>
       <c r="L430" t="n">
-        <v>128.3</v>
+        <v>147.7</v>
       </c>
     </row>
     <row r="431">
@@ -21082,12 +21082,12 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
@@ -21097,29 +21097,29 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F431" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G431" s="1" t="n">
-        <v>46301</v>
+        <v>46319</v>
       </c>
       <c r="H431" s="1" t="n">
-        <v>46302</v>
+        <v>46321</v>
       </c>
       <c r="I431" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J431" t="n">
         <v>35</v>
       </c>
       <c r="K431" t="n">
-        <v>37.5</v>
+        <v>51.3</v>
       </c>
       <c r="L431" t="n">
-        <v>107.1</v>
+        <v>146.6</v>
       </c>
     </row>
     <row r="432">
@@ -21130,12 +21130,12 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
@@ -21145,29 +21145,29 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F432" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G432" s="1" t="n">
-        <v>46301</v>
+        <v>46319</v>
       </c>
       <c r="H432" s="1" t="n">
-        <v>46302</v>
+        <v>46321</v>
       </c>
       <c r="I432" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J432" t="n">
         <v>35</v>
       </c>
       <c r="K432" t="n">
-        <v>36.4</v>
+        <v>53.4</v>
       </c>
       <c r="L432" t="n">
-        <v>104</v>
+        <v>152.6</v>
       </c>
     </row>
     <row r="433">
@@ -21178,12 +21178,12 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
@@ -21193,14 +21193,14 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F433" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G433" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H433" s="1" t="n">
         <v>46309</v>
@@ -21212,10 +21212,10 @@
         <v>35</v>
       </c>
       <c r="K433" t="n">
-        <v>43.9</v>
+        <v>42.6</v>
       </c>
       <c r="L433" t="n">
-        <v>125.4</v>
+        <v>121.7</v>
       </c>
     </row>
     <row r="434">
@@ -21226,12 +21226,12 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
@@ -21241,14 +21241,14 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F434" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G434" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H434" s="1" t="n">
         <v>46309</v>
@@ -21260,10 +21260,10 @@
         <v>35</v>
       </c>
       <c r="K434" t="n">
-        <v>43.7</v>
+        <v>43.5</v>
       </c>
       <c r="L434" t="n">
-        <v>124.9</v>
+        <v>124.3</v>
       </c>
     </row>
     <row r="435">
@@ -21274,12 +21274,12 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -21289,17 +21289,17 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F435" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G435" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H435" s="1" t="n">
         <v>46301</v>
-      </c>
-      <c r="H435" s="1" t="n">
-        <v>46302</v>
       </c>
       <c r="I435" t="n">
         <v>7</v>
@@ -21308,10 +21308,10 @@
         <v>35</v>
       </c>
       <c r="K435" t="n">
-        <v>38.5</v>
+        <v>36.4</v>
       </c>
       <c r="L435" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="436">
@@ -21322,12 +21322,12 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P59</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>No Especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
@@ -21337,17 +21337,17 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 60 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F436" s="1" t="n">
-        <v>46294</v>
+        <v>46291</v>
       </c>
       <c r="G436" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H436" s="1" t="n">
         <v>46301</v>
-      </c>
-      <c r="H436" s="1" t="n">
-        <v>46302</v>
       </c>
       <c r="I436" t="n">
         <v>7</v>
@@ -21356,10 +21356,10 @@
         <v>35</v>
       </c>
       <c r="K436" t="n">
-        <v>37.1</v>
+        <v>35.2</v>
       </c>
       <c r="L436" t="n">
-        <v>106</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="437">
@@ -21370,12 +21370,12 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -21385,17 +21385,17 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F437" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="G437" s="1" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="H437" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I437" t="n">
         <v>14</v>
@@ -21404,10 +21404,10 @@
         <v>35</v>
       </c>
       <c r="K437" t="n">
-        <v>33.5</v>
+        <v>49</v>
       </c>
       <c r="L437" t="n">
-        <v>95.7</v>
+        <v>140</v>
       </c>
     </row>
     <row r="438">
@@ -21418,12 +21418,12 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
@@ -21433,17 +21433,17 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F438" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="G438" s="1" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="H438" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I438" t="n">
         <v>14</v>
@@ -21452,10 +21452,10 @@
         <v>35</v>
       </c>
       <c r="K438" t="n">
-        <v>32</v>
+        <v>47.9</v>
       </c>
       <c r="L438" t="n">
-        <v>91.40000000000001</v>
+        <v>136.9</v>
       </c>
     </row>
     <row r="439">
@@ -21466,12 +21466,12 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
@@ -21481,17 +21481,17 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F439" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="G439" s="1" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="H439" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I439" t="n">
         <v>7</v>
@@ -21500,10 +21500,10 @@
         <v>35</v>
       </c>
       <c r="K439" t="n">
-        <v>24.4</v>
+        <v>41.4</v>
       </c>
       <c r="L439" t="n">
-        <v>69.7</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="440">
@@ -21514,12 +21514,12 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
@@ -21529,17 +21529,17 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F440" s="1" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="G440" s="1" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="H440" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I440" t="n">
         <v>7</v>
@@ -21548,10 +21548,10 @@
         <v>35</v>
       </c>
       <c r="K440" t="n">
-        <v>24.6</v>
+        <v>40.3</v>
       </c>
       <c r="L440" t="n">
-        <v>70.3</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="441">
@@ -21562,12 +21562,12 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
@@ -21577,17 +21577,17 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F441" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G441" s="1" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="H441" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I441" t="n">
         <v>14</v>
@@ -21596,10 +21596,10 @@
         <v>35</v>
       </c>
       <c r="K441" t="n">
-        <v>35.4</v>
+        <v>44.3</v>
       </c>
       <c r="L441" t="n">
-        <v>101.1</v>
+        <v>126.6</v>
       </c>
     </row>
     <row r="442">
@@ -21610,12 +21610,12 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
@@ -21625,17 +21625,17 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F442" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G442" s="1" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="H442" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I442" t="n">
         <v>14</v>
@@ -21644,10 +21644,10 @@
         <v>35</v>
       </c>
       <c r="K442" t="n">
-        <v>35.8</v>
+        <v>44.9</v>
       </c>
       <c r="L442" t="n">
-        <v>102.3</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="443">
@@ -21658,12 +21658,12 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
@@ -21673,17 +21673,17 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F443" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G443" s="1" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="H443" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I443" t="n">
         <v>7</v>
@@ -21692,10 +21692,10 @@
         <v>35</v>
       </c>
       <c r="K443" t="n">
-        <v>22.8</v>
+        <v>37.5</v>
       </c>
       <c r="L443" t="n">
-        <v>65.09999999999999</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="444">
@@ -21706,12 +21706,12 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
@@ -21721,17 +21721,17 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F444" s="1" t="n">
-        <v>46298</v>
+        <v>46294</v>
       </c>
       <c r="G444" s="1" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="H444" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I444" t="n">
         <v>7</v>
@@ -21740,10 +21740,10 @@
         <v>35</v>
       </c>
       <c r="K444" t="n">
-        <v>23.3</v>
+        <v>36.4</v>
       </c>
       <c r="L444" t="n">
-        <v>66.59999999999999</v>
+        <v>104</v>
       </c>
     </row>
     <row r="445">
@@ -21754,12 +21754,12 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
@@ -21769,17 +21769,17 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F445" s="1" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="G445" s="1" t="n">
-        <v>46314</v>
+        <v>46308</v>
       </c>
       <c r="H445" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I445" t="n">
         <v>14</v>
@@ -21788,10 +21788,10 @@
         <v>35</v>
       </c>
       <c r="K445" t="n">
-        <v>37.8</v>
+        <v>43.9</v>
       </c>
       <c r="L445" t="n">
-        <v>108</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="446">
@@ -21802,12 +21802,12 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
@@ -21817,17 +21817,17 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F446" s="1" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="G446" s="1" t="n">
-        <v>46314</v>
+        <v>46308</v>
       </c>
       <c r="H446" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I446" t="n">
         <v>14</v>
@@ -21836,10 +21836,10 @@
         <v>35</v>
       </c>
       <c r="K446" t="n">
-        <v>38.9</v>
+        <v>43.7</v>
       </c>
       <c r="L446" t="n">
-        <v>111.1</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="447">
@@ -21850,12 +21850,12 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
@@ -21865,17 +21865,17 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F447" s="1" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="G447" s="1" t="n">
-        <v>46307</v>
+        <v>46301</v>
       </c>
       <c r="H447" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I447" t="n">
         <v>7</v>
@@ -21884,10 +21884,10 @@
         <v>35</v>
       </c>
       <c r="K447" t="n">
-        <v>34.3</v>
+        <v>38.5</v>
       </c>
       <c r="L447" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="448">
@@ -21898,12 +21898,12 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
@@ -21913,17 +21913,17 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F448" s="1" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="G448" s="1" t="n">
-        <v>46307</v>
+        <v>46301</v>
       </c>
       <c r="H448" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I448" t="n">
         <v>7</v>
@@ -21932,10 +21932,10 @@
         <v>35</v>
       </c>
       <c r="K448" t="n">
-        <v>34.7</v>
+        <v>37.1</v>
       </c>
       <c r="L448" t="n">
-        <v>99.09999999999999</v>
+        <v>106</v>
       </c>
     </row>
     <row r="449">
@@ -21946,7 +21946,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -21961,17 +21961,17 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F449" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G449" s="1" t="n">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="H449" s="1" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="I449" t="n">
         <v>14</v>
@@ -21980,10 +21980,10 @@
         <v>35</v>
       </c>
       <c r="K449" t="n">
-        <v>38.8</v>
+        <v>33.5</v>
       </c>
       <c r="L449" t="n">
-        <v>110.9</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="450">
@@ -21994,7 +21994,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -22009,17 +22009,17 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F450" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G450" s="1" t="n">
-        <v>46314</v>
+        <v>46311</v>
       </c>
       <c r="H450" s="1" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="I450" t="n">
         <v>14</v>
@@ -22028,10 +22028,10 @@
         <v>35</v>
       </c>
       <c r="K450" t="n">
-        <v>38.3</v>
+        <v>32</v>
       </c>
       <c r="L450" t="n">
-        <v>109.4</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="451">
@@ -22042,7 +22042,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -22057,14 +22057,14 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F451" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G451" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="H451" s="1" t="n">
         <v>46309</v>
@@ -22076,10 +22076,10 @@
         <v>35</v>
       </c>
       <c r="K451" t="n">
-        <v>33.4</v>
+        <v>24.4</v>
       </c>
       <c r="L451" t="n">
-        <v>95.40000000000001</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="452">
@@ -22090,7 +22090,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -22105,14 +22105,14 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F452" s="1" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="G452" s="1" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="H452" s="1" t="n">
         <v>46309</v>
@@ -22124,10 +22124,10 @@
         <v>35</v>
       </c>
       <c r="K452" t="n">
-        <v>32.4</v>
+        <v>24.6</v>
       </c>
       <c r="L452" t="n">
-        <v>92.59999999999999</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="453">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -22153,17 +22153,17 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F453" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G453" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H453" s="1" t="n">
         <v>46315</v>
-      </c>
-      <c r="H453" s="1" t="n">
-        <v>46316</v>
       </c>
       <c r="I453" t="n">
         <v>14</v>
@@ -22172,10 +22172,10 @@
         <v>35</v>
       </c>
       <c r="K453" t="n">
-        <v>45.8</v>
+        <v>35.4</v>
       </c>
       <c r="L453" t="n">
-        <v>130.9</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="454">
@@ -22186,7 +22186,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -22201,17 +22201,17 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F454" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G454" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H454" s="1" t="n">
         <v>46315</v>
-      </c>
-      <c r="H454" s="1" t="n">
-        <v>46316</v>
       </c>
       <c r="I454" t="n">
         <v>14</v>
@@ -22220,10 +22220,10 @@
         <v>35</v>
       </c>
       <c r="K454" t="n">
-        <v>47</v>
+        <v>35.8</v>
       </c>
       <c r="L454" t="n">
-        <v>134.3</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="455">
@@ -22234,7 +22234,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -22249,14 +22249,14 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F455" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G455" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H455" s="1" t="n">
         <v>46309</v>
@@ -22268,10 +22268,10 @@
         <v>35</v>
       </c>
       <c r="K455" t="n">
-        <v>37.9</v>
+        <v>22.8</v>
       </c>
       <c r="L455" t="n">
-        <v>108.3</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="456">
@@ -22282,7 +22282,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -22297,14 +22297,14 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F456" s="1" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G456" s="1" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="H456" s="1" t="n">
         <v>46309</v>
@@ -22316,10 +22316,10 @@
         <v>35</v>
       </c>
       <c r="K456" t="n">
-        <v>38.4</v>
+        <v>23.3</v>
       </c>
       <c r="L456" t="n">
-        <v>109.7</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="457">
@@ -22330,7 +22330,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -22345,17 +22345,17 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F457" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G457" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H457" s="1" t="n">
         <v>46315</v>
-      </c>
-      <c r="H457" s="1" t="n">
-        <v>46316</v>
       </c>
       <c r="I457" t="n">
         <v>14</v>
@@ -22364,10 +22364,10 @@
         <v>35</v>
       </c>
       <c r="K457" t="n">
-        <v>46.3</v>
+        <v>37.8</v>
       </c>
       <c r="L457" t="n">
-        <v>132.3</v>
+        <v>108</v>
       </c>
     </row>
     <row r="458">
@@ -22378,7 +22378,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -22393,17 +22393,17 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F458" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G458" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H458" s="1" t="n">
         <v>46315</v>
-      </c>
-      <c r="H458" s="1" t="n">
-        <v>46316</v>
       </c>
       <c r="I458" t="n">
         <v>14</v>
@@ -22412,10 +22412,10 @@
         <v>35</v>
       </c>
       <c r="K458" t="n">
-        <v>45.7</v>
+        <v>38.9</v>
       </c>
       <c r="L458" t="n">
-        <v>130.6</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="459">
@@ -22426,7 +22426,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -22441,14 +22441,14 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F459" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G459" s="1" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="H459" s="1" t="n">
         <v>46309</v>
@@ -22460,10 +22460,10 @@
         <v>35</v>
       </c>
       <c r="K459" t="n">
-        <v>38.9</v>
+        <v>34.3</v>
       </c>
       <c r="L459" t="n">
-        <v>111.1</v>
+        <v>98</v>
       </c>
     </row>
     <row r="460">
@@ -22474,7 +22474,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -22489,14 +22489,14 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F460" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G460" s="1" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="H460" s="1" t="n">
         <v>46309</v>
@@ -22508,10 +22508,10 @@
         <v>35</v>
       </c>
       <c r="K460" t="n">
-        <v>38</v>
+        <v>34.7</v>
       </c>
       <c r="L460" t="n">
-        <v>108.6</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="461">
@@ -22522,12 +22522,12 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -22537,17 +22537,17 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F461" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G461" s="1" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="H461" s="1" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="I461" t="n">
         <v>14</v>
@@ -22556,10 +22556,10 @@
         <v>35</v>
       </c>
       <c r="K461" t="n">
-        <v>48</v>
+        <v>38.8</v>
       </c>
       <c r="L461" t="n">
-        <v>137.1</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="462">
@@ -22570,12 +22570,12 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -22585,17 +22585,17 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F462" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G462" s="1" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="H462" s="1" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="I462" t="n">
         <v>14</v>
@@ -22604,10 +22604,10 @@
         <v>35</v>
       </c>
       <c r="K462" t="n">
-        <v>48.7</v>
+        <v>38.3</v>
       </c>
       <c r="L462" t="n">
-        <v>139.1</v>
+        <v>109.4</v>
       </c>
     </row>
     <row r="463">
@@ -22618,12 +22618,12 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -22633,17 +22633,17 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F463" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G463" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H463" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H463" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I463" t="n">
         <v>7</v>
@@ -22652,10 +22652,10 @@
         <v>35</v>
       </c>
       <c r="K463" t="n">
-        <v>41.2</v>
+        <v>33.4</v>
       </c>
       <c r="L463" t="n">
-        <v>117.7</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="464">
@@ -22666,12 +22666,12 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -22681,17 +22681,17 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F464" s="1" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="G464" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H464" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H464" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I464" t="n">
         <v>7</v>
@@ -22700,10 +22700,10 @@
         <v>35</v>
       </c>
       <c r="K464" t="n">
-        <v>41.7</v>
+        <v>32.4</v>
       </c>
       <c r="L464" t="n">
-        <v>119.1</v>
+        <v>92.59999999999999</v>
       </c>
     </row>
     <row r="465">
@@ -22714,12 +22714,12 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -22729,14 +22729,14 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F465" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G465" s="1" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="H465" s="1" t="n">
         <v>46316</v>
@@ -22748,10 +22748,10 @@
         <v>35</v>
       </c>
       <c r="K465" t="n">
-        <v>39.8</v>
+        <v>45.8</v>
       </c>
       <c r="L465" t="n">
-        <v>113.7</v>
+        <v>130.9</v>
       </c>
     </row>
     <row r="466">
@@ -22762,12 +22762,12 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -22777,14 +22777,14 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F466" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G466" s="1" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="H466" s="1" t="n">
         <v>46316</v>
@@ -22796,10 +22796,10 @@
         <v>35</v>
       </c>
       <c r="K466" t="n">
-        <v>38.2</v>
+        <v>47</v>
       </c>
       <c r="L466" t="n">
-        <v>109.1</v>
+        <v>134.3</v>
       </c>
     </row>
     <row r="467">
@@ -22810,12 +22810,12 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -22825,17 +22825,17 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F467" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G467" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H467" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H467" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I467" t="n">
         <v>7</v>
@@ -22844,10 +22844,10 @@
         <v>35</v>
       </c>
       <c r="K467" t="n">
-        <v>32.8</v>
+        <v>37.9</v>
       </c>
       <c r="L467" t="n">
-        <v>93.7</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="468">
@@ -22858,12 +22858,12 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -22873,17 +22873,17 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F468" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G468" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H468" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H468" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I468" t="n">
         <v>7</v>
@@ -22892,10 +22892,10 @@
         <v>35</v>
       </c>
       <c r="K468" t="n">
-        <v>31.8</v>
+        <v>38.4</v>
       </c>
       <c r="L468" t="n">
-        <v>90.90000000000001</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="469">
@@ -22906,12 +22906,12 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
@@ -22921,17 +22921,17 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F469" s="1" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="G469" s="1" t="n">
-        <v>46317</v>
+        <v>46315</v>
       </c>
       <c r="H469" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I469" t="n">
         <v>14</v>
@@ -22940,10 +22940,10 @@
         <v>35</v>
       </c>
       <c r="K469" t="n">
-        <v>43.2</v>
+        <v>46.3</v>
       </c>
       <c r="L469" t="n">
-        <v>123.4</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="470">
@@ -22954,12 +22954,12 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -22969,17 +22969,17 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F470" s="1" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="G470" s="1" t="n">
-        <v>46317</v>
+        <v>46315</v>
       </c>
       <c r="H470" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I470" t="n">
         <v>14</v>
@@ -22988,10 +22988,10 @@
         <v>35</v>
       </c>
       <c r="K470" t="n">
-        <v>42.7</v>
+        <v>45.7</v>
       </c>
       <c r="L470" t="n">
-        <v>122</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="471">
@@ -23002,12 +23002,12 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -23017,17 +23017,17 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F471" s="1" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="G471" s="1" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="H471" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="I471" t="n">
         <v>7</v>
@@ -23036,10 +23036,10 @@
         <v>35</v>
       </c>
       <c r="K471" t="n">
-        <v>35.7</v>
+        <v>38.9</v>
       </c>
       <c r="L471" t="n">
-        <v>102</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="472">
@@ -23050,12 +23050,12 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
@@ -23065,17 +23065,17 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F472" s="1" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="G472" s="1" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="H472" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="I472" t="n">
         <v>7</v>
@@ -23084,10 +23084,10 @@
         <v>35</v>
       </c>
       <c r="K472" t="n">
-        <v>36.2</v>
+        <v>38</v>
       </c>
       <c r="L472" t="n">
-        <v>103.4</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="473">
@@ -23098,7 +23098,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
@@ -23113,29 +23113,29 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F473" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G473" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H473" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I473" t="n">
         <v>14</v>
       </c>
       <c r="J473" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K473" t="n">
-        <v>29.1</v>
+        <v>48</v>
       </c>
       <c r="L473" t="n">
-        <v>118.8</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="474">
@@ -23146,7 +23146,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -23161,29 +23161,29 @@
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F474" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G474" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H474" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I474" t="n">
         <v>14</v>
       </c>
       <c r="J474" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K474" t="n">
-        <v>28.8</v>
+        <v>48.7</v>
       </c>
       <c r="L474" t="n">
-        <v>117.6</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="475">
@@ -23194,7 +23194,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
@@ -23209,14 +23209,14 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F475" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G475" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H475" s="1" t="n">
         <v>46310</v>
@@ -23225,13 +23225,13 @@
         <v>7</v>
       </c>
       <c r="J475" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K475" t="n">
-        <v>24.4</v>
+        <v>41.2</v>
       </c>
       <c r="L475" t="n">
-        <v>99.59999999999999</v>
+        <v>117.7</v>
       </c>
     </row>
     <row r="476">
@@ -23242,7 +23242,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
@@ -23257,14 +23257,14 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F476" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G476" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H476" s="1" t="n">
         <v>46310</v>
@@ -23273,13 +23273,13 @@
         <v>7</v>
       </c>
       <c r="J476" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K476" t="n">
-        <v>23.6</v>
+        <v>41.7</v>
       </c>
       <c r="L476" t="n">
-        <v>96.3</v>
+        <v>119.1</v>
       </c>
     </row>
     <row r="477">
@@ -23290,7 +23290,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
@@ -23305,29 +23305,29 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F477" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G477" s="1" t="n">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="H477" s="1" t="n">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="I477" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J477" t="n">
         <v>35</v>
       </c>
       <c r="K477" t="n">
-        <v>34.6</v>
+        <v>39.8</v>
       </c>
       <c r="L477" t="n">
-        <v>98.90000000000001</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="478">
@@ -23338,7 +23338,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -23353,29 +23353,29 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F478" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G478" s="1" t="n">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="H478" s="1" t="n">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="I478" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J478" t="n">
         <v>35</v>
       </c>
       <c r="K478" t="n">
-        <v>34.7</v>
+        <v>38.2</v>
       </c>
       <c r="L478" t="n">
-        <v>99.09999999999999</v>
+        <v>109.1</v>
       </c>
     </row>
     <row r="479">
@@ -23386,12 +23386,12 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D479" t="inlineStr">
@@ -23401,17 +23401,17 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F479" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G479" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="H479" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="I479" t="n">
         <v>7</v>
@@ -23420,10 +23420,10 @@
         <v>35</v>
       </c>
       <c r="K479" t="n">
-        <v>32.5</v>
+        <v>32.8</v>
       </c>
       <c r="L479" t="n">
-        <v>92.90000000000001</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="480">
@@ -23434,12 +23434,12 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
@@ -23449,17 +23449,17 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F480" s="1" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="G480" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="H480" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="I480" t="n">
         <v>7</v>
@@ -23468,10 +23468,10 @@
         <v>35</v>
       </c>
       <c r="K480" t="n">
-        <v>32.2</v>
+        <v>31.8</v>
       </c>
       <c r="L480" t="n">
-        <v>92</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="481">
@@ -23482,12 +23482,12 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
@@ -23497,29 +23497,29 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F481" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G481" s="1" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H481" s="1" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="I481" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J481" t="n">
         <v>35</v>
       </c>
       <c r="K481" t="n">
-        <v>42.5</v>
+        <v>43.2</v>
       </c>
       <c r="L481" t="n">
-        <v>121.4</v>
+        <v>123.4</v>
       </c>
     </row>
     <row r="482">
@@ -23530,12 +23530,12 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
@@ -23545,29 +23545,29 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F482" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G482" s="1" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H482" s="1" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="I482" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J482" t="n">
         <v>35</v>
       </c>
       <c r="K482" t="n">
-        <v>41.9</v>
+        <v>42.7</v>
       </c>
       <c r="L482" t="n">
-        <v>119.7</v>
+        <v>122</v>
       </c>
     </row>
     <row r="483">
@@ -23578,12 +23578,12 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
@@ -23593,17 +23593,17 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F483" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G483" s="1" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="H483" s="1" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="I483" t="n">
         <v>7</v>
@@ -23612,10 +23612,10 @@
         <v>35</v>
       </c>
       <c r="K483" t="n">
-        <v>40.7</v>
+        <v>35.7</v>
       </c>
       <c r="L483" t="n">
-        <v>116.3</v>
+        <v>102</v>
       </c>
     </row>
     <row r="484">
@@ -23626,12 +23626,12 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>P82</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -23641,17 +23641,17 @@
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F484" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G484" s="1" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="H484" s="1" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="I484" t="n">
         <v>7</v>
@@ -23660,10 +23660,10 @@
         <v>35</v>
       </c>
       <c r="K484" t="n">
-        <v>32.3</v>
+        <v>36.2</v>
       </c>
       <c r="L484" t="n">
-        <v>92.3</v>
+        <v>103.4</v>
       </c>
     </row>
     <row r="485">
@@ -23674,12 +23674,12 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>P82</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -23689,29 +23689,29 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F485" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G485" s="1" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H485" s="1" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="I485" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J485" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K485" t="n">
-        <v>30.9</v>
+        <v>29.1</v>
       </c>
       <c r="L485" t="n">
-        <v>88.3</v>
+        <v>118.8</v>
       </c>
     </row>
     <row r="486">
@@ -23722,12 +23722,12 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>P83</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -23737,29 +23737,29 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>Pilote 103 torre 2 tipo 1</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F486" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G486" s="1" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="H486" s="1" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="I486" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J486" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K486" t="n">
-        <v>20.2</v>
+        <v>28.8</v>
       </c>
       <c r="L486" t="n">
-        <v>57.7</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="487">
@@ -23770,12 +23770,12 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>P83</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
@@ -23785,29 +23785,29 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>Pilote 103 torre 2 tipo 1</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F487" s="1" t="n">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="G487" s="1" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="H487" s="1" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="I487" t="n">
         <v>7</v>
       </c>
       <c r="J487" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K487" t="n">
-        <v>20.6</v>
+        <v>24.4</v>
       </c>
       <c r="L487" t="n">
-        <v>58.9</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="488">
@@ -23818,12 +23818,12 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>P84</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
@@ -23833,29 +23833,29 @@
       </c>
       <c r="E488" t="inlineStr">
         <is>
-          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F488" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="G488" s="1" t="n">
         <v>46310</v>
       </c>
-      <c r="G488" s="1" t="n">
-        <v>46317</v>
-      </c>
       <c r="H488" s="1" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="I488" t="n">
         <v>7</v>
       </c>
       <c r="J488" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K488" t="n">
-        <v>35.5</v>
+        <v>23.6</v>
       </c>
       <c r="L488" t="n">
-        <v>101.4</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="489">
@@ -23866,12 +23866,12 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>P84</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
@@ -23881,29 +23881,29 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F489" s="1" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="G489" s="1" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H489" s="1" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="I489" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J489" t="n">
         <v>35</v>
       </c>
       <c r="K489" t="n">
-        <v>35.1</v>
+        <v>41.2</v>
       </c>
       <c r="L489" t="n">
-        <v>100.3</v>
+        <v>117.7</v>
       </c>
     </row>
     <row r="490">
@@ -23914,12 +23914,12 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>P85</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
@@ -23929,29 +23929,29 @@
       </c>
       <c r="E490" t="inlineStr">
         <is>
-          <t>Pilote 73 torre 2 tipo 2</t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F490" s="1" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="G490" s="1" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H490" s="1" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="I490" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J490" t="n">
         <v>35</v>
       </c>
       <c r="K490" t="n">
-        <v>42.5</v>
+        <v>41.9</v>
       </c>
       <c r="L490" t="n">
-        <v>121.4</v>
+        <v>119.7</v>
       </c>
     </row>
     <row r="491">
@@ -23962,12 +23962,12 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>P85</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
@@ -23977,17 +23977,17 @@
       </c>
       <c r="E491" t="inlineStr">
         <is>
-          <t>Pilote 73 torre 2 tipo 2</t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F491" s="1" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="G491" s="1" t="n">
-        <v>46317</v>
+        <v>46311</v>
       </c>
       <c r="H491" s="1" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="I491" t="n">
         <v>7</v>
@@ -23996,10 +23996,1066 @@
         <v>35</v>
       </c>
       <c r="K491" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="L491" t="n">
+        <v>98.90000000000001</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>P78</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F492" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G492" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H492" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I492" t="n">
+        <v>7</v>
+      </c>
+      <c r="J492" t="n">
+        <v>35</v>
+      </c>
+      <c r="K492" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="L492" t="n">
+        <v>99.09999999999999</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F493" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G493" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H493" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I493" t="n">
+        <v>14</v>
+      </c>
+      <c r="J493" t="n">
+        <v>35</v>
+      </c>
+      <c r="K493" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="L493" t="n">
+        <v>110.9</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F494" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G494" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H494" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I494" t="n">
+        <v>14</v>
+      </c>
+      <c r="J494" t="n">
+        <v>35</v>
+      </c>
+      <c r="K494" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="L494" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F495" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G495" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H495" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I495" t="n">
+        <v>7</v>
+      </c>
+      <c r="J495" t="n">
+        <v>35</v>
+      </c>
+      <c r="K495" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="L495" t="n">
+        <v>92.90000000000001</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>P79</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+        </is>
+      </c>
+      <c r="F496" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G496" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H496" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="I496" t="n">
+        <v>7</v>
+      </c>
+      <c r="J496" t="n">
+        <v>35</v>
+      </c>
+      <c r="K496" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="L496" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F497" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G497" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H497" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I497" t="n">
+        <v>7</v>
+      </c>
+      <c r="J497" t="n">
+        <v>35</v>
+      </c>
+      <c r="K497" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L497" t="n">
+        <v>121.4</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F498" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G498" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H498" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I498" t="n">
+        <v>7</v>
+      </c>
+      <c r="J498" t="n">
+        <v>35</v>
+      </c>
+      <c r="K498" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="L498" t="n">
+        <v>119.7</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>P81</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F499" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G499" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H499" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I499" t="n">
+        <v>7</v>
+      </c>
+      <c r="J499" t="n">
+        <v>35</v>
+      </c>
+      <c r="K499" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="L499" t="n">
+        <v>116.3</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>P82</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F500" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G500" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H500" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I500" t="n">
+        <v>7</v>
+      </c>
+      <c r="J500" t="n">
+        <v>35</v>
+      </c>
+      <c r="K500" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="L500" t="n">
+        <v>92.3</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>P82</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Pilote 63 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F501" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G501" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H501" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I501" t="n">
+        <v>7</v>
+      </c>
+      <c r="J501" t="n">
+        <v>35</v>
+      </c>
+      <c r="K501" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="L501" t="n">
+        <v>88.3</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>P83</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Pilote 103 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F502" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G502" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H502" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I502" t="n">
+        <v>7</v>
+      </c>
+      <c r="J502" t="n">
+        <v>35</v>
+      </c>
+      <c r="K502" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="L502" t="n">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>P83</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Pilote 103 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F503" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G503" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H503" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I503" t="n">
+        <v>7</v>
+      </c>
+      <c r="J503" t="n">
+        <v>35</v>
+      </c>
+      <c r="K503" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="L503" t="n">
+        <v>58.9</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>P84</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F504" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G504" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H504" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I504" t="n">
+        <v>7</v>
+      </c>
+      <c r="J504" t="n">
+        <v>35</v>
+      </c>
+      <c r="K504" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="L504" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>P84</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F505" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G505" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H505" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I505" t="n">
+        <v>7</v>
+      </c>
+      <c r="J505" t="n">
+        <v>35</v>
+      </c>
+      <c r="K505" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="L505" t="n">
+        <v>100.3</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>P85</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Pilote 73 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F506" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G506" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H506" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I506" t="n">
+        <v>7</v>
+      </c>
+      <c r="J506" t="n">
+        <v>35</v>
+      </c>
+      <c r="K506" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L506" t="n">
+        <v>121.4</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>P85</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Pilote 73 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F507" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="G507" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H507" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="I507" t="n">
+        <v>7</v>
+      </c>
+      <c r="J507" t="n">
+        <v>35</v>
+      </c>
+      <c r="K507" t="n">
         <v>41.6</v>
       </c>
-      <c r="L491" t="n">
+      <c r="L507" t="n">
         <v>118.9</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>P86</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Pilote 79 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F508" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G508" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H508" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I508" t="n">
+        <v>7</v>
+      </c>
+      <c r="J508" t="n">
+        <v>35</v>
+      </c>
+      <c r="K508" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="L508" t="n">
+        <v>98.59999999999999</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>P86</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Pilote 79 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F509" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G509" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H509" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I509" t="n">
+        <v>7</v>
+      </c>
+      <c r="J509" t="n">
+        <v>35</v>
+      </c>
+      <c r="K509" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="L509" t="n">
+        <v>94.90000000000001</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>P87</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Pilote 91 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F510" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G510" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H510" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I510" t="n">
+        <v>7</v>
+      </c>
+      <c r="J510" t="n">
+        <v>35</v>
+      </c>
+      <c r="K510" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="L510" t="n">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>P87</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Pilote 91 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F511" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G511" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H511" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I511" t="n">
+        <v>7</v>
+      </c>
+      <c r="J511" t="n">
+        <v>35</v>
+      </c>
+      <c r="K511" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="L511" t="n">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>P88</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F512" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G512" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H512" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I512" t="n">
+        <v>7</v>
+      </c>
+      <c r="J512" t="n">
+        <v>35</v>
+      </c>
+      <c r="K512" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="L512" t="n">
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>P88</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F513" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G513" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H513" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I513" t="n">
+        <v>7</v>
+      </c>
+      <c r="J513" t="n">
+        <v>35</v>
+      </c>
+      <c r="K513" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="L513" t="n">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[AUTO] Transformación Concrelab - 2026-10-27 20:33:00
</commit_message>
<xml_diff>
--- a/DatosTransformados/reporte_concrelab_VENTO.xlsx
+++ b/DatosTransformados/reporte_concrelab_VENTO.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L513"/>
+  <dimension ref="A1:L520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21392,22 +21392,22 @@
         <v>46293</v>
       </c>
       <c r="G437" s="1" t="n">
-        <v>46307</v>
+        <v>46321</v>
       </c>
       <c r="H437" s="1" t="n">
-        <v>46309</v>
+        <v>46322</v>
       </c>
       <c r="I437" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J437" t="n">
         <v>35</v>
       </c>
       <c r="K437" t="n">
-        <v>49</v>
+        <v>56.5</v>
       </c>
       <c r="L437" t="n">
-        <v>140</v>
+        <v>161.4</v>
       </c>
     </row>
     <row r="438">
@@ -21440,22 +21440,22 @@
         <v>46293</v>
       </c>
       <c r="G438" s="1" t="n">
-        <v>46307</v>
+        <v>46321</v>
       </c>
       <c r="H438" s="1" t="n">
-        <v>46309</v>
+        <v>46322</v>
       </c>
       <c r="I438" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="J438" t="n">
         <v>35</v>
       </c>
       <c r="K438" t="n">
-        <v>47.9</v>
+        <v>57.3</v>
       </c>
       <c r="L438" t="n">
-        <v>136.9</v>
+        <v>163.7</v>
       </c>
     </row>
     <row r="439">
@@ -21488,22 +21488,22 @@
         <v>46293</v>
       </c>
       <c r="G439" s="1" t="n">
-        <v>46300</v>
+        <v>46321</v>
       </c>
       <c r="H439" s="1" t="n">
-        <v>46302</v>
+        <v>46322</v>
       </c>
       <c r="I439" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="J439" t="n">
         <v>35</v>
       </c>
       <c r="K439" t="n">
-        <v>41.4</v>
+        <v>58</v>
       </c>
       <c r="L439" t="n">
-        <v>118.3</v>
+        <v>165.7</v>
       </c>
     </row>
     <row r="440">
@@ -21536,22 +21536,22 @@
         <v>46293</v>
       </c>
       <c r="G440" s="1" t="n">
-        <v>46300</v>
+        <v>46307</v>
       </c>
       <c r="H440" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I440" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J440" t="n">
         <v>35</v>
       </c>
       <c r="K440" t="n">
-        <v>40.3</v>
+        <v>49</v>
       </c>
       <c r="L440" t="n">
-        <v>115.1</v>
+        <v>140</v>
       </c>
     </row>
     <row r="441">
@@ -21562,7 +21562,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -21577,14 +21577,14 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F441" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G441" s="1" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="H441" s="1" t="n">
         <v>46309</v>
@@ -21596,10 +21596,10 @@
         <v>35</v>
       </c>
       <c r="K441" t="n">
-        <v>44.3</v>
+        <v>47.9</v>
       </c>
       <c r="L441" t="n">
-        <v>126.6</v>
+        <v>136.9</v>
       </c>
     </row>
     <row r="442">
@@ -21610,7 +21610,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -21625,29 +21625,29 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F442" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G442" s="1" t="n">
-        <v>46308</v>
+        <v>46300</v>
       </c>
       <c r="H442" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I442" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J442" t="n">
         <v>35</v>
       </c>
       <c r="K442" t="n">
-        <v>44.9</v>
+        <v>41.4</v>
       </c>
       <c r="L442" t="n">
-        <v>128.3</v>
+        <v>118.3</v>
       </c>
     </row>
     <row r="443">
@@ -21658,7 +21658,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>P61</t>
+          <t>P60</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -21673,14 +21673,14 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>Pilote 69 Torre 2 Tipo 2</t>
+          <t>Pilote 106 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F443" s="1" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="G443" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="H443" s="1" t="n">
         <v>46302</v>
@@ -21692,10 +21692,10 @@
         <v>35</v>
       </c>
       <c r="K443" t="n">
-        <v>37.5</v>
+        <v>40.3</v>
       </c>
       <c r="L443" t="n">
-        <v>107.1</v>
+        <v>115.1</v>
       </c>
     </row>
     <row r="444">
@@ -21728,22 +21728,22 @@
         <v>46294</v>
       </c>
       <c r="G444" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H444" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I444" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J444" t="n">
         <v>35</v>
       </c>
       <c r="K444" t="n">
-        <v>36.4</v>
+        <v>44.3</v>
       </c>
       <c r="L444" t="n">
-        <v>104</v>
+        <v>126.6</v>
       </c>
     </row>
     <row r="445">
@@ -21754,7 +21754,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -21769,7 +21769,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F445" s="1" t="n">
@@ -21788,10 +21788,10 @@
         <v>35</v>
       </c>
       <c r="K445" t="n">
-        <v>43.9</v>
+        <v>44.9</v>
       </c>
       <c r="L445" t="n">
-        <v>125.4</v>
+        <v>128.3</v>
       </c>
     </row>
     <row r="446">
@@ -21802,7 +21802,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -21817,29 +21817,29 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F446" s="1" t="n">
         <v>46294</v>
       </c>
       <c r="G446" s="1" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="H446" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I446" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J446" t="n">
         <v>35</v>
       </c>
       <c r="K446" t="n">
-        <v>43.7</v>
+        <v>37.5</v>
       </c>
       <c r="L446" t="n">
-        <v>124.9</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="447">
@@ -21850,7 +21850,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>P62</t>
+          <t>P61</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -21865,7 +21865,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
+          <t>Pilote 69 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F447" s="1" t="n">
@@ -21884,10 +21884,10 @@
         <v>35</v>
       </c>
       <c r="K447" t="n">
-        <v>38.5</v>
+        <v>36.4</v>
       </c>
       <c r="L447" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="448">
@@ -21920,22 +21920,22 @@
         <v>46294</v>
       </c>
       <c r="G448" s="1" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="H448" s="1" t="n">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="I448" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J448" t="n">
         <v>35</v>
       </c>
       <c r="K448" t="n">
-        <v>37.1</v>
+        <v>43.9</v>
       </c>
       <c r="L448" t="n">
-        <v>106</v>
+        <v>125.4</v>
       </c>
     </row>
     <row r="449">
@@ -21946,12 +21946,12 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
@@ -21961,17 +21961,17 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F449" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G449" s="1" t="n">
-        <v>46311</v>
+        <v>46308</v>
       </c>
       <c r="H449" s="1" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="I449" t="n">
         <v>14</v>
@@ -21980,10 +21980,10 @@
         <v>35</v>
       </c>
       <c r="K449" t="n">
-        <v>33.5</v>
+        <v>43.7</v>
       </c>
       <c r="L449" t="n">
-        <v>95.7</v>
+        <v>124.9</v>
       </c>
     </row>
     <row r="450">
@@ -21994,12 +21994,12 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
@@ -22009,29 +22009,29 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F450" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G450" s="1" t="n">
-        <v>46311</v>
+        <v>46301</v>
       </c>
       <c r="H450" s="1" t="n">
-        <v>46311</v>
+        <v>46302</v>
       </c>
       <c r="I450" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J450" t="n">
         <v>35</v>
       </c>
       <c r="K450" t="n">
-        <v>32</v>
+        <v>38.5</v>
       </c>
       <c r="L450" t="n">
-        <v>91.40000000000001</v>
+        <v>110</v>
       </c>
     </row>
     <row r="451">
@@ -22042,12 +22042,12 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>P68</t>
+          <t>P62</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No Especificado</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
@@ -22057,17 +22057,17 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
+          <t>Pilote 66 - 59 Torre 2 Tipo 2</t>
         </is>
       </c>
       <c r="F451" s="1" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="G451" s="1" t="n">
-        <v>46304</v>
+        <v>46301</v>
       </c>
       <c r="H451" s="1" t="n">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="I451" t="n">
         <v>7</v>
@@ -22076,10 +22076,10 @@
         <v>35</v>
       </c>
       <c r="K451" t="n">
-        <v>24.4</v>
+        <v>37.1</v>
       </c>
       <c r="L451" t="n">
-        <v>69.7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="452">
@@ -22112,22 +22112,22 @@
         <v>46297</v>
       </c>
       <c r="G452" s="1" t="n">
-        <v>46304</v>
+        <v>46311</v>
       </c>
       <c r="H452" s="1" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I452" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J452" t="n">
         <v>35</v>
       </c>
       <c r="K452" t="n">
-        <v>24.6</v>
+        <v>33.5</v>
       </c>
       <c r="L452" t="n">
-        <v>70.3</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="453">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -22153,17 +22153,17 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F453" s="1" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="G453" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="H453" s="1" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="I453" t="n">
         <v>14</v>
@@ -22172,10 +22172,10 @@
         <v>35</v>
       </c>
       <c r="K453" t="n">
-        <v>35.4</v>
+        <v>32</v>
       </c>
       <c r="L453" t="n">
-        <v>101.1</v>
+        <v>91.40000000000001</v>
       </c>
     </row>
     <row r="454">
@@ -22186,7 +22186,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -22201,29 +22201,29 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F454" s="1" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="G454" s="1" t="n">
-        <v>46312</v>
+        <v>46304</v>
       </c>
       <c r="H454" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I454" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J454" t="n">
         <v>35</v>
       </c>
       <c r="K454" t="n">
-        <v>35.8</v>
+        <v>24.4</v>
       </c>
       <c r="L454" t="n">
-        <v>102.3</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="455">
@@ -22234,7 +22234,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>P69</t>
+          <t>P68</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -22249,14 +22249,14 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
+          <t xml:space="preserve">Pilote 85 torre 2 tipo 2, pilote 77 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F455" s="1" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="G455" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="H455" s="1" t="n">
         <v>46309</v>
@@ -22268,10 +22268,10 @@
         <v>35</v>
       </c>
       <c r="K455" t="n">
-        <v>22.8</v>
+        <v>24.6</v>
       </c>
       <c r="L455" t="n">
-        <v>65.09999999999999</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="456">
@@ -22304,22 +22304,22 @@
         <v>46298</v>
       </c>
       <c r="G456" s="1" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="H456" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I456" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J456" t="n">
         <v>35</v>
       </c>
       <c r="K456" t="n">
-        <v>23.3</v>
+        <v>35.4</v>
       </c>
       <c r="L456" t="n">
-        <v>66.59999999999999</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="457">
@@ -22330,7 +22330,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -22345,14 +22345,14 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F457" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G457" s="1" t="n">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="H457" s="1" t="n">
         <v>46315</v>
@@ -22364,10 +22364,10 @@
         <v>35</v>
       </c>
       <c r="K457" t="n">
-        <v>37.8</v>
+        <v>35.8</v>
       </c>
       <c r="L457" t="n">
-        <v>108</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="458">
@@ -22378,7 +22378,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -22393,29 +22393,29 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F458" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G458" s="1" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="H458" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I458" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J458" t="n">
         <v>35</v>
       </c>
       <c r="K458" t="n">
-        <v>38.9</v>
+        <v>22.8</v>
       </c>
       <c r="L458" t="n">
-        <v>111.1</v>
+        <v>65.09999999999999</v>
       </c>
     </row>
     <row r="459">
@@ -22426,7 +22426,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>P70</t>
+          <t>P69</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -22441,14 +22441,14 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 107 torre 2 tipo 1 </t>
         </is>
       </c>
       <c r="F459" s="1" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G459" s="1" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="H459" s="1" t="n">
         <v>46309</v>
@@ -22460,10 +22460,10 @@
         <v>35</v>
       </c>
       <c r="K459" t="n">
-        <v>34.3</v>
+        <v>23.3</v>
       </c>
       <c r="L459" t="n">
-        <v>98</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="460">
@@ -22496,22 +22496,22 @@
         <v>46300</v>
       </c>
       <c r="G460" s="1" t="n">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="H460" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I460" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J460" t="n">
         <v>35</v>
       </c>
       <c r="K460" t="n">
-        <v>34.7</v>
+        <v>37.8</v>
       </c>
       <c r="L460" t="n">
-        <v>99.09999999999999</v>
+        <v>108</v>
       </c>
     </row>
     <row r="461">
@@ -22522,7 +22522,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -22537,7 +22537,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F461" s="1" t="n">
@@ -22556,10 +22556,10 @@
         <v>35</v>
       </c>
       <c r="K461" t="n">
-        <v>38.8</v>
+        <v>38.9</v>
       </c>
       <c r="L461" t="n">
-        <v>110.9</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="462">
@@ -22570,7 +22570,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -22585,29 +22585,29 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F462" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="G462" s="1" t="n">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="H462" s="1" t="n">
-        <v>46315</v>
+        <v>46309</v>
       </c>
       <c r="I462" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J462" t="n">
         <v>35</v>
       </c>
       <c r="K462" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="L462" t="n">
-        <v>109.4</v>
+        <v>98</v>
       </c>
     </row>
     <row r="463">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>P71</t>
+          <t>P70</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -22633,7 +22633,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
+          <t xml:space="preserve">Pilote 70 - 72 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F463" s="1" t="n">
@@ -22652,10 +22652,10 @@
         <v>35</v>
       </c>
       <c r="K463" t="n">
-        <v>33.4</v>
+        <v>34.7</v>
       </c>
       <c r="L463" t="n">
-        <v>95.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="464">
@@ -22688,22 +22688,22 @@
         <v>46300</v>
       </c>
       <c r="G464" s="1" t="n">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="H464" s="1" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="I464" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J464" t="n">
         <v>35</v>
       </c>
       <c r="K464" t="n">
-        <v>32.4</v>
+        <v>38.8</v>
       </c>
       <c r="L464" t="n">
-        <v>92.59999999999999</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="465">
@@ -22714,7 +22714,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -22729,17 +22729,17 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F465" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G465" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H465" s="1" t="n">
         <v>46315</v>
-      </c>
-      <c r="H465" s="1" t="n">
-        <v>46316</v>
       </c>
       <c r="I465" t="n">
         <v>14</v>
@@ -22748,10 +22748,10 @@
         <v>35</v>
       </c>
       <c r="K465" t="n">
-        <v>45.8</v>
+        <v>38.3</v>
       </c>
       <c r="L465" t="n">
-        <v>130.9</v>
+        <v>109.4</v>
       </c>
     </row>
     <row r="466">
@@ -22762,7 +22762,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -22777,29 +22777,29 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F466" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G466" s="1" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="H466" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I466" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J466" t="n">
         <v>35</v>
       </c>
       <c r="K466" t="n">
-        <v>47</v>
+        <v>33.4</v>
       </c>
       <c r="L466" t="n">
-        <v>134.3</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="467">
@@ -22810,7 +22810,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>P72</t>
+          <t>P71</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -22825,14 +22825,14 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
+          <t xml:space="preserve">Pilote 71 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F467" s="1" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G467" s="1" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="H467" s="1" t="n">
         <v>46309</v>
@@ -22844,10 +22844,10 @@
         <v>35</v>
       </c>
       <c r="K467" t="n">
-        <v>37.9</v>
+        <v>32.4</v>
       </c>
       <c r="L467" t="n">
-        <v>108.3</v>
+        <v>92.59999999999999</v>
       </c>
     </row>
     <row r="468">
@@ -22880,22 +22880,22 @@
         <v>46301</v>
       </c>
       <c r="G468" s="1" t="n">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="H468" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="I468" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J468" t="n">
         <v>35</v>
       </c>
       <c r="K468" t="n">
-        <v>38.4</v>
+        <v>45.8</v>
       </c>
       <c r="L468" t="n">
-        <v>109.7</v>
+        <v>130.9</v>
       </c>
     </row>
     <row r="469">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F469" s="1" t="n">
@@ -22940,10 +22940,10 @@
         <v>35</v>
       </c>
       <c r="K469" t="n">
-        <v>46.3</v>
+        <v>47</v>
       </c>
       <c r="L469" t="n">
-        <v>132.3</v>
+        <v>134.3</v>
       </c>
     </row>
     <row r="470">
@@ -22954,7 +22954,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -22969,29 +22969,29 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F470" s="1" t="n">
         <v>46301</v>
       </c>
       <c r="G470" s="1" t="n">
-        <v>46315</v>
+        <v>46308</v>
       </c>
       <c r="H470" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I470" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J470" t="n">
         <v>35</v>
       </c>
       <c r="K470" t="n">
-        <v>45.7</v>
+        <v>37.9</v>
       </c>
       <c r="L470" t="n">
-        <v>130.6</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="471">
@@ -23002,7 +23002,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>P73</t>
+          <t>P72</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -23017,7 +23017,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Pilote 61 torre 1 tipo 2</t>
+          <t xml:space="preserve">Pilote 28 torre 1 tipo 1 </t>
         </is>
       </c>
       <c r="F471" s="1" t="n">
@@ -23036,10 +23036,10 @@
         <v>35</v>
       </c>
       <c r="K471" t="n">
-        <v>38.9</v>
+        <v>38.4</v>
       </c>
       <c r="L471" t="n">
-        <v>111.1</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="472">
@@ -23072,22 +23072,22 @@
         <v>46301</v>
       </c>
       <c r="G472" s="1" t="n">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="H472" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="I472" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J472" t="n">
         <v>35</v>
       </c>
       <c r="K472" t="n">
-        <v>38</v>
+        <v>46.3</v>
       </c>
       <c r="L472" t="n">
-        <v>108.6</v>
+        <v>132.3</v>
       </c>
     </row>
     <row r="473">
@@ -23098,12 +23098,12 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -23113,14 +23113,14 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F473" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G473" s="1" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="H473" s="1" t="n">
         <v>46316</v>
@@ -23132,10 +23132,10 @@
         <v>35</v>
       </c>
       <c r="K473" t="n">
-        <v>48</v>
+        <v>45.7</v>
       </c>
       <c r="L473" t="n">
-        <v>137.1</v>
+        <v>130.6</v>
       </c>
     </row>
     <row r="474">
@@ -23146,12 +23146,12 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
@@ -23161,29 +23161,29 @@
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F474" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G474" s="1" t="n">
-        <v>46316</v>
+        <v>46308</v>
       </c>
       <c r="H474" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="I474" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J474" t="n">
         <v>35</v>
       </c>
       <c r="K474" t="n">
-        <v>48.7</v>
+        <v>38.9</v>
       </c>
       <c r="L474" t="n">
-        <v>139.1</v>
+        <v>111.1</v>
       </c>
     </row>
     <row r="475">
@@ -23194,12 +23194,12 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>P74</t>
+          <t>P73</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t xml:space="preserve">No especificado </t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
@@ -23209,17 +23209,17 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Piolote 80 - 31 torre 2 tipo 2</t>
+          <t>Pilote 61 torre 1 tipo 2</t>
         </is>
       </c>
       <c r="F475" s="1" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="G475" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H475" s="1" t="n">
         <v>46309</v>
-      </c>
-      <c r="H475" s="1" t="n">
-        <v>46310</v>
       </c>
       <c r="I475" t="n">
         <v>7</v>
@@ -23228,10 +23228,10 @@
         <v>35</v>
       </c>
       <c r="K475" t="n">
-        <v>41.2</v>
+        <v>38</v>
       </c>
       <c r="L475" t="n">
-        <v>117.7</v>
+        <v>108.6</v>
       </c>
     </row>
     <row r="476">
@@ -23264,22 +23264,22 @@
         <v>46302</v>
       </c>
       <c r="G476" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="H476" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I476" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J476" t="n">
         <v>35</v>
       </c>
       <c r="K476" t="n">
-        <v>41.7</v>
+        <v>48</v>
       </c>
       <c r="L476" t="n">
-        <v>119.1</v>
+        <v>137.1</v>
       </c>
     </row>
     <row r="477">
@@ -23290,7 +23290,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
@@ -23305,7 +23305,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F477" s="1" t="n">
@@ -23324,10 +23324,10 @@
         <v>35</v>
       </c>
       <c r="K477" t="n">
-        <v>39.8</v>
+        <v>48.7</v>
       </c>
       <c r="L477" t="n">
-        <v>113.7</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="478">
@@ -23338,7 +23338,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -23353,29 +23353,29 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F478" s="1" t="n">
         <v>46302</v>
       </c>
       <c r="G478" s="1" t="n">
-        <v>46316</v>
+        <v>46309</v>
       </c>
       <c r="H478" s="1" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="I478" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J478" t="n">
         <v>35</v>
       </c>
       <c r="K478" t="n">
-        <v>38.2</v>
+        <v>41.2</v>
       </c>
       <c r="L478" t="n">
-        <v>109.1</v>
+        <v>117.7</v>
       </c>
     </row>
     <row r="479">
@@ -23386,7 +23386,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>P75</t>
+          <t>P74</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -23401,7 +23401,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Pilote 99 torre 2 tipo 2</t>
+          <t>Piolote 80 - 31 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F479" s="1" t="n">
@@ -23420,10 +23420,10 @@
         <v>35</v>
       </c>
       <c r="K479" t="n">
-        <v>32.8</v>
+        <v>41.7</v>
       </c>
       <c r="L479" t="n">
-        <v>93.7</v>
+        <v>119.1</v>
       </c>
     </row>
     <row r="480">
@@ -23456,22 +23456,22 @@
         <v>46302</v>
       </c>
       <c r="G480" s="1" t="n">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="H480" s="1" t="n">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="I480" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J480" t="n">
         <v>35</v>
       </c>
       <c r="K480" t="n">
-        <v>31.8</v>
+        <v>39.8</v>
       </c>
       <c r="L480" t="n">
-        <v>90.90000000000001</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="481">
@@ -23482,7 +23482,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -23497,17 +23497,17 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F481" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G481" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H481" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I481" t="n">
         <v>14</v>
@@ -23516,10 +23516,10 @@
         <v>35</v>
       </c>
       <c r="K481" t="n">
-        <v>43.2</v>
+        <v>38.2</v>
       </c>
       <c r="L481" t="n">
-        <v>123.4</v>
+        <v>109.1</v>
       </c>
     </row>
     <row r="482">
@@ -23530,7 +23530,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
@@ -23545,29 +23545,29 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F482" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G482" s="1" t="n">
-        <v>46317</v>
+        <v>46309</v>
       </c>
       <c r="H482" s="1" t="n">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="I482" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J482" t="n">
         <v>35</v>
       </c>
       <c r="K482" t="n">
-        <v>42.7</v>
+        <v>32.8</v>
       </c>
       <c r="L482" t="n">
-        <v>122</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="483">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>P76</t>
+          <t>P75</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
@@ -23593,14 +23593,14 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Pilote 97 - 100 torre 2 tipo 1</t>
+          <t>Pilote 99 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F483" s="1" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="G483" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="H483" s="1" t="n">
         <v>46310</v>
@@ -23612,10 +23612,10 @@
         <v>35</v>
       </c>
       <c r="K483" t="n">
-        <v>35.7</v>
+        <v>31.8</v>
       </c>
       <c r="L483" t="n">
-        <v>102</v>
+        <v>90.90000000000001</v>
       </c>
     </row>
     <row r="484">
@@ -23648,22 +23648,22 @@
         <v>46303</v>
       </c>
       <c r="G484" s="1" t="n">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="H484" s="1" t="n">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="I484" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J484" t="n">
         <v>35</v>
       </c>
       <c r="K484" t="n">
-        <v>36.2</v>
+        <v>43.2</v>
       </c>
       <c r="L484" t="n">
-        <v>103.4</v>
+        <v>123.4</v>
       </c>
     </row>
     <row r="485">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -23689,7 +23689,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F485" s="1" t="n">
@@ -23705,13 +23705,13 @@
         <v>14</v>
       </c>
       <c r="J485" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K485" t="n">
-        <v>29.1</v>
+        <v>42.7</v>
       </c>
       <c r="L485" t="n">
-        <v>118.8</v>
+        <v>122</v>
       </c>
     </row>
     <row r="486">
@@ -23722,7 +23722,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -23737,29 +23737,29 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F486" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="G486" s="1" t="n">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="H486" s="1" t="n">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="I486" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J486" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K486" t="n">
-        <v>28.8</v>
+        <v>35.7</v>
       </c>
       <c r="L486" t="n">
-        <v>117.6</v>
+        <v>102</v>
       </c>
     </row>
     <row r="487">
@@ -23770,7 +23770,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>P77</t>
+          <t>P76</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
@@ -23785,7 +23785,7 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>Pilote 111 salón comunal</t>
+          <t>Pilote 97 - 100 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F487" s="1" t="n">
@@ -23801,13 +23801,13 @@
         <v>7</v>
       </c>
       <c r="J487" t="n">
-        <v>24.5</v>
+        <v>35</v>
       </c>
       <c r="K487" t="n">
-        <v>24.4</v>
+        <v>36.2</v>
       </c>
       <c r="L487" t="n">
-        <v>99.59999999999999</v>
+        <v>103.4</v>
       </c>
     </row>
     <row r="488">
@@ -23840,22 +23840,22 @@
         <v>46303</v>
       </c>
       <c r="G488" s="1" t="n">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="H488" s="1" t="n">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="I488" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J488" t="n">
         <v>24.5</v>
       </c>
       <c r="K488" t="n">
-        <v>23.6</v>
+        <v>29.1</v>
       </c>
       <c r="L488" t="n">
-        <v>96.3</v>
+        <v>118.8</v>
       </c>
     </row>
     <row r="489">
@@ -23866,7 +23866,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
@@ -23881,29 +23881,29 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F489" s="1" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="G489" s="1" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="H489" s="1" t="n">
-        <v>46321</v>
+        <v>46317</v>
       </c>
       <c r="I489" t="n">
         <v>14</v>
       </c>
       <c r="J489" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K489" t="n">
-        <v>41.2</v>
+        <v>28.8</v>
       </c>
       <c r="L489" t="n">
-        <v>117.7</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="490">
@@ -23914,7 +23914,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
@@ -23929,29 +23929,29 @@
       </c>
       <c r="E490" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F490" s="1" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="G490" s="1" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="H490" s="1" t="n">
-        <v>46321</v>
+        <v>46310</v>
       </c>
       <c r="I490" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J490" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K490" t="n">
-        <v>41.9</v>
+        <v>24.4</v>
       </c>
       <c r="L490" t="n">
-        <v>119.7</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="491">
@@ -23962,7 +23962,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>P78</t>
+          <t>P77</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
@@ -23977,29 +23977,29 @@
       </c>
       <c r="E491" t="inlineStr">
         <is>
-          <t>Pilote 78 - 82 torre 2 tipo 2</t>
+          <t>Pilote 111 salón comunal</t>
         </is>
       </c>
       <c r="F491" s="1" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="G491" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="H491" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="I491" t="n">
         <v>7</v>
       </c>
       <c r="J491" t="n">
-        <v>35</v>
+        <v>24.5</v>
       </c>
       <c r="K491" t="n">
-        <v>34.6</v>
+        <v>23.6</v>
       </c>
       <c r="L491" t="n">
-        <v>98.90000000000001</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="492">
@@ -24032,22 +24032,22 @@
         <v>46304</v>
       </c>
       <c r="G492" s="1" t="n">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="H492" s="1" t="n">
-        <v>46311</v>
+        <v>46321</v>
       </c>
       <c r="I492" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J492" t="n">
         <v>35</v>
       </c>
       <c r="K492" t="n">
-        <v>34.7</v>
+        <v>41.2</v>
       </c>
       <c r="L492" t="n">
-        <v>99.09999999999999</v>
+        <v>117.7</v>
       </c>
     </row>
     <row r="493">
@@ -24058,12 +24058,12 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
@@ -24073,7 +24073,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F493" s="1" t="n">
@@ -24092,10 +24092,10 @@
         <v>35</v>
       </c>
       <c r="K493" t="n">
-        <v>38.8</v>
+        <v>41.9</v>
       </c>
       <c r="L493" t="n">
-        <v>110.9</v>
+        <v>119.7</v>
       </c>
     </row>
     <row r="494">
@@ -24106,12 +24106,12 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
@@ -24121,29 +24121,29 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F494" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="G494" s="1" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="H494" s="1" t="n">
-        <v>46321</v>
+        <v>46311</v>
       </c>
       <c r="I494" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J494" t="n">
         <v>35</v>
       </c>
       <c r="K494" t="n">
-        <v>39.2</v>
+        <v>34.6</v>
       </c>
       <c r="L494" t="n">
-        <v>112</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="495">
@@ -24154,12 +24154,12 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>P79</t>
+          <t>P78</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t xml:space="preserve">No especificado </t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
@@ -24169,7 +24169,7 @@
       </c>
       <c r="E495" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
+          <t>Pilote 78 - 82 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F495" s="1" t="n">
@@ -24188,10 +24188,10 @@
         <v>35</v>
       </c>
       <c r="K495" t="n">
-        <v>32.5</v>
+        <v>34.7</v>
       </c>
       <c r="L495" t="n">
-        <v>92.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="496">
@@ -24224,22 +24224,22 @@
         <v>46304</v>
       </c>
       <c r="G496" s="1" t="n">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="H496" s="1" t="n">
-        <v>46311</v>
+        <v>46321</v>
       </c>
       <c r="I496" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J496" t="n">
         <v>35</v>
       </c>
       <c r="K496" t="n">
-        <v>32.2</v>
+        <v>38.8</v>
       </c>
       <c r="L496" t="n">
-        <v>92</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="497">
@@ -24250,7 +24250,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P79</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -24265,29 +24265,29 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F497" s="1" t="n">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="G497" s="1" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="H497" s="1" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="I497" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J497" t="n">
         <v>35</v>
       </c>
       <c r="K497" t="n">
-        <v>42.5</v>
+        <v>39.2</v>
       </c>
       <c r="L497" t="n">
-        <v>121.4</v>
+        <v>112</v>
       </c>
     </row>
     <row r="498">
@@ -24298,7 +24298,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P79</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
@@ -24313,17 +24313,17 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F498" s="1" t="n">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="G498" s="1" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="H498" s="1" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="I498" t="n">
         <v>7</v>
@@ -24332,10 +24332,10 @@
         <v>35</v>
       </c>
       <c r="K498" t="n">
-        <v>41.9</v>
+        <v>32.5</v>
       </c>
       <c r="L498" t="n">
-        <v>119.7</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="499">
@@ -24346,7 +24346,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>P81</t>
+          <t>P79</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -24361,17 +24361,17 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Pilote 63 torre 2 tipo 2</t>
+          <t xml:space="preserve">Pilote 102 torre 2 tipo 2 </t>
         </is>
       </c>
       <c r="F499" s="1" t="n">
-        <v>46309</v>
+        <v>46304</v>
       </c>
       <c r="G499" s="1" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="H499" s="1" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="I499" t="n">
         <v>7</v>
@@ -24380,10 +24380,10 @@
         <v>35</v>
       </c>
       <c r="K499" t="n">
-        <v>40.7</v>
+        <v>32.2</v>
       </c>
       <c r="L499" t="n">
-        <v>116.3</v>
+        <v>92</v>
       </c>
     </row>
     <row r="500">
@@ -24394,7 +24394,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>P82</t>
+          <t>P81</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -24428,10 +24428,10 @@
         <v>35</v>
       </c>
       <c r="K500" t="n">
-        <v>32.3</v>
+        <v>42.5</v>
       </c>
       <c r="L500" t="n">
-        <v>92.3</v>
+        <v>121.4</v>
       </c>
     </row>
     <row r="501">
@@ -24442,7 +24442,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>P82</t>
+          <t>P81</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -24476,10 +24476,10 @@
         <v>35</v>
       </c>
       <c r="K501" t="n">
-        <v>30.9</v>
+        <v>41.9</v>
       </c>
       <c r="L501" t="n">
-        <v>88.3</v>
+        <v>119.7</v>
       </c>
     </row>
     <row r="502">
@@ -24490,7 +24490,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>P83</t>
+          <t>P81</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
@@ -24505,7 +24505,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>Pilote 103 torre 2 tipo 1</t>
+          <t>Pilote 63 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F502" s="1" t="n">
@@ -24524,10 +24524,10 @@
         <v>35</v>
       </c>
       <c r="K502" t="n">
-        <v>20.2</v>
+        <v>40.7</v>
       </c>
       <c r="L502" t="n">
-        <v>57.7</v>
+        <v>116.3</v>
       </c>
     </row>
     <row r="503">
@@ -24538,7 +24538,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>P83</t>
+          <t>P82</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -24553,7 +24553,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>Pilote 103 torre 2 tipo 1</t>
+          <t>Pilote 63 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F503" s="1" t="n">
@@ -24572,10 +24572,10 @@
         <v>35</v>
       </c>
       <c r="K503" t="n">
-        <v>20.6</v>
+        <v>32.3</v>
       </c>
       <c r="L503" t="n">
-        <v>58.9</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="504">
@@ -24586,7 +24586,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>P84</t>
+          <t>P82</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
@@ -24601,14 +24601,14 @@
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+          <t>Pilote 63 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F504" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="G504" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H504" s="1" t="n">
         <v>46318</v>
@@ -24620,10 +24620,10 @@
         <v>35</v>
       </c>
       <c r="K504" t="n">
-        <v>35.5</v>
+        <v>30.9</v>
       </c>
       <c r="L504" t="n">
-        <v>101.4</v>
+        <v>88.3</v>
       </c>
     </row>
     <row r="505">
@@ -24634,7 +24634,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>P84</t>
+          <t>P83</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -24649,14 +24649,14 @@
       </c>
       <c r="E505" t="inlineStr">
         <is>
-          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
+          <t>Pilote 103 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F505" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="G505" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H505" s="1" t="n">
         <v>46318</v>
@@ -24668,10 +24668,10 @@
         <v>35</v>
       </c>
       <c r="K505" t="n">
-        <v>35.1</v>
+        <v>20.2</v>
       </c>
       <c r="L505" t="n">
-        <v>100.3</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="506">
@@ -24682,7 +24682,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>P85</t>
+          <t>P83</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
@@ -24697,14 +24697,14 @@
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>Pilote 73 torre 2 tipo 2</t>
+          <t>Pilote 103 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F506" s="1" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="G506" s="1" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="H506" s="1" t="n">
         <v>46318</v>
@@ -24716,10 +24716,10 @@
         <v>35</v>
       </c>
       <c r="K506" t="n">
-        <v>42.5</v>
+        <v>20.6</v>
       </c>
       <c r="L506" t="n">
-        <v>121.4</v>
+        <v>58.9</v>
       </c>
     </row>
     <row r="507">
@@ -24730,7 +24730,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>P85</t>
+          <t>P84</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -24745,7 +24745,7 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>Pilote 73 torre 2 tipo 2</t>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F507" s="1" t="n">
@@ -24764,10 +24764,10 @@
         <v>35</v>
       </c>
       <c r="K507" t="n">
-        <v>41.6</v>
+        <v>35.5</v>
       </c>
       <c r="L507" t="n">
-        <v>118.9</v>
+        <v>101.4</v>
       </c>
     </row>
     <row r="508">
@@ -24778,7 +24778,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>P86</t>
+          <t>P84</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
@@ -24793,17 +24793,17 @@
       </c>
       <c r="E508" t="inlineStr">
         <is>
-          <t>Pilote 79 torre 2 tipo 2</t>
+          <t>Pilote 74 torre 2 tipo 2 Pilote 83 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F508" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="G508" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H508" s="1" t="n">
         <v>46318</v>
-      </c>
-      <c r="H508" s="1" t="n">
-        <v>46321</v>
       </c>
       <c r="I508" t="n">
         <v>7</v>
@@ -24812,10 +24812,10 @@
         <v>35</v>
       </c>
       <c r="K508" t="n">
-        <v>34.5</v>
+        <v>35.1</v>
       </c>
       <c r="L508" t="n">
-        <v>98.59999999999999</v>
+        <v>100.3</v>
       </c>
     </row>
     <row r="509">
@@ -24826,7 +24826,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>P86</t>
+          <t>P85</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -24841,17 +24841,17 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>Pilote 79 torre 2 tipo 2</t>
+          <t>Pilote 73 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F509" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="G509" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H509" s="1" t="n">
         <v>46318</v>
-      </c>
-      <c r="H509" s="1" t="n">
-        <v>46321</v>
       </c>
       <c r="I509" t="n">
         <v>7</v>
@@ -24860,10 +24860,10 @@
         <v>35</v>
       </c>
       <c r="K509" t="n">
-        <v>33.2</v>
+        <v>42.5</v>
       </c>
       <c r="L509" t="n">
-        <v>94.90000000000001</v>
+        <v>121.4</v>
       </c>
     </row>
     <row r="510">
@@ -24874,7 +24874,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>P87</t>
+          <t>P85</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -24889,17 +24889,17 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>Pilote 91 torre 2 tipo 1</t>
+          <t>Pilote 73 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F510" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="G510" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H510" s="1" t="n">
         <v>46318</v>
-      </c>
-      <c r="H510" s="1" t="n">
-        <v>46321</v>
       </c>
       <c r="I510" t="n">
         <v>7</v>
@@ -24908,10 +24908,10 @@
         <v>35</v>
       </c>
       <c r="K510" t="n">
-        <v>36.7</v>
+        <v>41.6</v>
       </c>
       <c r="L510" t="n">
-        <v>104.9</v>
+        <v>118.9</v>
       </c>
     </row>
     <row r="511">
@@ -24922,7 +24922,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>P87</t>
+          <t>P86</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -24937,7 +24937,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>Pilote 91 torre 2 tipo 1</t>
+          <t>Pilote 79 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F511" s="1" t="n">
@@ -24956,10 +24956,10 @@
         <v>35</v>
       </c>
       <c r="K511" t="n">
-        <v>37.3</v>
+        <v>34.5</v>
       </c>
       <c r="L511" t="n">
-        <v>106.6</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="512">
@@ -24970,7 +24970,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>P88</t>
+          <t>P86</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -24985,14 +24985,14 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+          <t>Pilote 79 torre 2 tipo 2</t>
         </is>
       </c>
       <c r="F512" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="G512" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="H512" s="1" t="n">
         <v>46321</v>
@@ -25004,10 +25004,10 @@
         <v>35</v>
       </c>
       <c r="K512" t="n">
-        <v>28.1</v>
+        <v>33.2</v>
       </c>
       <c r="L512" t="n">
-        <v>80.3</v>
+        <v>94.90000000000001</v>
       </c>
     </row>
     <row r="513">
@@ -25018,7 +25018,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>P88</t>
+          <t>P87</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -25033,14 +25033,14 @@
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+          <t>Pilote 91 torre 2 tipo 1</t>
         </is>
       </c>
       <c r="F513" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="G513" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="H513" s="1" t="n">
         <v>46321</v>
@@ -25052,10 +25052,346 @@
         <v>35</v>
       </c>
       <c r="K513" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="L513" t="n">
+        <v>104.9</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>P87</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Pilote 91 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F514" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G514" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H514" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I514" t="n">
+        <v>7</v>
+      </c>
+      <c r="J514" t="n">
+        <v>35</v>
+      </c>
+      <c r="K514" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="L514" t="n">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>P88</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F515" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G515" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H515" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I515" t="n">
+        <v>7</v>
+      </c>
+      <c r="J515" t="n">
+        <v>35</v>
+      </c>
+      <c r="K515" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="L515" t="n">
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>P88</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Pilote 96 y 92 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F516" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G516" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="H516" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I516" t="n">
+        <v>7</v>
+      </c>
+      <c r="J516" t="n">
+        <v>35</v>
+      </c>
+      <c r="K516" t="n">
         <v>27.3</v>
       </c>
-      <c r="L513" t="n">
+      <c r="L516" t="n">
         <v>78</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>P89</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Pilote 101 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F517" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G517" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H517" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I517" t="n">
+        <v>7</v>
+      </c>
+      <c r="J517" t="n">
+        <v>35</v>
+      </c>
+      <c r="K517" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="L517" t="n">
+        <v>106.3</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>P89</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Pilote 101 torre 2 tipo 2</t>
+        </is>
+      </c>
+      <c r="F518" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G518" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H518" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I518" t="n">
+        <v>7</v>
+      </c>
+      <c r="J518" t="n">
+        <v>35</v>
+      </c>
+      <c r="K518" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="L518" t="n">
+        <v>107.4</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Pilote 89 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F519" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G519" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H519" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I519" t="n">
+        <v>7</v>
+      </c>
+      <c r="J519" t="n">
+        <v>35</v>
+      </c>
+      <c r="K519" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="L519" t="n">
+        <v>112.3</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>29007 - VENTO TIPO C</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No especificado </t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Pilote 89 torre 2 tipo 1</t>
+        </is>
+      </c>
+      <c r="F520" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G520" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H520" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I520" t="n">
+        <v>7</v>
+      </c>
+      <c r="J520" t="n">
+        <v>35</v>
+      </c>
+      <c r="K520" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="L520" t="n">
+        <v>113.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>